<commit_message>
docs: T-C02 complete and merged — baseline 7c6f122; T-C03 scope locked; tracker F-021/F-029/F-030 in progress
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -686,13 +686,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
           <t>No</t>
@@ -713,7 +711,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
           <t>PATCHED v2: was AWS/GCP/Azure + Terraform/K8s - contradicted free-tier constraint and ADR-006. | Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -801,13 +798,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>No</t>
@@ -828,7 +823,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -916,13 +910,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
           <t>No</t>
@@ -943,7 +935,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -1031,13 +1022,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>No</t>
@@ -1058,7 +1047,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -1146,13 +1134,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1173,7 +1159,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -1261,13 +1246,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1288,7 +1271,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -1376,13 +1358,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1403,7 +1383,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -1491,13 +1470,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1518,7 +1495,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr">
         <is>
           <t>PATCHED v2: was Celery+Redis (Python stack) - contradicted Java ADR-001. | Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -1606,13 +1582,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1633,7 +1607,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -1721,13 +1694,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1748,7 +1719,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -1836,13 +1806,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1863,7 +1831,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -1951,13 +1918,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1978,8 +1943,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2062,13 +2025,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
           <t>No</t>
@@ -2089,8 +2050,6 @@
           <t>Partial (UI based on role)</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2173,13 +2132,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
           <t>No</t>
@@ -2200,8 +2157,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2284,13 +2239,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
           <t>No</t>
@@ -2311,8 +2264,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2395,13 +2346,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
           <t>No</t>
@@ -2422,8 +2371,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2506,13 +2453,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
           <t>No</t>
@@ -2533,8 +2478,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2617,13 +2560,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
           <t>No</t>
@@ -2644,8 +2585,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2728,13 +2667,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
           <t>No</t>
@@ -2755,8 +2692,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2874,7 +2809,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr"/>
       <c r="Y21" t="inlineStr">
         <is>
           <t>PATCHED v2: was PyPDF2+Neo4j nodes; now polyglot parser contract per ADR-011.</t>
@@ -2962,7 +2896,6 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
@@ -2980,7 +2913,7 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
@@ -2993,8 +2926,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>T-C02 GLM-OCR bridge MERGED to syllabai-core main @ 7c6f122 (PR #3, 2026-09-05): QP/MS pairs persist as canonical documents + T-011 paper/question/mark-scheme rows, all SUGGESTED (teacher validation gate before serving). Design: core docs/t-c02-bridge.md. Remaining: learner-facing paper browsing/filtering UI + first real batch review (T-C03).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3087,7 +3023,6 @@
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
           <t>No</t>
@@ -3108,8 +3043,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3192,13 +3125,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
           <t>No</t>
@@ -3219,8 +3150,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3303,13 +3232,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
           <t>No</t>
@@ -3330,8 +3257,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3414,13 +3339,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
           <t>No</t>
@@ -3441,8 +3364,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3525,13 +3446,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
           <t>No</t>
@@ -3552,8 +3471,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3646,7 +3563,6 @@
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
           <t>No</t>
@@ -3667,8 +3583,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3751,7 +3665,6 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
           <t>tagging accuracy + generation coverage</t>
@@ -3782,7 +3695,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr"/>
       <c r="Y29" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -3870,13 +3782,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
           <t>No</t>
@@ -3884,7 +3794,7 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
@@ -3897,10 +3807,9 @@
           <t>Partial (UI button)</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>T-C02 bridge merged @ 7c6f122: MS entries map to MarkScheme/MarkPoint rows (whole-entry mark points for cells without (N) markers); verbatim MS JSONB retained in V13 glm_ocr_bridge_records; review-findings endpoint surfaces conflicts (e.g. 1A 80-vs-120) instead of merging them away. Remaining: LaTeX mark-scheme rendering + validation workflow over imported schemes.</t>
         </is>
       </c>
     </row>
@@ -3985,13 +3894,11 @@
           <t>syllabai-parser</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
           <t>No</t>
@@ -3999,7 +3906,7 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
@@ -4012,8 +3919,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>T-C02 bridge merged @ 7c6f122: controlled ingestion entries exist — teacher-gated POST /api/v1/teacher/content/glm-ocr/pairs + ops CLI --syllabai.glmocr.pair-dir, rerun-idempotent. Batch real-corpus ingestion = T-C03 (one bounded batch + human review, in progress). Remaining: CSV/Excel teacher upload UI (Cycle 2+ scope of this row).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4096,13 +4006,11 @@
           <t>syllabai-parser</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
           <t>No</t>
@@ -4123,8 +4031,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr"/>
-      <c r="Y32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4242,7 +4148,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X33" t="inlineStr"/>
       <c r="Y33" t="inlineStr">
         <is>
           <t>PATCHED v2: was 'Neo4j' - Postgres graph is ADR-005 default; Neo4j-portable schema kept. | Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -4365,7 +4270,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X34" t="inlineStr"/>
       <c r="Y34" t="inlineStr">
         <is>
           <t>PATCHED v2: was (Student)-[:MASTERS]-&gt;(Topic) Cypher property model. | Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -4453,7 +4357,6 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
@@ -4484,7 +4387,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X35" t="inlineStr"/>
       <c r="Y35" t="inlineStr">
         <is>
           <t>PATCHED v2: was Cypher query + Neo4j driver.</t>
@@ -4572,13 +4474,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
           <t>No</t>
@@ -4599,7 +4499,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr"/>
       <c r="Y36" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -4687,13 +4586,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
           <t>No</t>
@@ -4714,8 +4611,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X37" t="inlineStr"/>
-      <c r="Y37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4833,7 +4728,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X38" t="inlineStr"/>
       <c r="Y38" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -4921,13 +4815,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
           <t>No</t>
@@ -4948,8 +4840,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X39" t="inlineStr"/>
-      <c r="Y39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5032,7 +4922,6 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
@@ -5063,7 +4952,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr">
         <is>
           <t>PATCHED v2: was Pinecone/Weaviate default - ADR-004 keeps vectors in Postgres. | Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -5186,7 +5074,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr"/>
       <c r="Y41" t="inlineStr">
         <is>
           <t>PATCHED v2: was generic chunk-retrieve-prompt; now Paper B KA-RAG spec. | Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -5274,13 +5161,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5301,8 +5186,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X42" t="inlineStr"/>
-      <c r="Y42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5385,13 +5268,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
           <t>No</t>
@@ -5412,7 +5293,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X43" t="inlineStr"/>
       <c r="Y43" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -5500,7 +5380,6 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
           <t>retrieval recall + citation precision/groundedness</t>
@@ -5531,8 +5410,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X44" t="inlineStr"/>
-      <c r="Y44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5615,13 +5492,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
           <t>No</t>
@@ -5642,7 +5517,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X45" t="inlineStr"/>
       <c r="Y45" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -5730,13 +5604,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
           <t>No</t>
@@ -5757,7 +5629,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X46" t="inlineStr"/>
       <c r="Y46" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -5845,13 +5716,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
           <t>No</t>
@@ -5872,7 +5741,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X47" t="inlineStr"/>
       <c r="Y47" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -5995,7 +5863,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X48" t="inlineStr"/>
       <c r="Y48" t="inlineStr">
         <is>
           <t>PATCHED v2: added Paper B kappa agreement gate to validation metric. | Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -6083,13 +5950,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
           <t>No</t>
@@ -6110,7 +5975,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr"/>
       <c r="Y49" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -6233,7 +6097,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X50" t="inlineStr"/>
       <c r="Y50" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -6321,13 +6184,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr">
         <is>
           <t>No</t>
@@ -6348,7 +6209,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X51" t="inlineStr"/>
       <c r="Y51" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -6436,13 +6296,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr">
         <is>
           <t>No</t>
@@ -6463,7 +6321,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X52" t="inlineStr"/>
       <c r="Y52" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -6551,13 +6408,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr">
         <is>
           <t>No</t>
@@ -6578,8 +6433,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X53" t="inlineStr"/>
-      <c r="Y53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6697,7 +6550,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X54" t="inlineStr"/>
       <c r="Y54" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -6785,13 +6637,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr">
         <is>
           <t>No</t>
@@ -6812,7 +6662,6 @@
           <t>Partial</t>
         </is>
       </c>
-      <c r="X55" t="inlineStr"/>
       <c r="Y55" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -6910,7 +6759,6 @@
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -6931,7 +6779,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X56" t="inlineStr"/>
       <c r="Y56" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -7019,13 +6866,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr">
         <is>
           <t>No</t>
@@ -7046,7 +6891,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X57" t="inlineStr"/>
       <c r="Y57" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -7134,13 +6978,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S58" t="inlineStr"/>
       <c r="T58" t="inlineStr">
         <is>
           <t>No</t>
@@ -7161,7 +7003,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X58" t="inlineStr"/>
       <c r="Y58" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -7249,13 +7090,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr">
         <is>
           <t>No</t>
@@ -7276,8 +7115,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X59" t="inlineStr"/>
-      <c r="Y59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -7360,13 +7197,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr">
         <is>
           <t>No</t>
@@ -7387,8 +7222,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X60" t="inlineStr"/>
-      <c r="Y60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7471,13 +7304,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q61" t="inlineStr"/>
       <c r="R61" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr">
         <is>
           <t>No</t>
@@ -7498,8 +7329,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X61" t="inlineStr"/>
-      <c r="Y61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7582,13 +7411,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q62" t="inlineStr"/>
       <c r="R62" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr">
         <is>
           <t>No</t>
@@ -7609,7 +7436,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X62" t="inlineStr"/>
       <c r="Y62" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -7707,7 +7533,6 @@
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S63" t="inlineStr"/>
       <c r="T63" t="inlineStr">
         <is>
           <t>No</t>
@@ -7728,8 +7553,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X63" t="inlineStr"/>
-      <c r="Y63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7812,13 +7635,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr">
         <is>
           <t>No</t>
@@ -7839,8 +7660,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X64" t="inlineStr"/>
-      <c r="Y64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7923,13 +7742,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S65" t="inlineStr"/>
       <c r="T65" t="inlineStr">
         <is>
           <t>No</t>
@@ -7950,8 +7767,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X65" t="inlineStr"/>
-      <c r="Y65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8034,13 +7849,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S66" t="inlineStr"/>
       <c r="T66" t="inlineStr">
         <is>
           <t>No</t>
@@ -8061,8 +7874,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X66" t="inlineStr"/>
-      <c r="Y66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8145,13 +7956,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q67" t="inlineStr"/>
       <c r="R67" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S67" t="inlineStr"/>
       <c r="T67" t="inlineStr">
         <is>
           <t>No</t>
@@ -8172,8 +7981,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X67" t="inlineStr"/>
-      <c r="Y67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8256,13 +8063,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S68" t="inlineStr"/>
       <c r="T68" t="inlineStr">
         <is>
           <t>No</t>
@@ -8283,8 +8088,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X68" t="inlineStr"/>
-      <c r="Y68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8367,13 +8170,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q69" t="inlineStr"/>
       <c r="R69" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S69" t="inlineStr"/>
       <c r="T69" t="inlineStr">
         <is>
           <t>No</t>
@@ -8394,8 +8195,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X69" t="inlineStr"/>
-      <c r="Y69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8478,13 +8277,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q70" t="inlineStr"/>
       <c r="R70" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S70" t="inlineStr"/>
       <c r="T70" t="inlineStr">
         <is>
           <t>No</t>
@@ -8505,8 +8302,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X70" t="inlineStr"/>
-      <c r="Y70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8589,13 +8384,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q71" t="inlineStr"/>
       <c r="R71" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S71" t="inlineStr"/>
       <c r="T71" t="inlineStr">
         <is>
           <t>No</t>
@@ -8616,8 +8409,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X71" t="inlineStr"/>
-      <c r="Y71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8700,13 +8491,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q72" t="inlineStr"/>
       <c r="R72" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S72" t="inlineStr"/>
       <c r="T72" t="inlineStr">
         <is>
           <t>No</t>
@@ -8727,8 +8516,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X72" t="inlineStr"/>
-      <c r="Y72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8821,7 +8608,6 @@
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S73" t="inlineStr"/>
       <c r="T73" t="inlineStr">
         <is>
           <t>No</t>
@@ -8842,7 +8628,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X73" t="inlineStr"/>
       <c r="Y73" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -8965,7 +8750,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X74" t="inlineStr"/>
       <c r="Y74" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -9053,13 +8837,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q75" t="inlineStr"/>
       <c r="R75" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S75" t="inlineStr"/>
       <c r="T75" t="inlineStr">
         <is>
           <t>No</t>
@@ -9080,8 +8862,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X75" t="inlineStr"/>
-      <c r="Y75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -9164,13 +8944,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S76" t="inlineStr"/>
       <c r="T76" t="inlineStr">
         <is>
           <t>No</t>
@@ -9191,8 +8969,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X76" t="inlineStr"/>
-      <c r="Y76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -9275,13 +9051,11 @@
           <t>syllabai-parser</t>
         </is>
       </c>
-      <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr">
         <is>
           <t>tagging accuracy + generation coverage</t>
         </is>
       </c>
-      <c r="S77" t="inlineStr"/>
       <c r="T77" t="inlineStr">
         <is>
           <t>No</t>
@@ -9302,8 +9076,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X77" t="inlineStr"/>
-      <c r="Y77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -9386,13 +9158,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q78" t="inlineStr"/>
       <c r="R78" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S78" t="inlineStr"/>
       <c r="T78" t="inlineStr">
         <is>
           <t>No</t>
@@ -9413,8 +9183,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X78" t="inlineStr"/>
-      <c r="Y78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -9497,13 +9265,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S79" t="inlineStr"/>
       <c r="T79" t="inlineStr">
         <is>
           <t>No</t>
@@ -9524,7 +9290,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X79" t="inlineStr"/>
       <c r="Y79" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -9612,13 +9377,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q80" t="inlineStr"/>
       <c r="R80" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S80" t="inlineStr"/>
       <c r="T80" t="inlineStr">
         <is>
           <t>No</t>
@@ -9639,7 +9402,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X80" t="inlineStr"/>
       <c r="Y80" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -9727,13 +9489,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q81" t="inlineStr"/>
       <c r="R81" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S81" t="inlineStr"/>
       <c r="T81" t="inlineStr">
         <is>
           <t>No</t>
@@ -9754,8 +9514,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X81" t="inlineStr"/>
-      <c r="Y81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -9838,13 +9596,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q82" t="inlineStr"/>
       <c r="R82" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S82" t="inlineStr"/>
       <c r="T82" t="inlineStr">
         <is>
           <t>No</t>
@@ -9865,8 +9621,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X82" t="inlineStr"/>
-      <c r="Y82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -9949,13 +9703,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S83" t="inlineStr"/>
       <c r="T83" t="inlineStr">
         <is>
           <t>No</t>
@@ -9976,8 +9728,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X83" t="inlineStr"/>
-      <c r="Y83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -10060,13 +9810,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q84" t="inlineStr"/>
       <c r="R84" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S84" t="inlineStr"/>
       <c r="T84" t="inlineStr">
         <is>
           <t>No</t>
@@ -10087,8 +9835,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X84" t="inlineStr"/>
-      <c r="Y84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -10171,13 +9917,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q85" t="inlineStr"/>
       <c r="R85" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S85" t="inlineStr"/>
       <c r="T85" t="inlineStr">
         <is>
           <t>No</t>
@@ -10198,8 +9942,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X85" t="inlineStr"/>
-      <c r="Y85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -10282,13 +10024,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S86" t="inlineStr"/>
       <c r="T86" t="inlineStr">
         <is>
           <t>No</t>
@@ -10309,8 +10049,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X86" t="inlineStr"/>
-      <c r="Y86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10393,13 +10131,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q87" t="inlineStr"/>
       <c r="R87" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S87" t="inlineStr"/>
       <c r="T87" t="inlineStr">
         <is>
           <t>No</t>
@@ -10420,8 +10156,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X87" t="inlineStr"/>
-      <c r="Y87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -10504,13 +10238,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q88" t="inlineStr"/>
       <c r="R88" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S88" t="inlineStr"/>
       <c r="T88" t="inlineStr">
         <is>
           <t>No</t>
@@ -10531,7 +10263,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X88" t="inlineStr"/>
       <c r="Y88" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -10619,13 +10350,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q89" t="inlineStr"/>
       <c r="R89" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S89" t="inlineStr"/>
       <c r="T89" t="inlineStr">
         <is>
           <t>No</t>
@@ -10646,7 +10375,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X89" t="inlineStr"/>
       <c r="Y89" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -10734,13 +10462,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q90" t="inlineStr"/>
       <c r="R90" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S90" t="inlineStr"/>
       <c r="T90" t="inlineStr">
         <is>
           <t>No</t>
@@ -10761,7 +10487,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X90" t="inlineStr"/>
       <c r="Y90" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -10849,13 +10574,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr">
         <is>
           <t>No</t>
@@ -10876,7 +10599,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X91" t="inlineStr"/>
       <c r="Y91" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -10964,13 +10686,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q92" t="inlineStr"/>
       <c r="R92" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S92" t="inlineStr"/>
       <c r="T92" t="inlineStr">
         <is>
           <t>No</t>
@@ -10991,7 +10711,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X92" t="inlineStr"/>
       <c r="Y92" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -11089,7 +10808,6 @@
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S93" t="inlineStr"/>
       <c r="T93" t="inlineStr">
         <is>
           <t>No</t>
@@ -11110,7 +10828,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X93" t="inlineStr"/>
       <c r="Y93" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -11198,13 +10915,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q94" t="inlineStr"/>
       <c r="R94" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S94" t="inlineStr"/>
       <c r="T94" t="inlineStr">
         <is>
           <t>No</t>
@@ -11225,8 +10940,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X94" t="inlineStr"/>
-      <c r="Y94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -11309,13 +11022,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q95" t="inlineStr"/>
       <c r="R95" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S95" t="inlineStr"/>
       <c r="T95" t="inlineStr">
         <is>
           <t>No</t>
@@ -11336,7 +11047,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X95" t="inlineStr"/>
       <c r="Y95" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -11459,7 +11169,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X96" t="inlineStr"/>
       <c r="Y96" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -11557,7 +11266,6 @@
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S97" t="inlineStr"/>
       <c r="T97" t="inlineStr">
         <is>
           <t>No</t>
@@ -11578,7 +11286,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X97" t="inlineStr"/>
       <c r="Y97" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -11666,13 +11373,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q98" t="inlineStr"/>
       <c r="R98" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S98" t="inlineStr"/>
       <c r="T98" t="inlineStr">
         <is>
           <t>No</t>
@@ -11693,7 +11398,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X98" t="inlineStr"/>
       <c r="Y98" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -11781,13 +11485,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q99" t="inlineStr"/>
       <c r="R99" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S99" t="inlineStr"/>
       <c r="T99" t="inlineStr">
         <is>
           <t>No</t>
@@ -11808,7 +11510,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X99" t="inlineStr"/>
       <c r="Y99" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -11896,13 +11597,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q100" t="inlineStr"/>
       <c r="R100" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S100" t="inlineStr"/>
       <c r="T100" t="inlineStr">
         <is>
           <t>No</t>
@@ -11923,8 +11622,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X100" t="inlineStr"/>
-      <c r="Y100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -12007,13 +11704,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q101" t="inlineStr"/>
       <c r="R101" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S101" t="inlineStr"/>
       <c r="T101" t="inlineStr">
         <is>
           <t>No</t>
@@ -12034,8 +11729,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X101" t="inlineStr"/>
-      <c r="Y101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -12118,13 +11811,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q102" t="inlineStr"/>
       <c r="R102" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S102" t="inlineStr"/>
       <c r="T102" t="inlineStr">
         <is>
           <t>No</t>
@@ -12145,8 +11836,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X102" t="inlineStr"/>
-      <c r="Y102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -12229,13 +11918,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q103" t="inlineStr"/>
       <c r="R103" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S103" t="inlineStr"/>
       <c r="T103" t="inlineStr">
         <is>
           <t>No</t>
@@ -12256,8 +11943,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X103" t="inlineStr"/>
-      <c r="Y103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -12340,13 +12025,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q104" t="inlineStr"/>
       <c r="R104" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S104" t="inlineStr"/>
       <c r="T104" t="inlineStr">
         <is>
           <t>No</t>
@@ -12367,8 +12050,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X104" t="inlineStr"/>
-      <c r="Y104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -12451,13 +12132,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q105" t="inlineStr"/>
       <c r="R105" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S105" t="inlineStr"/>
       <c r="T105" t="inlineStr">
         <is>
           <t>No</t>
@@ -12478,8 +12157,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X105" t="inlineStr"/>
-      <c r="Y105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -12562,13 +12239,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q106" t="inlineStr"/>
       <c r="R106" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S106" t="inlineStr"/>
       <c r="T106" t="inlineStr">
         <is>
           <t>No</t>
@@ -12584,9 +12259,6 @@
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W106" t="inlineStr"/>
-      <c r="X106" t="inlineStr"/>
-      <c r="Y106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -12669,13 +12341,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q107" t="inlineStr"/>
       <c r="R107" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S107" t="inlineStr"/>
       <c r="T107" t="inlineStr">
         <is>
           <t>No</t>
@@ -12696,8 +12366,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X107" t="inlineStr"/>
-      <c r="Y107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -12780,13 +12448,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q108" t="inlineStr"/>
       <c r="R108" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S108" t="inlineStr"/>
       <c r="T108" t="inlineStr">
         <is>
           <t>No</t>
@@ -12807,8 +12473,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X108" t="inlineStr"/>
-      <c r="Y108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -12891,13 +12555,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q109" t="inlineStr"/>
       <c r="R109" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S109" t="inlineStr"/>
       <c r="T109" t="inlineStr">
         <is>
           <t>No</t>
@@ -12918,8 +12580,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X109" t="inlineStr"/>
-      <c r="Y109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -13002,13 +12662,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q110" t="inlineStr"/>
       <c r="R110" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S110" t="inlineStr"/>
       <c r="T110" t="inlineStr">
         <is>
           <t>No</t>
@@ -13029,8 +12687,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X110" t="inlineStr"/>
-      <c r="Y110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -13038,7 +12694,6 @@
           <t>F-111</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr"/>
       <c r="C111" t="inlineStr">
         <is>
           <t>Progressive Web App (PWA)</t>
@@ -13109,13 +12764,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q111" t="inlineStr"/>
       <c r="R111" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S111" t="inlineStr"/>
       <c r="T111" t="inlineStr">
         <is>
           <t>No</t>
@@ -13136,8 +12789,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X111" t="inlineStr"/>
-      <c r="Y111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -13145,7 +12796,6 @@
           <t>F-113</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr">
         <is>
           <t>Offline Access to Downloaded Materials</t>
@@ -13216,13 +12866,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q112" t="inlineStr"/>
       <c r="R112" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S112" t="inlineStr"/>
       <c r="T112" t="inlineStr">
         <is>
           <t>No</t>
@@ -13243,8 +12891,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X112" t="inlineStr"/>
-      <c r="Y112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -13252,7 +12898,6 @@
           <t>F-115</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr">
         <is>
           <t>Mobile App (React Native / Flutter)</t>
@@ -13323,13 +12968,11 @@
           <t>syllabai-web</t>
         </is>
       </c>
-      <c r="Q113" t="inlineStr"/>
       <c r="R113" t="inlineStr">
         <is>
           <t>automated UI tests + accessibility checks</t>
         </is>
       </c>
-      <c r="S113" t="inlineStr"/>
       <c r="T113" t="inlineStr">
         <is>
           <t>No</t>
@@ -13350,8 +12993,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X113" t="inlineStr"/>
-      <c r="Y113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -13434,13 +13075,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q114" t="inlineStr"/>
       <c r="R114" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S114" t="inlineStr"/>
       <c r="T114" t="inlineStr">
         <is>
           <t>No</t>
@@ -13461,7 +13100,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X114" t="inlineStr"/>
       <c r="Y114" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -13549,13 +13187,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q115" t="inlineStr"/>
       <c r="R115" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S115" t="inlineStr"/>
       <c r="T115" t="inlineStr">
         <is>
           <t>No</t>
@@ -13576,8 +13212,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X115" t="inlineStr"/>
-      <c r="Y115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -13660,13 +13294,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q116" t="inlineStr"/>
       <c r="R116" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S116" t="inlineStr"/>
       <c r="T116" t="inlineStr">
         <is>
           <t>No</t>
@@ -13687,7 +13319,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X116" t="inlineStr"/>
       <c r="Y116" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -13775,13 +13406,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q117" t="inlineStr"/>
       <c r="R117" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S117" t="inlineStr"/>
       <c r="T117" t="inlineStr">
         <is>
           <t>No</t>
@@ -13802,7 +13431,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X117" t="inlineStr"/>
       <c r="Y117" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -13890,13 +13518,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q118" t="inlineStr"/>
       <c r="R118" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S118" t="inlineStr"/>
       <c r="T118" t="inlineStr">
         <is>
           <t>No</t>
@@ -13917,7 +13543,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X118" t="inlineStr"/>
       <c r="Y118" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -14005,13 +13630,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q119" t="inlineStr"/>
       <c r="R119" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S119" t="inlineStr"/>
       <c r="T119" t="inlineStr">
         <is>
           <t>No</t>
@@ -14032,7 +13655,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X119" t="inlineStr"/>
       <c r="Y119" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -14120,13 +13742,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q120" t="inlineStr"/>
       <c r="R120" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S120" t="inlineStr"/>
       <c r="T120" t="inlineStr">
         <is>
           <t>No</t>
@@ -14147,7 +13767,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X120" t="inlineStr"/>
       <c r="Y120" t="inlineStr">
         <is>
           <t>PATCHED v2: was FastAPI/DRF - contradicted Java ADR-001. | Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -14235,13 +13854,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q121" t="inlineStr"/>
       <c r="R121" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S121" t="inlineStr"/>
       <c r="T121" t="inlineStr">
         <is>
           <t>No</t>
@@ -14262,8 +13879,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X121" t="inlineStr"/>
-      <c r="Y121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -14346,13 +13961,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q122" t="inlineStr"/>
       <c r="R122" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S122" t="inlineStr"/>
       <c r="T122" t="inlineStr">
         <is>
           <t>No</t>
@@ -14373,8 +13986,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X122" t="inlineStr"/>
-      <c r="Y122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -14457,13 +14068,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q123" t="inlineStr"/>
       <c r="R123" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S123" t="inlineStr"/>
       <c r="T123" t="inlineStr">
         <is>
           <t>No</t>
@@ -14484,7 +14093,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X123" t="inlineStr"/>
       <c r="Y123" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -14572,13 +14180,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q124" t="inlineStr"/>
       <c r="R124" t="inlineStr">
         <is>
           <t>integration tests + uptime/error metrics</t>
         </is>
       </c>
-      <c r="S124" t="inlineStr"/>
       <c r="T124" t="inlineStr">
         <is>
           <t>No</t>
@@ -14599,7 +14205,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X124" t="inlineStr"/>
       <c r="Y124" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -14687,13 +14292,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q125" t="inlineStr"/>
       <c r="R125" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S125" t="inlineStr"/>
       <c r="T125" t="inlineStr">
         <is>
           <t>No</t>
@@ -14714,8 +14317,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X125" t="inlineStr"/>
-      <c r="Y125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -14798,13 +14399,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q126" t="inlineStr"/>
       <c r="R126" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S126" t="inlineStr"/>
       <c r="T126" t="inlineStr">
         <is>
           <t>No</t>
@@ -14825,8 +14424,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X126" t="inlineStr"/>
-      <c r="Y126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -14909,13 +14506,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q127" t="inlineStr"/>
       <c r="R127" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S127" t="inlineStr"/>
       <c r="T127" t="inlineStr">
         <is>
           <t>No</t>
@@ -14936,8 +14531,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X127" t="inlineStr"/>
-      <c r="Y127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -15020,13 +14613,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q128" t="inlineStr"/>
       <c r="R128" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S128" t="inlineStr"/>
       <c r="T128" t="inlineStr">
         <is>
           <t>No</t>
@@ -15047,8 +14638,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X128" t="inlineStr"/>
-      <c r="Y128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -15131,13 +14720,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q129" t="inlineStr"/>
       <c r="R129" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S129" t="inlineStr"/>
       <c r="T129" t="inlineStr">
         <is>
           <t>No</t>
@@ -15158,8 +14745,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X129" t="inlineStr"/>
-      <c r="Y129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -15242,13 +14827,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q130" t="inlineStr"/>
       <c r="R130" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S130" t="inlineStr"/>
       <c r="T130" t="inlineStr">
         <is>
           <t>No</t>
@@ -15269,8 +14852,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X130" t="inlineStr"/>
-      <c r="Y130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -15353,13 +14934,11 @@
           <t>syllabai-core</t>
         </is>
       </c>
-      <c r="Q131" t="inlineStr"/>
       <c r="R131" t="inlineStr">
         <is>
           <t>feature acceptance criteria</t>
         </is>
       </c>
-      <c r="S131" t="inlineStr"/>
       <c r="T131" t="inlineStr">
         <is>
           <t>No</t>
@@ -15380,8 +14959,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X131" t="inlineStr"/>
-      <c r="Y131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -15474,7 +15051,6 @@
           <t>schema contract tests</t>
         </is>
       </c>
-      <c r="S132" t="inlineStr"/>
       <c r="T132" t="inlineStr">
         <is>
           <t>No</t>
@@ -15495,8 +15071,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X132" t="inlineStr"/>
-      <c r="Y132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -15589,7 +15163,6 @@
           <t>contract + integration tests</t>
         </is>
       </c>
-      <c r="S133" t="inlineStr"/>
       <c r="T133" t="inlineStr">
         <is>
           <t>No</t>
@@ -15610,7 +15183,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X133" t="inlineStr"/>
       <c r="Y133" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -15708,7 +15280,6 @@
           <t>retrieval benchmark + contract tests</t>
         </is>
       </c>
-      <c r="S134" t="inlineStr"/>
       <c r="T134" t="inlineStr">
         <is>
           <t>No</t>
@@ -15729,7 +15300,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X134" t="inlineStr"/>
       <c r="Y134" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -15827,7 +15397,6 @@
           <t>state transition tests + schema validation</t>
         </is>
       </c>
-      <c r="S135" t="inlineStr"/>
       <c r="T135" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -15848,7 +15417,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X135" t="inlineStr"/>
       <c r="Y135" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -15946,7 +15514,6 @@
           <t>simulation + bias/RMSE</t>
         </is>
       </c>
-      <c r="S136" t="inlineStr"/>
       <c r="T136" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -15967,7 +15534,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X136" t="inlineStr"/>
       <c r="Y136" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -16065,7 +15631,6 @@
           <t>bias &lt; threshold; RMSE &lt; threshold</t>
         </is>
       </c>
-      <c r="S137" t="inlineStr"/>
       <c r="T137" t="inlineStr">
         <is>
           <t>No</t>
@@ -16086,7 +15651,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X137" t="inlineStr"/>
       <c r="Y137" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -16184,7 +15748,6 @@
           <t>expert agreement + calibration</t>
         </is>
       </c>
-      <c r="S138" t="inlineStr"/>
       <c r="T138" t="inlineStr">
         <is>
           <t>No</t>
@@ -16205,7 +15768,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X138" t="inlineStr"/>
       <c r="Y138" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -16303,7 +15865,6 @@
           <t>precision/recall + expert agreement</t>
         </is>
       </c>
-      <c r="S139" t="inlineStr"/>
       <c r="T139" t="inlineStr">
         <is>
           <t>No</t>
@@ -16324,8 +15885,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X139" t="inlineStr"/>
-      <c r="Y139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -16418,7 +15977,6 @@
           <t>citation precision + lineage tests</t>
         </is>
       </c>
-      <c r="S140" t="inlineStr"/>
       <c r="T140" t="inlineStr">
         <is>
           <t>No</t>
@@ -16439,7 +15997,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X140" t="inlineStr"/>
       <c r="Y140" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -16537,7 +16094,6 @@
           <t>reproducibility test</t>
         </is>
       </c>
-      <c r="S141" t="inlineStr"/>
       <c r="T141" t="inlineStr">
         <is>
           <t>No</t>
@@ -16558,7 +16114,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X141" t="inlineStr"/>
       <c r="Y141" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -16656,7 +16211,6 @@
           <t>inter-rater agreement + audit completeness</t>
         </is>
       </c>
-      <c r="S142" t="inlineStr"/>
       <c r="T142" t="inlineStr">
         <is>
           <t>No</t>
@@ -16677,7 +16231,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X142" t="inlineStr"/>
       <c r="Y142" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -16775,7 +16328,6 @@
           <t>agreement/correlation/calibration</t>
         </is>
       </c>
-      <c r="S143" t="inlineStr"/>
       <c r="T143" t="inlineStr">
         <is>
           <t>No</t>
@@ -16796,7 +16348,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X143" t="inlineStr"/>
       <c r="Y143" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -16894,7 +16445,6 @@
           <t>schema + reproducibility checks</t>
         </is>
       </c>
-      <c r="S144" t="inlineStr"/>
       <c r="T144" t="inlineStr">
         <is>
           <t>No</t>
@@ -16915,7 +16465,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X144" t="inlineStr"/>
       <c r="Y144" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -17013,7 +16562,6 @@
           <t>contract tests</t>
         </is>
       </c>
-      <c r="S145" t="inlineStr"/>
       <c r="T145" t="inlineStr">
         <is>
           <t>No</t>
@@ -17034,8 +16582,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X145" t="inlineStr"/>
-      <c r="Y145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -17128,7 +16674,6 @@
           <t>provider contract + mock tests</t>
         </is>
       </c>
-      <c r="S146" t="inlineStr"/>
       <c r="T146" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -17149,7 +16694,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X146" t="inlineStr"/>
       <c r="Y146" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -17247,7 +16791,6 @@
           <t>upload/download integrity</t>
         </is>
       </c>
-      <c r="S147" t="inlineStr"/>
       <c r="T147" t="inlineStr">
         <is>
           <t>No</t>
@@ -17268,7 +16811,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X147" t="inlineStr"/>
       <c r="Y147" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -17366,7 +16908,6 @@
           <t>consent/audit test suite</t>
         </is>
       </c>
-      <c r="S148" t="inlineStr"/>
       <c r="T148" t="inlineStr">
         <is>
           <t>No</t>
@@ -17387,8 +16928,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X148" t="inlineStr"/>
-      <c r="Y148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -17481,7 +17020,6 @@
           <t>audit completeness</t>
         </is>
       </c>
-      <c r="S149" t="inlineStr"/>
       <c r="T149" t="inlineStr">
         <is>
           <t>No</t>
@@ -17502,7 +17040,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X149" t="inlineStr"/>
       <c r="Y149" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -17600,7 +17137,6 @@
           <t>mapping coverage/accuracy</t>
         </is>
       </c>
-      <c r="S150" t="inlineStr"/>
       <c r="T150" t="inlineStr">
         <is>
           <t>No</t>
@@ -17621,7 +17157,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X150" t="inlineStr"/>
       <c r="Y150" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -17719,7 +17254,6 @@
           <t>contract tests</t>
         </is>
       </c>
-      <c r="S151" t="inlineStr"/>
       <c r="T151" t="inlineStr">
         <is>
           <t>No</t>
@@ -17740,7 +17274,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X151" t="inlineStr"/>
       <c r="Y151" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -17838,7 +17371,6 @@
           <t>schema validation + privacy checks</t>
         </is>
       </c>
-      <c r="S152" t="inlineStr"/>
       <c r="T152" t="inlineStr">
         <is>
           <t>No</t>
@@ -17859,7 +17391,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X152" t="inlineStr"/>
       <c r="Y152" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -17957,7 +17488,6 @@
           <t>axe/WCAG checks</t>
         </is>
       </c>
-      <c r="S153" t="inlineStr"/>
       <c r="T153" t="inlineStr">
         <is>
           <t>No</t>
@@ -17978,8 +17508,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="X153" t="inlineStr"/>
-      <c r="Y153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -18072,7 +17600,6 @@
           <t>e2e cold-start test</t>
         </is>
       </c>
-      <c r="S154" t="inlineStr"/>
       <c r="T154" t="inlineStr">
         <is>
           <t>No</t>
@@ -18093,8 +17620,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X154" t="inlineStr"/>
-      <c r="Y154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -18187,7 +17712,6 @@
           <t>coverage audit</t>
         </is>
       </c>
-      <c r="S155" t="inlineStr"/>
       <c r="T155" t="inlineStr">
         <is>
           <t>No</t>
@@ -18208,7 +17732,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X155" t="inlineStr"/>
       <c r="Y155" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -18306,7 +17829,6 @@
           <t>migration/version tests</t>
         </is>
       </c>
-      <c r="S156" t="inlineStr"/>
       <c r="T156" t="inlineStr">
         <is>
           <t>No</t>
@@ -18327,7 +17849,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="X156" t="inlineStr"/>
       <c r="Y156" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
@@ -18440,13 +17961,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V157" t="inlineStr"/>
       <c r="W157" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="X157" t="inlineStr"/>
       <c r="Y157" t="inlineStr">
         <is>
           <t>ADDED v2: decay engine was missing from ChatGPT v1 backlog (Task 7 gap).</t>
@@ -18559,13 +18078,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V158" t="inlineStr"/>
       <c r="W158" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="X158" t="inlineStr"/>
       <c r="Y158" t="inlineStr">
         <is>
           <t>ADDED v2: research telemetry was the single biggest paper-fidelity gap.</t>
@@ -18678,13 +18195,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V159" t="inlineStr"/>
       <c r="W159" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="X159" t="inlineStr"/>
       <c r="Y159" t="inlineStr">
         <is>
           <t>ADDED v2: validation gate was missing; Smart Mark pilot integrity depends on it.</t>
@@ -18797,13 +18312,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V160" t="inlineStr"/>
       <c r="W160" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="X160" t="inlineStr"/>
       <c r="Y160" t="inlineStr">
         <is>
           <t>ADDED v2: F-053 was only a product timer; the paired-condition construct was missing.</t>
@@ -18916,13 +18429,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V161" t="inlineStr"/>
       <c r="W161" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="X161" t="inlineStr"/>
       <c r="Y161" t="inlineStr">
         <is>
           <t>ADDED v2: ChatGPT v1 listed OpenAI/Anthropic with no free-tier strategy.</t>

</xml_diff>

<commit_message>
docs: T-C03 merged (parser PR #1 @ ba36ceb + core PR #5 @ 1976540) — review added rollback + learner-serving regression proofs; post-merge CI verified; next gate T-C04 human content validation
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -2928,7 +2928,7 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>T-C02 GLM-OCR bridge MERGED to syllabai-core main @ 7c6f122 (PR #3, 2026-09-05): QP/MS pairs persist as canonical documents + T-011 paper/question/mark-scheme rows, all SUGGESTED (teacher validation gate before serving). Design: core docs/t-c02-bridge.md. Remaining: learner-facing paper browsing/filtering UI + first real batch review (T-C03).</t>
+          <t>T-C02 bridge merged @ 7c6f122 + T-C03 controlled batch MERGED 2026-09-06 (core main 1976540, parser main ba36ceb; post-merge CI 34015454011: 196/196 unit + 22/22 IT; parser 34015403577: 71/71 + conformance): the 3 real WPH11 pairs persist as canonical documents + T-011 paper/question/mark-scheme rows via the bounded GlmOcrBatchService (firehose guard, ONE transaction — whole-batch atomic, proven by a late-failure rollback IT; all SUGGESTED; rerun zero-new-rows; batch audit artifact for human review). Next gate: T-C04 human content validation before any wider batch. Remaining: learner-facing paper browsing/filtering UI.</t>
         </is>
       </c>
     </row>
@@ -3809,7 +3809,7 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>T-C02 bridge merged @ 7c6f122: MS entries map to MarkScheme/MarkPoint rows (whole-entry mark points for cells without (N) markers); verbatim MS JSONB retained in V13 glm_ocr_bridge_records; review-findings endpoint surfaces conflicts (e.g. 1A 80-vs-120) instead of merging them away. Remaining: LaTeX mark-scheme rendering + validation workflow over imported schemes.</t>
+          <t>T-C02 bridge merged @ 7c6f122; T-C03 batch MERGED 2026-09-06: 59 mark schemes + 173 mark points landed across the 3 real pairs in one controlled batch (whole-entry mark points for cells without (N) markers; verbatim MS JSONB in V13 glm_ocr_bridge_records; review findings per pair 25/27/32 — October Q18 + 1A 80-vs-120 conflicts preserved, never merged). Batch evidence: +59 versions/+59 schemes/+173 points, all SUGGESTED. Next gate: T-C04 human content validation. Remaining: LaTeX mark-scheme rendering + validation workflow over imported schemes.</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>T-C02 bridge merged @ 7c6f122: controlled ingestion entries exist — teacher-gated POST /api/v1/teacher/content/glm-ocr/pairs + ops CLI --syllabai.glmocr.pair-dir, rerun-idempotent. Batch real-corpus ingestion = T-C03 (one bounded batch + human review, in progress). Remaining: CSV/Excel teacher upload UI (Cycle 2+ scope of this row).</t>
+          <t>T-C02 bridge merged @ 7c6f122; T-C03 batch ops MERGED 2026-09-06: batch ingestion entry = ops CLI --syllabai.glmocr.batch-dir (bounded, default max 10 pairs, refused beyond; ONE transaction; deterministic reruns; batch-audit-report.json written for human review, non-zero exit on invariant failure) alongside the single-pair teacher endpoint; parser side gains the committed GlmOcrPairCli production command (markdown -&gt; five-file bundle). Regression-proven: whole-batch rollback + not-learner-servable through the real QuestionController. Next gate: T-C04 human content validation, then a batch-size decision. Remaining: CSV/Excel teacher upload UI (Cycle 2+ scope of this row).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: defer T-C04 and prioritize product UI sequence
T-C03 is complete and merged (core 1976540, parser ba36ceb). T-C04 human content
validation is READY but intentionally DEFERRED (not blocked, not abandoned) so
product-facing implementation can proceed: T-025 Tutor Chat UI -> T-028 Mastery
Dashboard -> T-029 Teacher Review UI. The 9 ordered resume prerequisites and the
validation package references are recorded in TODO.md (T-C04). The controlled
3-pair WPH11 corpus remains the only GLM-OCR production test corpus - no batch
expansion, no unvalidated serving until T-C04 passes. Core PR #1 (T-026/T-027)
stays open/draft/unmerged and isolated. Trackers (TSV+XLSX parity): F-041/F-043/F-022
notes record the active T-025 entry point (statuses honestly Not Started); F-021/
F-029/F-030 notes append the deferral record (statuses stay In Progress).
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -2928,7 +2928,7 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>T-C02 bridge merged @ 7c6f122 + T-C03 controlled batch MERGED 2026-09-06 (core main 1976540, parser main ba36ceb; post-merge CI 34015454011: 196/196 unit + 22/22 IT; parser 34015403577: 71/71 + conformance): the 3 real WPH11 pairs persist as canonical documents + T-011 paper/question/mark-scheme rows via the bounded GlmOcrBatchService (firehose guard, ONE transaction — whole-batch atomic, proven by a late-failure rollback IT; all SUGGESTED; rerun zero-new-rows; batch audit artifact for human review). Next gate: T-C04 human content validation before any wider batch. Remaining: learner-facing paper browsing/filtering UI.</t>
+          <t>T-C02 bridge merged @ 7c6f122 + T-C03 controlled batch MERGED 2026-09-06 (core main 1976540, parser main ba36ceb; post-merge CI 34015454011: 196/196 unit + 22/22 IT; parser 34015403577: 71/71 + conformance): the 3 real WPH11 pairs persist as canonical documents + T-011 paper/question/mark-scheme rows via the bounded GlmOcrBatchService (firehose guard, ONE transaction — whole-batch atomic, proven by a late-failure rollback IT; all SUGGESTED; rerun zero-new-rows; batch audit artifact for human review). Next gate: T-C04 human content validation before any wider batch. Remaining: learner-facing paper browsing/filtering UI. SESSION-13 SEQUENCING: T-C04 human validation DEFERRED (ready to resume, not blocked/abandoned — resume prerequisites in TODO.md T-C04) so product UI can proceed (T-025 -&gt; T-028 -&gt; T-029). The 3-pair controlled corpus remains the ONLY GLM-OCR production test corpus; no batch expansion and no learner serving of unvalidated GLM-OCR content until T-C04 passes.</t>
         </is>
       </c>
     </row>
@@ -3043,6 +3043,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>Referenced by T-025 (PDF deep-links / mark-scheme toggle is the companion of citation display): NOT started with T-025 v0 - citation labels + source pages render in the chat first; the in-app PDF viewer surface is scoped when T-025 lands. T-C04 is deferred/resumable (session 13); imported GLM-OCR content stays SUGGESTED and non-servable, so no unvalidated paper PDFs surface to learners.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3809,7 +3814,7 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>T-C02 bridge merged @ 7c6f122; T-C03 batch MERGED 2026-09-06: 59 mark schemes + 173 mark points landed across the 3 real pairs in one controlled batch (whole-entry mark points for cells without (N) markers; verbatim MS JSONB in V13 glm_ocr_bridge_records; review findings per pair 25/27/32 — October Q18 + 1A 80-vs-120 conflicts preserved, never merged). Batch evidence: +59 versions/+59 schemes/+173 points, all SUGGESTED. Next gate: T-C04 human content validation. Remaining: LaTeX mark-scheme rendering + validation workflow over imported schemes.</t>
+          <t>T-C02 bridge merged @ 7c6f122; T-C03 batch MERGED 2026-09-06: 59 mark schemes + 173 mark points landed across the 3 real pairs in one controlled batch (whole-entry mark points for cells without (N) markers; verbatim MS JSONB in V13 glm_ocr_bridge_records; review findings per pair 25/27/32 — October Q18 + 1A 80-vs-120 conflicts preserved, never merged). Batch evidence: +59 versions/+59 schemes/+173 points, all SUGGESTED. Next gate: T-C04 human content validation. Remaining: LaTeX mark-scheme rendering + validation workflow over imported schemes. SESSION-13 SEQUENCING: T-C04 human validation DEFERRED (ready to resume, not blocked/abandoned — resume prerequisites in TODO.md T-C04) so product UI can proceed (T-025 -&gt; T-028 -&gt; T-029). The 3-pair controlled corpus remains the ONLY GLM-OCR production test corpus; no batch expansion and no learner serving of unvalidated GLM-OCR content until T-C04 passes.</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3926,7 @@
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>T-C02 bridge merged @ 7c6f122; T-C03 batch ops MERGED 2026-09-06: batch ingestion entry = ops CLI --syllabai.glmocr.batch-dir (bounded, default max 10 pairs, refused beyond; ONE transaction; deterministic reruns; batch-audit-report.json written for human review, non-zero exit on invariant failure) alongside the single-pair teacher endpoint; parser side gains the committed GlmOcrPairCli production command (markdown -&gt; five-file bundle). Regression-proven: whole-batch rollback + not-learner-servable through the real QuestionController. Next gate: T-C04 human content validation, then a batch-size decision. Remaining: CSV/Excel teacher upload UI (Cycle 2+ scope of this row).</t>
+          <t>T-C02 bridge merged @ 7c6f122; T-C03 batch ops MERGED 2026-09-06: batch ingestion entry = ops CLI --syllabai.glmocr.batch-dir (bounded, default max 10 pairs, refused beyond; ONE transaction; deterministic reruns; batch-audit-report.json written for human review, non-zero exit on invariant failure) alongside the single-pair teacher endpoint; parser side gains the committed GlmOcrPairCli production command (markdown -&gt; five-file bundle). Regression-proven: whole-batch rollback + not-learner-servable through the real QuestionController. Next gate: T-C04 human content validation, then a batch-size decision. Remaining: CSV/Excel teacher upload UI (Cycle 2+ scope of this row). SESSION-13 SEQUENCING: T-C04 human validation DEFERRED (ready to resume, not blocked/abandoned — resume prerequisites in TODO.md T-C04) so product UI can proceed (T-025 -&gt; T-028 -&gt; T-029). The 3-pair controlled corpus remains the ONLY GLM-OCR production test corpus; no batch expansion and no learner serving of unvalidated GLM-OCR content until T-C04 passes.</t>
         </is>
       </c>
     </row>
@@ -5186,6 +5191,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>ACTIVE next task (session-13 sequencing: T-025 -&gt; T-028 -&gt; T-029; T-C04 deferred/resumable). Backend surface already merged on main (T-024): POST /api/v1/tutor/ask -&gt; TutorAnswerView (grounded answer with [n] citation markers, 1-based citations with labels + deep links, matched topics, refusal flag, model/provider/latency traceability; JWT + @CurrentUserId). No SSE backend yet - v0 is synchronous with loading/error/refusal states. Frontend lands in syllabai-web on the existing typed API client + tab shell. Diagnosis-aware policy (T-026/T-027) stays on unmerged PR #1; integrates only if/when PR #1 merges (human decision). Status stays 'Not Started' until code lands - do not mark complete because work is beginning.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5408,6 +5418,11 @@
       <c r="W44" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>ACTIVE with T-025 (citation display is the core of the chat UI): the TutorAnswerView already carries 1-based citations (label, source, page, deep link) that render under the answer next to their [n] markers. Deep links currently target the teacher content API / KG nodes - the learner-facing citation presentation is the deliberate T-025 frontend decision (SimpleCitationResolver javadoc says the learner-facing citation view arrives with T-025). ACTIVE next task (session-13 sequencing: T-025 -&gt; T-028 -&gt; T-029; T-C04 deferred/resumable). Backend surface already merged on main (T-024): POST /api/v1/tutor/ask -&gt; TutorAnswerView (grounded answer with [n] citation markers, 1-based citations with labels + deep links, matched topics, refusal flag, model/provider/latency traceability; JWT + @CurrentUserId). No SSE backend yet - v0 is synchronous with loading/error/refusal states. Frontend lands in syllabai-web on the existing typed API client + tab shell. Diagnosis-aware policy (T-026/T-027) stays on unmerged PR #1; integrates only if/when PR #1 merges (human decision). Status stays 'Not Started' until code lands.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: T-025 implemented on branch (web PR #1, CI green) — merge pending human decision
T-025 Tutor Chat UI shipped on syllabai-web codex/t-025-tutor-chat @ 3402230
(web PR #1, open): TutorChatView with [n] citation markers -> citation cards,
refusal + traceability states, transcript surviving tab switches; consumes the
merged T-024 surface only (no backend change). PR CI run 34047801205 SUCCESS
(lint + type-checked build); local lint/build verified. Trackers: F-041/F-043
-> In Progress (on branch, not merged); F-022 stays Not Started. T-C04 remains
deferred/resumable; core PR #1 (T-026/T-027) remains isolated.
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -3045,7 +3045,7 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Referenced by T-025 (PDF deep-links / mark-scheme toggle is the companion of citation display): NOT started with T-025 v0 - citation labels + source pages render in the chat first; the in-app PDF viewer surface is scoped when T-025 lands. T-C04 is deferred/resumable (session 13); imported GLM-OCR content stays SUGGESTED and non-servable, so no unvalidated paper PDFs surface to learners.</t>
+          <t>NOT started with T-025 v0 (deliberate): citation cards render verbatim source labels + pages in the chat; the in-app PDF viewer / mark-scheme toggle remains this row's scope and is revisited after the Tutor Chat UI merges. T-C04 is deferred/resumable (session 13); imported GLM-OCR content stays SUGGESTED and non-servable, so no unvalidated paper PDFs surface to learners.</t>
         </is>
       </c>
     </row>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V42" t="inlineStr">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>ACTIVE next task (session-13 sequencing: T-025 -&gt; T-028 -&gt; T-029; T-C04 deferred/resumable). Backend surface already merged on main (T-024): POST /api/v1/tutor/ask -&gt; TutorAnswerView (grounded answer with [n] citation markers, 1-based citations with labels + deep links, matched topics, refusal flag, model/provider/latency traceability; JWT + @CurrentUserId). No SSE backend yet - v0 is synchronous with loading/error/refusal states. Frontend lands in syllabai-web on the existing typed API client + tab shell. Diagnosis-aware policy (T-026/T-027) stays on unmerged PR #1; integrates only if/when PR #1 merges (human decision). Status stays 'Not Started' until code lands - do not mark complete because work is beginning.</t>
+          <t>T-025 IMPLEMENTED ON BRANCH (session 13): syllabai-web codex/t-025-tutor-chat @ 3402230, web PR #1 OPEN (not merged - human decision). PR CI run 34047801205 SUCCESS (lint + type-checked production build). Chat UI consumes the merged T-024 surface POST /api/v1/tutor/ask (synchronous v0 - no SSE backend exists; loading/error/refusal states). Transcript survives tab switches (state lifted to page; server-side sessions arrive with Spec 22 tutor/sessions endpoints). Diagnosis-aware policy (T-026/T-027) stays on unmerged core PR #1; integrates only if/when that PR merges. Remaining after merge: browser verification against the live backend; SSE when the backend ships it.</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V44" t="inlineStr">
@@ -5422,7 +5422,7 @@
       </c>
       <c r="Y44" t="inlineStr">
         <is>
-          <t>ACTIVE with T-025 (citation display is the core of the chat UI): the TutorAnswerView already carries 1-based citations (label, source, page, deep link) that render under the answer next to their [n] markers. Deep links currently target the teacher content API / KG nodes - the learner-facing citation presentation is the deliberate T-025 frontend decision (SimpleCitationResolver javadoc says the learner-facing citation view arrives with T-025). ACTIVE next task (session-13 sequencing: T-025 -&gt; T-028 -&gt; T-029; T-C04 deferred/resumable). Backend surface already merged on main (T-024): POST /api/v1/tutor/ask -&gt; TutorAnswerView (grounded answer with [n] citation markers, 1-based citations with labels + deep links, matched topics, refusal flag, model/provider/latency traceability; JWT + @CurrentUserId). No SSE backend yet - v0 is synchronous with loading/error/refusal states. Frontend lands in syllabai-web on the existing typed API client + tab shell. Diagnosis-aware policy (T-026/T-027) stays on unmerged PR #1; integrates only if/when PR #1 merges (human decision). Status stays 'Not Started' until code lands.</t>
+          <t>T-025 (on branch, web PR #1, CI green - not merged): citation display shipped as the core of the chat UI - [n] markers in the answer render as reference chips that jump to the matching citation card; cards show verbatim source labels (e.g. 'Mark scheme - p6') + source type. Role-aware deep links (documented v0 decision): teachers get 'Open source' anchors into the content/KG API; learners see reference cards (in-app PDF deep-links are F-022's surface). Traceability footer on every answer: model / provider / latency / evidence count (Spec 19).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: T-025 merged (web PR #1 fast-forward 1685f4c -> 3402230, post-merge CI 34049500636 green) — active next: T-028 Mastery Dashboard
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -3045,7 +3045,7 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>NOT started with T-025 v0 (deliberate): citation cards render verbatim source labels + pages in the chat; the in-app PDF viewer / mark-scheme toggle remains this row's scope and is revisited after the Tutor Chat UI merges. T-C04 is deferred/resumable (session 13); imported GLM-OCR content stays SUGGESTED and non-servable, so no unvalidated paper PDFs surface to learners.</t>
+          <t>NOT started (deliberate, unchanged by the T-025 merge): citation cards render verbatim source labels + pages in the chat (now on main); the in-app PDF viewer / mark-scheme toggle remains this row's own scope, revisited after the product-UI sequence (T-025 merged -&gt; T-028 active -&gt; T-029). T-C04 is deferred/resumable; imported GLM-OCR content stays SUGGESTED and non-servable, so no unvalidated paper PDFs surface to learners.</t>
         </is>
       </c>
     </row>
@@ -5193,7 +5193,7 @@
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>T-025 IMPLEMENTED ON BRANCH (session 13): syllabai-web codex/t-025-tutor-chat @ 3402230, web PR #1 OPEN (not merged - human decision). PR CI run 34047801205 SUCCESS (lint + type-checked production build). Chat UI consumes the merged T-024 surface POST /api/v1/tutor/ask (synchronous v0 - no SSE backend exists; loading/error/refusal states). Transcript survives tab switches (state lifted to page; server-side sessions arrive with Spec 22 tutor/sessions endpoints). Diagnosis-aware policy (T-026/T-027) stays on unmerged core PR #1; integrates only if/when that PR merges. Remaining after merge: browser verification against the live backend; SSE when the backend ships it.</t>
+          <t>T-025 MERGED 2026-09-07 (web PR #1, fast-forward 1685f4c -&gt; 3402230 on explicit user instruction; post-merge CI run 34049500636 SUCCESS - lint + type-checked production build, step-level verified). Chat UI consumes the merged T-024 surface POST /api/v1/tutor/ask (synchronous v0 - no SSE backend exists; loading/error/refusal states). Transcript survives tab switches (server-side sessions arrive with Spec 22 tutor/sessions endpoints). Diagnosis-aware policy (T-026/T-027) stays on unmerged core PR #1; integrates only if/when that PR merges. Remaining open (why status stays In Progress): browser verification of the chat flow against the live backend at pilot time; SSE/streaming when the backend ships it.</t>
         </is>
       </c>
     </row>
@@ -5422,7 +5422,7 @@
       </c>
       <c r="Y44" t="inlineStr">
         <is>
-          <t>T-025 (on branch, web PR #1, CI green - not merged): citation display shipped as the core of the chat UI - [n] markers in the answer render as reference chips that jump to the matching citation card; cards show verbatim source labels (e.g. 'Mark scheme - p6') + source type. Role-aware deep links (documented v0 decision): teachers get 'Open source' anchors into the content/KG API; learners see reference cards (in-app PDF deep-links are F-022's surface). Traceability footer on every answer: model / provider / latency / evidence count (Spec 19).</t>
+          <t>T-025 MERGED 2026-09-07 (web PR #1, post-merge CI green): citation display shipped as the core of the chat UI - [n] markers in the answer render as reference chips that jump to the matching citation card; cards show verbatim source labels (e.g. 'Mark scheme - p6') + source type. Role-aware deep links (documented v0 decision): teachers get 'Open source' anchors into the content/KG API; learners see reference cards (in-app PDF deep-links are F-022's surface). Traceability footer on every answer: model / provider / latency / evidence count (Spec 19). Validation metrics (retrieval recall + citation precision/groundedness) remain unmeasured - measured at pilot/research time, status stays In Progress.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: T-028 implemented on branch (core PR #6 + web PR #2, both CI green) — merges pending human decisions; core-first merge order
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -4379,7 +4379,7 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>PATCHED v2: was Cypher query + Neo4j driver.</t>
+          <t>T-028 IMPLEMENTED ON BRANCH (session 14): syllabai-core codex/t-028-mastery-dashboard @ ab7a52b, PR #6 OPEN (not merged - human decision; merge BEFORE web PR #2). Local mvn test 204/204 (196 existing + 8 new); PR CI run 34050895468 SUCCESS (mvn verify, log-inspected: 204/204 unit + 22/22 IT, BUILD SUCCESS). GET /api/v1/learners/me/knowledge-graph?rootId=... composes the VERIFIED read services (recursive-CTE tree + BKT skill states with real Ebbinghaus decay + BDT misconceptions + earliest pending review per node) + batched prerequisiteRelations - no new persistence/traversal. Honesty rules test-pinned: unpractised nodes render nulls (never zeros); misconception annotations only on MISCONCEPTION nodes; asOf pins the decay instant. Status stays In Progress until PR #6 merges and the surface is browser-verified at pilot time.</t>
         </is>
       </c>
     </row>
@@ -4603,7 +4603,7 @@
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
@@ -4614,6 +4614,11 @@
       <c r="W37" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>T-028 IMPLEMENTED ON BRANCH (session 14): syllabai-web codex/t-028-mastery-dashboard @ 18543d2, PR #2 OPEN (not merged - human decision; merge AFTER core PR #6). Local bun lint clean + type-checked production build SUCCESS; PR CI run 34051246049 SUCCESS (step-verified). 2D-first SVG KG visualizer over the F-034 personalized payload: layered columns by KG depth, band-colored nodes, solid PART_OF + dashed prerequisite edges with arrowheads, legend, keyboard-selectable nodes with aria-labels; the tree view stays the accessible alternative (view toggle in the Mastery map). 'Simplified 2D first' per TODO scope - 3D force-graph deliberately deferred. Automated UI tests + accessibility checks (this row's validation metric) remain open - web CI covers lint + type-checked build; measured at pilot time.</t>
         </is>
       </c>
     </row>
@@ -7331,7 +7336,7 @@
       </c>
       <c r="U61" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V61" t="inlineStr">
@@ -7342,6 +7347,11 @@
       <c r="W61" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>T-028 IMPLEMENTED ON BRANCH (session 14): syllabai-web codex/t-028-mastery-dashboard @ 18543d2, PR #2 OPEN (not merged - human decision). New default Dashboard tab over REAL read-model data only: mastery summary (band chips + avg effective mastery + as-of), due reviews (overdue first + Practise CTA), focus areas (lowest MEASURED mastery - labeled facts, NOT recommendations; the recommendation package stays empty), misconception watch, recent activity (attempts/accuracy/last practised). Predicted grade renders an explicit not-implemented state - never a fabricated number (research integrity). Dashboard -&gt; practice topic deep links via controlled tabs. Status stays In Progress until PR #2 merges and the surface is browser-verified at pilot time.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: T-028 merged (core PR #6 + web PR #2, user-authorized, core-first order; post-merge CI 34053354490/34053451121 green) — active next: T-029 Teacher Review UI
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -4394,7 +4394,7 @@
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>T-028 IMPLEMENTED ON BRANCH (session 14): syllabai-core codex/t-028-mastery-dashboard @ ab7a52b, PR #6 OPEN (not merged - human decision; merge BEFORE web PR #2). Local mvn test 204/204 (196 existing + 8 new); PR CI run 34050895468 SUCCESS (mvn verify, log-inspected: 204/204 unit + 22/22 IT, BUILD SUCCESS). GET /api/v1/learners/me/knowledge-graph?rootId=... composes the VERIFIED read services (recursive-CTE tree + BKT skill states with real Ebbinghaus decay + BDT misconceptions + earliest pending review per node) + batched prerequisiteRelations - no new persistence/traversal. Honesty rules test-pinned: unpractised nodes render nulls (never zeros); misconception annotations only on MISCONCEPTION nodes; asOf pins the decay instant. Status stays In Progress until PR #6 merges and the surface is browser-verified at pilot time.</t>
+          <t>T-028 MERGED 2026-09-07 (session 15, user-authorized 'OKAY PROCEED'): core PR #6 merged FIRST as a fast-forward push (main 1976540 -&gt; ab7a52b, PR closed/merged, merge_commit_sha ab7a52b; post-merge push CI run 34053354490 on main - BUILD SUCCESS, step-level verified). Pre-merge: PR CI 34050895468 success (204/204 unit + 22/22 IT, log-inspected). GET /api/v1/learners/me/knowledge-graph?rootId=... composes the VERIFIED read services (tree + misconceptions, BKT skill states with real decay, BDT states, earliest pending review); batched prerequisiteRelations; DecayParams.bandOf shared vocabulary so /state and /knowledge-graph can never disagree. Honesty rules test-pinned: unpractised nodes carry nulls (never zeros), misconception annotations only on MISCONCEPTION nodes, asOf pins the decay instant. Browser verification of the endpoint through the live UI at pilot time remains open (tracked, not blocking) - status stays In Progress.</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>T-028 IMPLEMENTED ON BRANCH (session 14): syllabai-web codex/t-028-mastery-dashboard @ 18543d2, PR #2 OPEN (not merged - human decision; merge AFTER core PR #6). Local bun lint clean + type-checked production build SUCCESS; PR CI run 34051246049 SUCCESS (step-verified). 2D-first SVG KG visualizer over the F-034 personalized payload: layered columns by KG depth, band-colored nodes, solid PART_OF + dashed prerequisite edges with arrowheads, legend, keyboard-selectable nodes with aria-labels; the tree view stays the accessible alternative (view toggle in the Mastery map). 'Simplified 2D first' per TODO scope - 3D force-graph deliberately deferred. Automated UI tests + accessibility checks (this row's validation metric) remain open - web CI covers lint + type-checked build; measured at pilot time.</t>
+          <t>T-028 MERGED 2026-09-07 (session 15, user-authorized 'OKAY PROCEED'): web PR #2 merged SECOND (after core PR #6, the runtime dependency) as a fast-forward push (main 3402230 -&gt; 18543d2, PR closed/merged, merge_commit_sha 18543d2; post-merge push CI run 34053451121 on main - Lint + type-checked production build SUCCESS, step-level verified). 2D-first SVG KG visualizer over the F-034 personalized payload: layered columns by KG depth, band-colored nodes, solid PART_OF + dashed prerequisite edges with arrowheads, legend, keyboard-selectable nodes with aria-labels; tree view stays the accessible alternative; Tree/Graph toggle + node detail card with on-demand prerequisite chains + Practise CTAs. Remaining open (why status stays In Progress): pilot-time browser verification of the graph flows; pan/zoom and 3D force-graph are explicitly out of Cycle-1 scope (2D-first by scope definition).</t>
         </is>
       </c>
     </row>
@@ -7351,7 +7351,7 @@
       </c>
       <c r="Y61" t="inlineStr">
         <is>
-          <t>T-028 IMPLEMENTED ON BRANCH (session 14): syllabai-web codex/t-028-mastery-dashboard @ 18543d2, PR #2 OPEN (not merged - human decision). New default Dashboard tab over REAL read-model data only: mastery summary (band chips + avg effective mastery + as-of), due reviews (overdue first + Practise CTA), focus areas (lowest MEASURED mastery - labeled facts, NOT recommendations; the recommendation package stays empty), misconception watch, recent activity (attempts/accuracy/last practised). Predicted grade renders an explicit not-implemented state - never a fabricated number (research integrity). Dashboard -&gt; practice topic deep links via controlled tabs. Status stays In Progress until PR #2 merges and the surface is browser-verified at pilot time.</t>
+          <t>T-028 MERGED 2026-09-07 (session 15, user-authorized 'OKAY PROCEED'): web PR #2 merged (fast-forward 3402230 -&gt; 18543d2; post-merge CI 34053451121 SUCCESS). New default Dashboard tab over REAL read-model data only: mastery summary (band chips + avg effective mastery + as-of), due reviews (overdue-first + Practise CTA), focus areas (lowest MEASURED mastery - labeled facts, NOT recommendations; the recommendation package stays empty), misconception watch, recent activity, predicted grade = explicit not-implemented state (never a fabricated number), dashboard -&gt; practice topic deep links with honest empty states. Pilot-time browser verification against the live backend remains open (tracked, not blocking) - status stays In Progress.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: T-029 implemented on branch (core PR #7 + web PR #3, both CI green; 214/214 unit + 23/23 IT incl. real-boundary teacher-surface test) — merges pending human decisions, core-first
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -5885,7 +5885,7 @@
       </c>
       <c r="Y48" t="inlineStr">
         <is>
-          <t>PATCHED v2: added Paper B kappa agreement gate to validation metric. | Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>T-029 IMPLEMENTED ON BRANCH (session 15, 2026-09-07): the Smart Mark review surface now exists end-to-end. Backend pipeline since T-021/T-022 on main (candidate generation -&gt; deterministic validation -&gt; append-only results; PROVIDER_UNAVAILABLE fails honestly). New: core PR #7 (CI 34054418641 green, 214/214 unit + 23/23 IT) + web PR #3 (CI 34054265161 green: lint + type-checked build) - both open, NOT merged (human decision; core-first). The teacher UI renders the queue, runs Smart Mark per answer, shows failure reasons verbatim (never fabricated scores). Status stays honest: merge pending + browser verification of the marking flow against the live backend at pilot time.</t>
         </is>
       </c>
     </row>
@@ -16258,7 +16258,7 @@
       </c>
       <c r="Y142" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>T-029 IMPLEMENTED ON BRANCH (session 15, 2026-09-07): human-mark override surface ships as the teacher UI's record-mark form (marks 0..part bound, per-point decisions for kappa pairing seeded from the smart breakdown, rationale comments). Backend semantics unchanged from T-022 on main: first human mark is authoritative and fires evidence exactly once; later marks revise without re-firing BKT - surfaced in the UI copy. core PR #7 + web PR #3, both CI green, NOT merged (human decision). Status stays honest until merge + pilot-time browser verification.</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="Y159" t="inlineStr">
         <is>
-          <t>ADDED v2: validation gate was missing; Smart Mark pilot integrity depends on it.</t>
+          <t>T-029 IMPLEMENTED ON BRANCH (session 15, 2026-09-07): the kappa agreement gate is now visible to teachers - latest evaluation card (kappa value, sample size, threshold, passed badge, scope, age) + recompute action with honest states (404 'no evaluation recorded yet'; 409 'no paired decisions available yet'). Fail-closed semantics unchanged from T-022 on main: below threshold, smart marks stay provisional. core PR #7 + web PR #3, both CI green, NOT merged (human decision). Status stays honest until merge.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: T-029 merged (core PR #7 @ c7d22b9 + web PR #3 @ 2c404a4, audit-passed, core-first, both post-merge CIs green) — audit added the real-HTTP JWT RBAC regression proof before merging; T-026/T-027 isolation and T-C04 deferral re-verified intact; Wave 4 not started
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -5870,7 +5870,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V48" t="inlineStr">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="Y48" t="inlineStr">
         <is>
-          <t>T-029 IMPLEMENTED ON BRANCH (session 15, 2026-09-07): the Smart Mark review surface now exists end-to-end. Backend pipeline since T-021/T-022 on main (candidate generation -&gt; deterministic validation -&gt; append-only results; PROVIDER_UNAVAILABLE fails honestly). New: core PR #7 (CI 34054418641 green, 214/214 unit + 23/23 IT) + web PR #3 (CI 34054265161 green: lint + type-checked build) - both open, NOT merged (human decision; core-first). The teacher UI renders the queue, runs Smart Mark per answer, shows failure reasons verbatim (never fabricated scores). Status stays honest: merge pending + browser verification of the marking flow against the live backend at pilot time.</t>
+          <t>T-029 MERGED 2026-09-07 (session 16, after the user-mandated pre-merge audit): the Smart Mark review surface is complete end-to-end. Backend pipeline since T-021/T-022 on main (candidate generation -&gt; deterministic validation -&gt; append-only results; PROVIDER_UNAVAILABLE fails honestly; marks drive evidence only when the k&gt;=0.60 gate has passed, fail-closed otherwise). Merged: core PR #7 fast-forward ab7a52b -&gt; c7d22b9 (post-merge CI 34094254832: 240/240 tests incl. the audit-added TeacherRouteSecurityIT 3/3 real-HTTP JWT RBAC proof) + web PR #3 fast-forward 18543d2 -&gt; 2c404a4 (post-merge CI 34094459463: lint + type-checked build). The teacher UI renders the queue, runs Smart Mark per answer, shows failure reasons verbatim (never fabricated scores). Remaining: pilot-time browser verification of the marking flow against the live backend; real-LLM agreement calibration (kappa &gt;= 0.60 on double-marked data) is the release gate and still requires human markers. κ per-paper scoping UI + queue pagination noted as future work (audit class C).</t>
         </is>
       </c>
     </row>
@@ -16243,7 +16243,7 @@
       </c>
       <c r="U142" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V142" t="inlineStr">
@@ -16258,7 +16258,7 @@
       </c>
       <c r="Y142" t="inlineStr">
         <is>
-          <t>T-029 IMPLEMENTED ON BRANCH (session 15, 2026-09-07): human-mark override surface ships as the teacher UI's record-mark form (marks 0..part bound, per-point decisions for kappa pairing seeded from the smart breakdown, rationale comments). Backend semantics unchanged from T-022 on main: first human mark is authoritative and fires evidence exactly once; later marks revise without re-firing BKT - surfaced in the UI copy. core PR #7 + web PR #3, both CI green, NOT merged (human decision). Status stays honest until merge + pilot-time browser verification.</t>
+          <t>T-029 MERGED 2026-09-07 (session 16, audit passed): the human-mark override surface ships as the teacher UI's record-mark form (marks 0..partMarks bound client-side AND server-side via ConflictException, per-point decisions for kappa pairing seeded from the smart breakdown, rationale comments). Backend semantics unchanged from T-022 on main: first human mark is authoritative and fires evidence exactly once; later marks revise without re-firing BKT — surfaced in the UI copy. Merged evidence: core PR #7 fast-forward ab7a52b -&gt; c7d22b9 (post-merge CI 34094254832 green, 240/240); web PR #3 fast-forward 18543d2 -&gt; 2c404a4 (post-merge CI 34094459463 green). Authorization is backend-enforced (SecurityConfig route rule /api/v1/teacher/** = TEACHER/ADMIN) and regression-proven by TeacherRouteSecurityIT. Remaining: pilot-time browser verification of the override flow against the live backend.</t>
         </is>
       </c>
     </row>
@@ -18217,7 +18217,7 @@
       </c>
       <c r="U159" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="W159" t="inlineStr">
@@ -18227,7 +18227,7 @@
       </c>
       <c r="Y159" t="inlineStr">
         <is>
-          <t>T-029 IMPLEMENTED ON BRANCH (session 15, 2026-09-07): the kappa agreement gate is now visible to teachers - latest evaluation card (kappa value, sample size, threshold, passed badge, scope, age) + recompute action with honest states (404 'no evaluation recorded yet'; 409 'no paired decisions available yet'). Fail-closed semantics unchanged from T-022 on main: below threshold, smart marks stay provisional. core PR #7 + web PR #3, both CI green, NOT merged (human decision). Status stays honest until merge.</t>
+          <t>T-029 MERGED 2026-09-07 (session 16, audit passed): the kappa agreement gate is now visible to teachers — latest evaluation card (kappa value, sample size, threshold, passed badge, scope, age) + recompute action with honest states (404 'no evaluation recorded yet'; 409 'no paired smart/human point decisions available yet'). Fail-closed semantics unchanged from T-022 on main: below threshold (or with no evaluation at all), smart marks stay provisional and never drive evidence; SmartMarkService checks the newest ALL/paper evaluation before firing. Merged evidence: core PR #7 fast-forward ab7a52b -&gt; c7d22b9 (post-merge CI 34094254832 green); web PR #3 fast-forward 18543d2 -&gt; 2c404a4 (post-merge CI 34094459463 green). Remaining: the actual agreement calibration (human double-marking to produce the paired decisions) is a pilot-time human activity, not a code task; per-paper scoping exists in the backend API but the UI currently calls the ALL scope (future work, audit class C).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: session 19 — finish-the-product directive executed: all merges landed, E2E adaptive loop closed, pilot configs merged
- T-033 (core PR #8 + web PR #4) MERGED: local re-verified, core-first order,
  fast-forward, post-merge CIs green
- T-026/T-027 (core PR #1) MERGED after rebase + V13→V14 migration renumber
  (git-mergeable but Flyway-duplicate — the collision is a recorded lesson);
  CI green on rebased head incl. Docker ITs; post-merge CI green
- T-034 attempt history + tutor handoff (F-059 attempt-history slice,
  charter §14): core PR #9 + web PR #5 MERGED — the missing E2E loop leg;
  read-only view over the evidence rows, honesty rules pinned by tests
- T-031 prep (core PR #10): render.yaml + pilot deployment runbook
- Workbook: F-059 → In Progress / Cycle 1 minimal-slice promotion;
  F-092/F-141/F-001 Agent Notes appended (parity 181×25 verified)
- TODO/PROGRESS/WORKLOG session records; merge ledger fully resolved
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -710,7 +710,8 @@
       </c>
       <c r="Y2" s="6" t="inlineStr">
         <is>
-          <t>PATCHED v2: was AWS/GCP/Azure + Terraform/K8s - contradicted free-tier constraint and ADR-006. | Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>PATCHED v2: was AWS/GCP/Azure + Terraform/K8s - contradicted free-tier constraint and ADR-006. | Repo remapped v2 (4-repo plan, ADR-012).
+T-031 prep MERGED (2026-09-08, core PR #10): render.yaml Blueprint + docs/DEPLOYMENT.md pilot runbook. The Render/Vercel deployment itself remains a manual operator step until the runbook checklist passes against a live URL.</t>
         </is>
       </c>
     </row>
@@ -7226,7 +7227,7 @@
       </c>
       <c r="N60" s="9" t="inlineStr">
         <is>
-          <t>Cycle 2+</t>
+          <t>Cycle 1</t>
         </is>
       </c>
       <c r="O60" s="6" t="inlineStr">
@@ -7251,7 +7252,7 @@
       </c>
       <c r="U60" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V60" s="6" t="inlineStr">
@@ -7266,7 +7267,8 @@
       </c>
       <c r="Y60" s="6" t="inlineStr">
         <is>
-          <t>ADR-016 (2026-09-07): Core student experience — subject-scoped Review Hub over unresolved problems, attempt history, measured weak areas, due reviews; measured facts stay separate from recommendations.</t>
+          <t>ADR-016 (2026-09-07): Core student experience — subject-scoped Review Hub over unresolved problems, attempt history, measured weak areas, due reviews; measured facts stay separate from recommendations.
+T-034 (2026-09-08): attempt-history minimal slice MERGED per the user's finish-the-product directive — core PR #9 (GET /api/v1/learners/me/attempts: read-only view over the immutable attempts/answers evidence rows, honesty rules pinned by tests) + web PR #5 (History tab with outcome/marks/marking-state/topic per attempt, Practise-topic deep links, honest pending/empty/error states; Ask-tutor handoff from wrong answers). Only the attempt-history leg is Cycle 1; the problematic-questions aggregation, filters and due-review cross-links stay Cycle 2+.</t>
         </is>
       </c>
     </row>
@@ -10882,7 +10884,8 @@
       </c>
       <c r="Y93" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Promoted as the primary learner-facing orchestration — next best learning action (notes, video, questions, Target Test, Tutor, review, assignment) from learner state, diagnosis, prerequisite graph, evidence, goals; recommendations are actions, not just resources. Syllabus completion / goal pacing stays a contextual ranking signal (coverage, mastery, prerequisites, review needs, exam date, study time) — completion means appropriate evidence, not mere exposure. | T-033 (2026-09-08): minimal Cycle-1 slice implemented per the user's finish-the-product directive — deterministic nba-rules/v1 baseline (GET /api/v1/learners/me/recommendations, ADR-017 rule tiers with structured evidence-backed reason codes; NextBestActionsCard on the student dashboard) on core PR #8 + web PR #4, CI green, awaiting human merge. Full F-087..F-093 architecture (learned ranking, collaborative filtering, exploration machinery, exposure evaluation) stays Cycle 2+.</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Promoted as the primary learner-facing orchestration — next best learning action (notes, video, questions, Target Test, Tutor, review, assignment) from learner state, diagnosis, prerequisite graph, evidence, goals; recommendations are actions, not just resources. Syllabus completion / goal pacing stays a contextual ranking signal (coverage, mastery, prerequisites, review needs, exam date, study time) — completion means appropriate evidence, not mere exposure. | T-033 (2026-09-08): minimal Cycle-1 slice implemented per the user's finish-the-product directive — deterministic nba-rules/v1 baseline (GET /api/v1/learners/me/recommendations, ADR-017 rule tiers with structured evidence-backed reason codes; NextBestActionsCard on the student dashboard) on core PR #8 + web PR #4, CI green, awaiting human merge. Full F-087..F-093 architecture (learned ranking, collaborative filtering, exploration machinery, exposure evaluation) stays Cycle 2+.
+T-033 MERGE (2026-09-08): core PR #8 (main c7d22b9 -&gt; 18e92ee, post-merge CI 34151756702 SUCCESS) then web PR #4 (main 2c404a4 -&gt; 9e2931d, post-merge CI 34151763333 SUCCESS) — the documented merge order respected, both fast-forward, user-authorized. Status stays In Progress: pilot-time browser verification of the full loop remains open; the full F-087..F-093 architecture stays Cycle 2+.</t>
         </is>
       </c>
     </row>
@@ -15940,6 +15943,11 @@
       <c r="W139" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="Y139" t="inlineStr">
+        <is>
+          <t>T-027 MERGED with T-026 (2026-09-08, core PR #1 rebased onto main, V13-&gt;V14 migration renumber, CI green incl. Docker ITs): prereq-gap / 3b fluency / 5a self-doubt signals live; supersede-keeps-history, 7-day expiry on reads, unsupported types never emitted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: session 20 — browser-verified adaptive loop, two critical bugs fixed on PRs (misconception read path, API base), hardening PRs open (core #11 + web #6)
- PROGRESS session-20 header + headline block: the loop is BROWSER-VERIFIED
  on a live local stack (not merely CI-verified); the required proof holds
  (same learner → real evidence → real state change → different NBA);
  deployment remains the open critical item (operator credentials).
- TODO: T-031 session-20 note (runbook checklist proven executable locally;
  env-var fix in core PR #11) + Wave 5 pilot-hardening tasks (T-035 merge
  decision, T-036 operator provisioning, T-037 pilot data seeding).
- WORKLOG session-20 entry (full evidence trail incl. the four bugs found
  live, authorization proofs, curriculum validation workflow, and the
  mocked-boundary lesson).
- Tracker: F-034/F-036/F-059/F-092 Agent Notes appended — browser-verified
  (local) state; TSV/XLSX parity 182=182 (scripts/session20_update_tracker.py).
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="Y35" s="6" t="inlineStr">
         <is>
-          <t>T-028 MERGED 2026-09-07 (session 15, user-authorized 'OKAY PROCEED'): core PR #6 merged FIRST as a fast-forward push (main 1976540 -&gt; ab7a52b, PR closed/merged, merge_commit_sha ab7a52b; post-merge push CI run 34053354490 on main - BUILD SUCCESS, step-level verified). Pre-merge: PR CI 34050895468 success (204/204 unit + 22/22 IT, log-inspected). GET /api/v1/learners/me/knowledge-graph?rootId=... composes the VERIFIED read services (tree + misconceptions, BKT skill states with real decay, BDT states, earliest pending review); batched prerequisiteRelations; DecayParams.bandOf shared vocabulary so /state and /knowledge-graph can never disagree. Honesty rules test-pinned: unpractised nodes carry nulls (never zeros), misconception annotations only on MISCONCEPTION nodes, asOf pins the decay instant. Browser verification of the endpoint through the live UI at pilot time remains open (tracked, not blocking) - status stays In Progress.</t>
+          <t>T-028 MERGED 2026-09-07 (session 15, user-authorized 'OKAY PROCEED'): core PR #6 merged FIRST as a fast-forward push (main 1976540 -&gt; ab7a52b, PR closed/merged, merge_commit_sha ab7a52b; post-merge push CI run 34053354490 on main - BUILD SUCCESS, step-level verified). Pre-merge: PR CI 34050895468 success (204/204 unit + 22/22 IT, log-inspected). GET /api/v1/learners/me/knowledge-graph?rootId=... composes the VERIFIED read services (tree + misconceptions, BKT skill states with real decay, BDT states, earliest pending review); batched prerequisiteRelations; DecayParams.bandOf shared vocabulary so /state and /knowledge-graph can never disagree. Honesty rules test-pinned: unpractised nodes carry nulls (never zeros), misconception annotations only on MISCONCEPTION nodes, asOf pins the decay instant. Browser verification of the endpoint through the live UI at pilot time remains open (tracked, not blocking) - status stays In Progress. | Session 20 (2026-09-08): browser-verified live on a real local stack (portable PG17+pgvector, core PR #11 branch): personalized KG renders mastery bands + the ACTIVE misconception annotation on MISCONCEPTION nodes — which was impossible pre-PR-#11 (the MISCONCEPTION_OF read query was doubly inverted; unit tests mocked the tree so CI stayed green). Deployed verification still pending.</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="Y37" s="6" t="inlineStr">
         <is>
-          <t>T-028 MERGED 2026-09-07 (session 15, user-authorized 'OKAY PROCEED'): web PR #2 merged SECOND (after core PR #6, the runtime dependency) as a fast-forward push (main 3402230 -&gt; 18543d2, PR closed/merged, merge_commit_sha 18543d2; post-merge push CI run 34053451121 on main - Lint + type-checked production build SUCCESS, step-level verified). 2D-first SVG KG visualizer over the F-034 personalized payload: layered columns by KG depth, band-colored nodes, solid PART_OF + dashed prerequisite edges with arrowheads, legend, keyboard-selectable nodes with aria-labels; tree view stays the accessible alternative; Tree/Graph toggle + node detail card with on-demand prerequisite chains + Practise CTAs. Remaining open (why status stays In Progress): pilot-time browser verification of the graph flows; pan/zoom and 3D force-graph are explicitly out of Cycle-1 scope (2D-first by scope definition).</t>
+          <t>T-028 MERGED 2026-09-07 (session 15, user-authorized 'OKAY PROCEED'): web PR #2 merged SECOND (after core PR #6, the runtime dependency) as a fast-forward push (main 3402230 -&gt; 18543d2, PR closed/merged, merge_commit_sha 18543d2; post-merge push CI run 34053451121 on main - Lint + type-checked production build SUCCESS, step-level verified). 2D-first SVG KG visualizer over the F-034 personalized payload: layered columns by KG depth, band-colored nodes, solid PART_OF + dashed prerequisite edges with arrowheads, legend, keyboard-selectable nodes with aria-labels; tree view stays the accessible alternative; Tree/Graph toggle + node detail card with on-demand prerequisite chains + Practise CTAs. Remaining open (why status stays In Progress): pilot-time browser verification of the graph flows; pan/zoom and 3D force-graph are explicitly out of Cycle-1 scope (2D-first by scope definition). | Session 20 (2026-09-08): browser-verified live (tree + 2D graph views render: mastery-band colors, prerequisite edges, misconception annotation after core PR #11; graph view a11y-label verified). Deployed verification still pending.</t>
         </is>
       </c>
     </row>
@@ -7268,7 +7268,7 @@
       <c r="Y60" s="6" t="inlineStr">
         <is>
           <t>ADR-016 (2026-09-07): Core student experience — subject-scoped Review Hub over unresolved problems, attempt history, measured weak areas, due reviews; measured facts stay separate from recommendations.
-T-034 (2026-09-08): attempt-history minimal slice MERGED per the user's finish-the-product directive — core PR #9 (GET /api/v1/learners/me/attempts: read-only view over the immutable attempts/answers evidence rows, honesty rules pinned by tests) + web PR #5 (History tab with outcome/marks/marking-state/topic per attempt, Practise-topic deep links, honest pending/empty/error states; Ask-tutor handoff from wrong answers). Only the attempt-history leg is Cycle 1; the problematic-questions aggregation, filters and due-review cross-links stay Cycle 2+.</t>
+T-034 (2026-09-08): attempt-history minimal slice MERGED per the user's finish-the-product directive — core PR #9 (GET /api/v1/learners/me/attempts: read-only view over the immutable attempts/answers evidence rows, honesty rules pinned by tests) + web PR #5 (History tab with outcome/marks/marking-state/topic per attempt, Practise-topic deep links, honest pending/empty/error states; Ask-tutor handoff from wrong answers). Only the attempt-history leg is Cycle 1; the problematic-questions aggregation, filters and due-review cross-links stay Cycle 2+. | Session 20 (2026-09-08): browser-verified live — MCQ attempts (option labels, misconception marker, timing, confidence) + a human-marked structured attempt (2/2 authoritative total, part breakdown, teacher-marked state); learner isolation verified (second student sees 0 attempts); refresh persists. Web PR #6 fixes the marked-structured 'awaiting marks' badge contradiction. Deployed verification pending.</t>
         </is>
       </c>
     </row>
@@ -10885,7 +10885,7 @@
       <c r="Y93" s="6" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Promoted as the primary learner-facing orchestration — next best learning action (notes, video, questions, Target Test, Tutor, review, assignment) from learner state, diagnosis, prerequisite graph, evidence, goals; recommendations are actions, not just resources. Syllabus completion / goal pacing stays a contextual ranking signal (coverage, mastery, prerequisites, review needs, exam date, study time) — completion means appropriate evidence, not mere exposure. | T-033 (2026-09-08): minimal Cycle-1 slice implemented per the user's finish-the-product directive — deterministic nba-rules/v1 baseline (GET /api/v1/learners/me/recommendations, ADR-017 rule tiers with structured evidence-backed reason codes; NextBestActionsCard on the student dashboard) on core PR #8 + web PR #4, CI green, awaiting human merge. Full F-087..F-093 architecture (learned ranking, collaborative filtering, exploration machinery, exposure evaluation) stays Cycle 2+.
-T-033 MERGE (2026-09-08): core PR #8 (main c7d22b9 -&gt; 18e92ee, post-merge CI 34151756702 SUCCESS) then web PR #4 (main 2c404a4 -&gt; 9e2931d, post-merge CI 34151763333 SUCCESS) — the documented merge order respected, both fast-forward, user-authorized. Status stays In Progress: pilot-time browser verification of the full loop remains open; the full F-087..F-093 architecture stays Cycle 2+.</t>
+T-033 MERGE (2026-09-08): core PR #8 (main c7d22b9 -&gt; 18e92ee, post-merge CI 34151756702 SUCCESS) then web PR #4 (main 2c404a4 -&gt; 9e2931d, post-merge CI 34151763333 SUCCESS) — the documented merge order respected, both fast-forward, user-authorized. Status stays In Progress: pilot-time browser verification of the full loop remains open; the full F-087..F-093 architecture stays Cycle 2+. | Session 20 (2026-09-08): browser-verified THE ADAPTIVE LOOP live: same learner, one real wrong misconception-tagged answer -&gt; NBA changed from UNCOVERED_TOPIC to MISCONCEPTION_SUSPECTED (prob 0.75, 1 evidence, parent topic cited); after a correct retry -&gt; weakened 0.50 + LOW_MASTERY (0.38 measured, 2 attempts) ranked action. The MISCONCEPTION rule family NEVER fired before core PR #11 (inverted read query); now pinned by MisconceptionSurfaceFlowIT (CI 30/30 ITs). Deployed verification pending.</t>
         </is>
       </c>
     </row>
@@ -15945,7 +15945,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Y139" t="inlineStr">
+      <c r="Y139" s="6" t="inlineStr">
         <is>
           <t>T-027 MERGED with T-026 (2026-09-08, core PR #1 rebased onto main, V13-&gt;V14 migration renumber, CI green incl. Docker ITs): prereq-gap / 3b fluency / 5a self-doubt signals live; supersede-keeps-history, 7-day expiry on reads, unsupported types never emitted.</t>
         </is>

</xml_diff>

<commit_message>
ledger: T-C38 closeout — TSV<->XLSX parity restored (TFA-07 rows 25/25 equal, F-040/F-160 synced), PROGRESS marker refreshed, AGENT.md repo table -> syllabai-hub; anchor B2 flip + B3 pin recorded (core PR #35, sweep 12/12 GREEN); T-C37 drill partial (deploy fingerprinted, teacher leg pending operator creds)
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -5079,7 +5079,7 @@
       </c>
       <c r="U41" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V41" s="6" t="inlineStr">
@@ -5094,7 +5094,7 @@
       </c>
       <c r="Y41" s="6" t="inlineStr">
         <is>
-          <t>PATCHED v2: was generic chunk-retrieve-prompt; now Paper B KA-RAG spec. | Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>PATCHED v2: was generic chunk-retrieve-prompt; now Paper B KA-RAG spec. | Repo remapped v2 (4-repo plan, ADR-012). | Status amended 2026-09-13 (tracker audit): TODO T-024 is [x] complete &amp; merged, but this row was left Not Started — a Master Spec §37 Definition-of-Done violation. Set to In Progress per the F-092 precedent (merged; pilot-time verification ongoing).</t>
         </is>
       </c>
     </row>
@@ -18140,7 +18140,7 @@
       </c>
       <c r="U158" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="W158" s="6" t="inlineStr">
@@ -18150,7 +18150,7 @@
       </c>
       <c r="Y158" s="6" t="inlineStr">
         <is>
-          <t>ADDED v2: research telemetry was the single biggest paper-fidelity gap.</t>
+          <t>ADDED v2: research telemetry was the single biggest paper-fidelity gap. | Status amended 2026-09-13 (tracker audit): TODO T-020 is [x] complete &amp; merged, but this row was left Not Started — a Master Spec §37 Definition-of-Done violation. Set to In Progress per the F-092 precedent (merged; pilot-time verification ongoing).</t>
         </is>
       </c>
     </row>
@@ -20024,12 +20024,12 @@
       </c>
       <c r="U175" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="V175" s="6" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>superz (T-C37)</t>
         </is>
       </c>
       <c r="Y175" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs: reconciliation pass — ADR ledger backfill 031-037 + ADR-037 banner + tracker v2-cutover sync (operator trace 1a15e714070287a9)
- DECISIONS.md: ledger entries backfilled for ADR-031..037 from the standalone files (mirror pattern restored; statuses verbatim: 031-035 Accepted, 036 Proposed, 037 Proposal v0.2)
- ADR-037-OFFICIAL_PAPER_QUESTION_EXTRACTION.md: verbatim-preserving status banner documenting the v2 execution divergence; GO-gated items stay open
- backlog tracker (TSV + XLSX in logical parity): Implementation Repo remapped core->v2 (148 cells, per-row Agent Notes patch markers); v2-era epics F-177..F-181 registered (ADDED v2)
- MASTER_SPEC.md: v1.3.2 (doc-accuracy alignment; 39a Cycle-1 count 36->39); README.md: spec pointer, ADR range, Execution scope count aligned
- docs-only; no code/DB/serving change; the ADR-037 GO question remains with the operator
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y182"/>
+  <dimension ref="A1:Y187"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="6" min="1" max="1"/>
@@ -680,7 +680,7 @@
       </c>
       <c r="P2" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R2" s="6" t="inlineStr">
@@ -711,7 +711,7 @@
       <c r="Y2" s="6" t="inlineStr">
         <is>
           <t>PATCHED v2: was AWS/GCP/Azure + Terraform/K8s - contradicted free-tier constraint and ADR-006. | Repo remapped v2 (4-repo plan, ADR-012).
-T-031 prep MERGED (2026-09-08, core PR #10): render.yaml Blueprint + docs/DEPLOYMENT.md pilot runbook. The Render/Vercel deployment itself remains a manual operator step until the runbook checklist passes against a live URL.</t>
+T-031 prep MERGED (2026-09-08, core PR #10): render.yaml Blueprint + docs/DEPLOYMENT.md pilot runbook. The Render/Vercel deployment itself remains a manual operator step until the runbook checklist passes against a live URL. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="P3" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R3" s="6" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="Y3" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="P4" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R4" s="6" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="Y4" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R5" s="6" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="Y5" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="P6" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R6" s="6" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="Y6" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="Y7" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="P8" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="Y8" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="Y9" s="6" t="inlineStr">
         <is>
-          <t>PATCHED v2: was Celery+Redis (Python stack) - contradicted Java ADR-001. | Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>PATCHED v2: was Celery+Redis (Python stack) - contradicted Java ADR-001. | Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1577,7 @@
       </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="Y10" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="Y11" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R12" s="6" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="Y12" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="P13" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R13" s="6" t="inlineStr">
@@ -1939,6 +1939,11 @@
       <c r="W13" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2025,7 @@
       </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R14" s="6" t="inlineStr">
@@ -2046,6 +2051,11 @@
       <c r="W14" s="6" t="inlineStr">
         <is>
           <t>Partial (UI based on role)</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2137,7 @@
       </c>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R15" s="6" t="inlineStr">
@@ -2153,6 +2163,11 @@
       <c r="W15" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2249,7 @@
       </c>
       <c r="P16" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R16" s="6" t="inlineStr">
@@ -2260,6 +2275,11 @@
       <c r="W16" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2361,7 @@
       </c>
       <c r="P17" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R17" s="6" t="inlineStr">
@@ -2367,6 +2387,11 @@
       <c r="W17" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2473,7 @@
       </c>
       <c r="P18" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R18" s="6" t="inlineStr">
@@ -2474,6 +2499,11 @@
       <c r="W18" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2585,7 @@
       </c>
       <c r="P19" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R19" s="6" t="inlineStr">
@@ -2581,6 +2611,11 @@
       <c r="W19" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2926,7 @@
       </c>
       <c r="P22" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R22" s="6" t="inlineStr">
@@ -2926,7 +2961,7 @@
       </c>
       <c r="Y22" s="6" t="inlineStr">
         <is>
-          <t>T-C02 bridge merged @ 7c6f122 + T-C03 controlled batch MERGED 2026-09-06 (core main 1976540, parser main ba36ceb; post-merge CI 34015454011: 196/196 unit + 22/22 IT; parser 34015403577: 71/71 + conformance): the 3 real WPH11 pairs persist as canonical documents + T-011 paper/question/mark-scheme rows via the bounded GlmOcrBatchService (firehose guard, ONE transaction — whole-batch atomic, proven by a late-failure rollback IT; all SUGGESTED; rerun zero-new-rows; batch audit artifact for human review). Next gate: T-C04 human content validation before any wider batch. Remaining: learner-facing paper browsing/filtering UI. SESSION-13 SEQUENCING: T-C04 human validation DEFERRED (ready to resume, not blocked/abandoned — resume prerequisites in TODO.md T-C04) so product UI can proceed (T-025 -&gt; T-028 -&gt; T-029). The 3-pair controlled corpus remains the ONLY GLM-OCR production test corpus; no batch expansion and no learner serving of unvalidated GLM-OCR content until T-C04 passes.</t>
+          <t>T-C02 bridge merged @ 7c6f122 + T-C03 controlled batch MERGED 2026-09-06 (core main 1976540, parser main ba36ceb; post-merge CI 34015454011: 196/196 unit + 22/22 IT; parser 34015403577: 71/71 + conformance): the 3 real WPH11 pairs persist as canonical documents + T-011 paper/question/mark-scheme rows via the bounded GlmOcrBatchService (firehose guard, ONE transaction — whole-batch atomic, proven by a late-failure rollback IT; all SUGGESTED; rerun zero-new-rows; batch audit artifact for human review). Next gate: T-C04 human content validation before any wider batch. Remaining: learner-facing paper browsing/filtering UI. SESSION-13 SEQUENCING: T-C04 human validation DEFERRED (ready to resume, not blocked/abandoned — resume prerequisites in TODO.md T-C04) so product UI can proceed (T-025 -&gt; T-028 -&gt; T-029). The 3-pair controlled corpus remains the ONLY GLM-OCR production test corpus; no batch expansion and no learner serving of unvalidated GLM-OCR content until T-C04 passes. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3160,7 @@
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R24" s="6" t="inlineStr">
@@ -3151,6 +3186,11 @@
       <c r="W24" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3272,7 @@
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R25" s="6" t="inlineStr">
@@ -3258,6 +3298,11 @@
       <c r="W25" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3384,7 @@
       </c>
       <c r="P26" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R26" s="6" t="inlineStr">
@@ -3369,7 +3414,7 @@
       </c>
       <c r="Y26" s="6" t="inlineStr">
         <is>
-          <t>ADR-017 (2026-09-07): Redesign as education-scoped video discovery — approved/validated subject-scoped sources, videos mapped to SpecificationPoints, served through the learning-first recommender; YouTube is a source, not the optimization objective (canonical: RECOMMENDATION_SYSTEM_ARCHITECTURE.md).</t>
+          <t>ADR-017 (2026-09-07): Redesign as education-scoped video discovery — approved/validated subject-scoped sources, videos mapped to SpecificationPoints, served through the learning-first recommender; YouTube is a source, not the optimization objective (canonical: RECOMMENDATION_SYSTEM_ARCHITECTURE.md). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3496,7 @@
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R27" s="6" t="inlineStr">
@@ -3481,7 +3526,7 @@
       </c>
       <c r="Y27" s="6" t="inlineStr">
         <is>
-          <t>ADR-017 (2026-09-07): Redesign as learning evidence/telemetry — record impression/start/progress/completion/repeat/exit with downstream learning linkage; watch time is a signal, never mastery.</t>
+          <t>ADR-017 (2026-09-07): Redesign as learning evidence/telemetry — record impression/start/progress/completion/repeat/exit with downstream learning linkage; watch time is a signal, never mastery. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3608,7 @@
       </c>
       <c r="P28" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q28" s="6" t="inlineStr">
@@ -3594,6 +3639,11 @@
       <c r="W28" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -3675,7 +3725,7 @@
       </c>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R29" s="6" t="inlineStr">
@@ -3710,7 +3760,7 @@
       </c>
       <c r="Y29" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3842,7 @@
       </c>
       <c r="P30" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R30" s="6" t="inlineStr">
@@ -3822,7 +3872,7 @@
       </c>
       <c r="Y30" s="6" t="inlineStr">
         <is>
-          <t>T-C02 bridge merged @ 7c6f122; T-C03 batch MERGED 2026-09-06: 59 mark schemes + 173 mark points landed across the 3 real pairs in one controlled batch (whole-entry mark points for cells without (N) markers; verbatim MS JSONB in V13 glm_ocr_bridge_records; review findings per pair 25/27/32 — October Q18 + 1A 80-vs-120 conflicts preserved, never merged). Batch evidence: +59 versions/+59 schemes/+173 points, all SUGGESTED. Next gate: T-C04 human content validation. Remaining: LaTeX mark-scheme rendering + validation workflow over imported schemes. SESSION-13 SEQUENCING: T-C04 human validation DEFERRED (ready to resume, not blocked/abandoned — resume prerequisites in TODO.md T-C04) so product UI can proceed (T-025 -&gt; T-028 -&gt; T-029). The 3-pair controlled corpus remains the ONLY GLM-OCR production test corpus; no batch expansion and no learner serving of unvalidated GLM-OCR content until T-C04 passes. | ADR-016 (2026-09-07): Cross-surface integration — provenance-preserving mark scheme/model answer exposed from every question surface (inline or collapsible panel, assessment context kept).</t>
+          <t>T-C02 bridge merged @ 7c6f122; T-C03 batch MERGED 2026-09-06: 59 mark schemes + 173 mark points landed across the 3 real pairs in one controlled batch (whole-entry mark points for cells without (N) markers; verbatim MS JSONB in V13 glm_ocr_bridge_records; review findings per pair 25/27/32 — October Q18 + 1A 80-vs-120 conflicts preserved, never merged). Batch evidence: +59 versions/+59 schemes/+173 points, all SUGGESTED. Next gate: T-C04 human content validation. Remaining: LaTeX mark-scheme rendering + validation workflow over imported schemes. SESSION-13 SEQUENCING: T-C04 human validation DEFERRED (ready to resume, not blocked/abandoned — resume prerequisites in TODO.md T-C04) so product UI can proceed (T-025 -&gt; T-028 -&gt; T-029). The 3-pair controlled corpus remains the ONLY GLM-OCR production test corpus; no batch expansion and no learner serving of unvalidated GLM-OCR content until T-C04 passes. | ADR-016 (2026-09-07): Cross-surface integration — provenance-preserving mark scheme/model answer exposed from every question surface (inline or collapsible panel, assessment context kept). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -4123,7 +4173,7 @@
       </c>
       <c r="P33" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q33" s="6" t="inlineStr">
@@ -4163,7 +4213,7 @@
       </c>
       <c r="Y33" s="6" t="inlineStr">
         <is>
-          <t>PATCHED v2: was 'Neo4j' - Postgres graph is ADR-005 default; Neo4j-portable schema kept. | Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>PATCHED v2: was 'Neo4j' - Postgres graph is ADR-005 default; Neo4j-portable schema kept. | Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -4245,7 +4295,7 @@
       </c>
       <c r="P34" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q34" s="6" t="inlineStr">
@@ -4285,7 +4335,7 @@
       </c>
       <c r="Y34" s="6" t="inlineStr">
         <is>
-          <t>PATCHED v2: was (Student)-[:MASTERS]-&gt;(Topic) Cypher property model. | Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Core learner-model integration — attempts map QuestionPart to SpecificationPoint(s) into learner-model inference and the KG overlay; flags/confidence may influence inference but never mutate official curriculum nodes.</t>
+          <t>PATCHED v2: was (Student)-[:MASTERS]-&gt;(Topic) Cypher property model. | Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Core learner-model integration — attempts map QuestionPart to SpecificationPoint(s) into learner-model inference and the KG overlay; flags/confidence may influence inference but never mutate official curriculum nodes. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -4367,7 +4417,7 @@
       </c>
       <c r="P35" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
@@ -4402,7 +4452,7 @@
       </c>
       <c r="Y35" s="6" t="inlineStr">
         <is>
-          <t>T-028 MERGED 2026-09-07 (session 15, user-authorized 'OKAY PROCEED'): core PR #6 merged FIRST as a fast-forward push (main 1976540 -&gt; ab7a52b, PR closed/merged, merge_commit_sha ab7a52b; post-merge push CI run 34053354490 on main - BUILD SUCCESS, step-level verified). Pre-merge: PR CI 34050895468 success (204/204 unit + 22/22 IT, log-inspected). GET /api/v1/learners/me/knowledge-graph?rootId=... composes the VERIFIED read services (tree + misconceptions, BKT skill states with real decay, BDT states, earliest pending review); batched prerequisiteRelations; DecayParams.bandOf shared vocabulary so /state and /knowledge-graph can never disagree. Honesty rules test-pinned: unpractised nodes carry nulls (never zeros), misconception annotations only on MISCONCEPTION nodes, asOf pins the decay instant. Browser verification of the endpoint through the live UI at pilot time remains open (tracked, not blocking) - status stays In Progress. | Session 20 (2026-09-08): browser-verified live on a real local stack (portable PG17+pgvector, core PR #11 branch): personalized KG renders mastery bands + the ACTIVE misconception annotation on MISCONCEPTION nodes — which was impossible pre-PR-#11 (the MISCONCEPTION_OF read query was doubly inverted; unit tests mocked the tree so CI stayed green). Deployed verification still pending.</t>
+          <t>T-028 MERGED 2026-09-07 (session 15, user-authorized 'OKAY PROCEED'): core PR #6 merged FIRST as a fast-forward push (main 1976540 -&gt; ab7a52b, PR closed/merged, merge_commit_sha ab7a52b; post-merge push CI run 34053354490 on main - BUILD SUCCESS, step-level verified). Pre-merge: PR CI 34050895468 success (204/204 unit + 22/22 IT, log-inspected). GET /api/v1/learners/me/knowledge-graph?rootId=... composes the VERIFIED read services (tree + misconceptions, BKT skill states with real decay, BDT states, earliest pending review); batched prerequisiteRelations; DecayParams.bandOf shared vocabulary so /state and /knowledge-graph can never disagree. Honesty rules test-pinned: unpractised nodes carry nulls (never zeros), misconception annotations only on MISCONCEPTION nodes, asOf pins the decay instant. Browser verification of the endpoint through the live UI at pilot time remains open (tracked, not blocking) - status stays In Progress. | Session 20 (2026-09-08): browser-verified live on a real local stack (portable PG17+pgvector, core PR #11 branch): personalized KG renders mastery bands + the ACTIVE misconception annotation on MISCONCEPTION nodes — which was impossible pre-PR-#11 (the MISCONCEPTION_OF read query was doubly inverted; unit tests mocked the tree so CI stayed green). Deployed verification still pending. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -4484,7 +4534,7 @@
       </c>
       <c r="P36" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
@@ -4514,7 +4564,7 @@
       </c>
       <c r="Y36" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -4708,7 +4758,7 @@
       </c>
       <c r="P38" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q38" s="6" t="inlineStr">
@@ -4748,7 +4798,7 @@
       </c>
       <c r="Y38" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -4937,7 +4987,7 @@
       </c>
       <c r="P40" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R40" s="6" t="inlineStr">
@@ -4972,7 +5022,7 @@
       </c>
       <c r="Y40" s="6" t="inlineStr">
         <is>
-          <t>PATCHED v2: was Pinecone/Weaviate default - ADR-004 keeps vectors in Postgres. | Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>PATCHED v2: was Pinecone/Weaviate default - ADR-004 keeps vectors in Postgres. | Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5104,7 @@
       </c>
       <c r="P41" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q41" s="6" t="inlineStr">
@@ -5094,7 +5144,7 @@
       </c>
       <c r="Y41" s="6" t="inlineStr">
         <is>
-          <t>PATCHED v2: was generic chunk-retrieve-prompt; now Paper B KA-RAG spec. | Repo remapped v2 (4-repo plan, ADR-012). | Status amended 2026-09-13 (tracker audit): TODO T-024 is [x] complete &amp; merged, but this row was left Not Started — a Master Spec §37 Definition-of-Done violation. Set to In Progress per the F-092 precedent (merged; pilot-time verification ongoing).</t>
+          <t>PATCHED v2: was generic chunk-retrieve-prompt; now Paper B KA-RAG spec. | Repo remapped v2 (4-repo plan, ADR-012). | Status amended 2026-09-13 (tracker audit): TODO T-024 is [x] complete &amp; merged, but this row was left Not Started — a Master Spec §37 Definition-of-Done violation. Set to In Progress per the F-092 precedent (merged; pilot-time verification ongoing). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -5288,7 +5338,7 @@
       </c>
       <c r="P43" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R43" s="6" t="inlineStr">
@@ -5318,7 +5368,7 @@
       </c>
       <c r="Y43" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -5517,7 +5567,7 @@
       </c>
       <c r="P45" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R45" s="6" t="inlineStr">
@@ -5547,7 +5597,7 @@
       </c>
       <c r="Y45" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5679,7 @@
       </c>
       <c r="P46" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R46" s="6" t="inlineStr">
@@ -5659,7 +5709,7 @@
       </c>
       <c r="Y46" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -5741,7 +5791,7 @@
       </c>
       <c r="P47" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R47" s="6" t="inlineStr">
@@ -5771,7 +5821,7 @@
       </c>
       <c r="Y47" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -5853,7 +5903,7 @@
       </c>
       <c r="P48" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q48" s="6" t="inlineStr">
@@ -5893,7 +5943,7 @@
       </c>
       <c r="Y48" s="6" t="inlineStr">
         <is>
-          <t>T-029 MERGED 2026-09-07 (session 16, after the user-mandated pre-merge audit): the Smart Mark review surface is complete end-to-end. Backend pipeline since T-021/T-022 on main (candidate generation -&gt; deterministic validation -&gt; append-only results; PROVIDER_UNAVAILABLE fails honestly; marks drive evidence only when the k&gt;=0.60 gate has passed, fail-closed otherwise). Merged: core PR #7 fast-forward ab7a52b -&gt; c7d22b9 (post-merge CI 34094254832: 240/240 tests incl. the audit-added TeacherRouteSecurityIT 3/3 real-HTTP JWT RBAC proof) + web PR #3 fast-forward 18543d2 -&gt; 2c404a4 (post-merge CI 34094459463: lint + type-checked build). The teacher UI renders the queue, runs Smart Mark per answer, shows failure reasons verbatim (never fabricated scores). Remaining: pilot-time browser verification of the marking flow against the live backend; real-LLM agreement calibration (kappa &gt;= 0.60 on double-marked data) is the release gate and still requires human markers. κ per-paper scoping UI + queue pagination noted as future work (audit class C). | ADR-016 (2026-09-07): Cross-surface integration — Smart Mark auto-logs attempt/evidence with AI execution metadata; AI marks are calibration evidence, never automatically human truth.</t>
+          <t>T-029 MERGED 2026-09-07 (session 16, after the user-mandated pre-merge audit): the Smart Mark review surface is complete end-to-end. Backend pipeline since T-021/T-022 on main (candidate generation -&gt; deterministic validation -&gt; append-only results; PROVIDER_UNAVAILABLE fails honestly; marks drive evidence only when the k&gt;=0.60 gate has passed, fail-closed otherwise). Merged: core PR #7 fast-forward ab7a52b -&gt; c7d22b9 (post-merge CI 34094254832: 240/240 tests incl. the audit-added TeacherRouteSecurityIT 3/3 real-HTTP JWT RBAC proof) + web PR #3 fast-forward 18543d2 -&gt; 2c404a4 (post-merge CI 34094459463: lint + type-checked build). The teacher UI renders the queue, runs Smart Mark per answer, shows failure reasons verbatim (never fabricated scores). Remaining: pilot-time browser verification of the marking flow against the live backend; real-LLM agreement calibration (kappa &gt;= 0.60 on double-marked data) is the release gate and still requires human markers. κ per-paper scoping UI + queue pagination noted as future work (audit class C). | ADR-016 (2026-09-07): Cross-surface integration — Smart Mark auto-logs attempt/evidence with AI execution metadata; AI marks are calibration evidence, never automatically human truth. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -5975,7 +6025,7 @@
       </c>
       <c r="P49" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R49" s="6" t="inlineStr">
@@ -6005,7 +6055,7 @@
       </c>
       <c r="Y49" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -6087,7 +6137,7 @@
       </c>
       <c r="P50" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q50" s="6" t="inlineStr">
@@ -6127,7 +6177,7 @@
       </c>
       <c r="Y50" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -6209,7 +6259,7 @@
       </c>
       <c r="P51" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
@@ -6239,7 +6289,7 @@
       </c>
       <c r="Y51" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Cross-surface integration (P0 aspect within this P1 feature) — Test Builder/Target Test submissions auto-log each canonical question attempt; the source test is provenance, not a new question identity.</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Cross-surface integration (P0 aspect within this P1 feature) — Test Builder/Target Test submissions auto-log each canonical question attempt; the source test is provenance, not a new question identity. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -6321,7 +6371,7 @@
       </c>
       <c r="P52" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q52" s="6" t="inlineStr">
@@ -6361,7 +6411,7 @@
       </c>
       <c r="Y52" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-018 (2026-09-07): Extended into a blueprint-driven Mock Exam Generator — versioned blueprint registry (Board→Qualification→Subject→CurriculumVersion→PaperCode→PaperType/Variant→BlueprintVersion), constrained paper assembly over validated Question/QuestionPart/AssessmentBlock candidates, hard constraints separately enforced from soft objectives, component-level fidelity validation; attempts feed the existing Learning Evidence substrate (canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md; supporting rows F-171–F-176 synced 2026-09-08).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-018 (2026-09-07): Extended into a blueprint-driven Mock Exam Generator — versioned blueprint registry (Board→Qualification→Subject→CurriculumVersion→PaperCode→PaperType/Variant→BlueprintVersion), constrained paper assembly over validated Question/QuestionPart/AssessmentBlock candidates, hard constraints separately enforced from soft objectives, component-level fidelity validation; attempts feed the existing Learning Evidence substrate (canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md; supporting rows F-171–F-176 synced 2026-09-08). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -6443,7 +6493,7 @@
       </c>
       <c r="P53" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R53" s="6" t="inlineStr">
@@ -6469,6 +6519,11 @@
       <c r="W53" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -6550,7 +6605,7 @@
       </c>
       <c r="P54" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q54" s="6" t="inlineStr">
@@ -6590,7 +6645,7 @@
       </c>
       <c r="Y54" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6727,7 @@
       </c>
       <c r="P55" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R55" s="6" t="inlineStr">
@@ -6702,7 +6757,7 @@
       </c>
       <c r="Y55" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Redesign — fixed 1/3/7/14/30-day intervals are the MVP fallback only; long-term scheduling weighs evidence, mastery, confidence, difficulty, retrieval history; the scheduler never mutates immutable attempts.</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Redesign — fixed 1/3/7/14/30-day intervals are the MVP fallback only; long-term scheduling weighs evidence, mastery, confidence, difficulty, retrieval history; the scheduler never mutates immutable attempts. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6839,7 @@
       </c>
       <c r="P56" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q56" s="6" t="inlineStr">
@@ -6819,7 +6874,7 @@
       </c>
       <c r="Y56" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Promoted to foundational evidence subsystem — immutable attempt evidence across all question sources is the canonical bridge to AssessmentEvidence/learner model/diagnosis/recommendations/teacher analytics (canonical: QUESTION_ATTEMPT_AND_LEARNING_EVIDENCE.md).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Promoted to foundational evidence subsystem — immutable attempt evidence across all question sources is the canonical bridge to AssessmentEvidence/learner model/diagnosis/recommendations/teacher analytics (canonical: QUESTION_ATTEMPT_AND_LEARNING_EVIDENCE.md). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6956,7 @@
       </c>
       <c r="P57" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R57" s="6" t="inlineStr">
@@ -6931,7 +6986,7 @@
       </c>
       <c r="Y57" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Core learner review state — problematic/doubt/self-doubt flags are mutable review state around immutable attempts; evidence, not deterministic mastery penalties (the old -0.02/+0.01 rule is rejected).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Core learner review state — problematic/doubt/self-doubt flags are mutable review state around immutable attempts; evidence, not deterministic mastery penalties (the old -0.02/+0.01 rule is rejected). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -7013,7 +7068,7 @@
       </c>
       <c r="P58" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R58" s="6" t="inlineStr">
@@ -7043,7 +7098,7 @@
       </c>
       <c r="Y58" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Review lifecycle — resolution clears urgent review state but does not prove mastery; history preserved, later review re-entry allowed.</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Review lifecycle — resolution clears urgent review state but does not prove mastery; history preserved, later review re-entry allowed. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -7462,7 +7517,7 @@
       </c>
       <c r="P62" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R62" s="6" t="inlineStr">
@@ -7492,7 +7547,7 @@
       </c>
       <c r="Y62" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7629,7 @@
       </c>
       <c r="P63" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q63" s="6" t="inlineStr">
@@ -7605,6 +7660,11 @@
       <c r="W63" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -7686,7 +7746,7 @@
       </c>
       <c r="P64" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R64" s="6" t="inlineStr">
@@ -7712,6 +7772,11 @@
       <c r="W64" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -7793,7 +7858,7 @@
       </c>
       <c r="P65" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R65" s="6" t="inlineStr">
@@ -7819,6 +7884,11 @@
       <c r="W65" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -7900,7 +7970,7 @@
       </c>
       <c r="P66" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R66" s="6" t="inlineStr">
@@ -7926,6 +7996,11 @@
       <c r="W66" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -8114,7 +8189,7 @@
       </c>
       <c r="P68" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R68" s="6" t="inlineStr">
@@ -8140,6 +8215,11 @@
       <c r="W68" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -8221,7 +8301,7 @@
       </c>
       <c r="P69" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R69" s="6" t="inlineStr">
@@ -8247,6 +8327,11 @@
       <c r="W69" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -8328,7 +8413,7 @@
       </c>
       <c r="P70" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R70" s="6" t="inlineStr">
@@ -8354,6 +8439,11 @@
       <c r="W70" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -8435,7 +8525,7 @@
       </c>
       <c r="P71" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R71" s="6" t="inlineStr">
@@ -8461,6 +8551,11 @@
       <c r="W71" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8637,7 @@
       </c>
       <c r="P72" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R72" s="6" t="inlineStr">
@@ -8568,6 +8663,11 @@
       <c r="W72" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -8649,7 +8749,7 @@
       </c>
       <c r="P73" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q73" s="6" t="inlineStr">
@@ -8684,7 +8784,7 @@
       </c>
       <c r="Y73" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -8766,7 +8866,7 @@
       </c>
       <c r="P74" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q74" s="6" t="inlineStr">
@@ -8806,7 +8906,7 @@
       </c>
       <c r="Y74" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -8995,7 +9095,7 @@
       </c>
       <c r="P76" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R76" s="6" t="inlineStr">
@@ -9021,6 +9121,11 @@
       <c r="W76" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -9209,7 +9314,7 @@
       </c>
       <c r="P78" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R78" s="6" t="inlineStr">
@@ -9235,6 +9340,11 @@
       <c r="W78" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -9316,7 +9426,7 @@
       </c>
       <c r="P79" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R79" s="6" t="inlineStr">
@@ -9346,7 +9456,7 @@
       </c>
       <c r="Y79" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Teacher lens — aggregate flags, doubt types, unresolved counts and weak SpecificationPoints for authorized classes with time windows and evidence lineage; no parallel teacher tracking model.</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 (2026-09-07): Teacher lens — aggregate flags, doubt types, unresolved counts and weak SpecificationPoints for authorized classes with time windows and evidence lineage; no parallel teacher tracking model. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -9428,7 +9538,7 @@
       </c>
       <c r="P80" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R80" s="6" t="inlineStr">
@@ -9458,7 +9568,7 @@
       </c>
       <c r="Y80" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -9540,7 +9650,7 @@
       </c>
       <c r="P81" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R81" s="6" t="inlineStr">
@@ -9566,6 +9676,11 @@
       <c r="W81" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -9647,7 +9762,7 @@
       </c>
       <c r="P82" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R82" s="6" t="inlineStr">
@@ -9673,6 +9788,11 @@
       <c r="W82" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -9754,7 +9874,7 @@
       </c>
       <c r="P83" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R83" s="6" t="inlineStr">
@@ -9780,6 +9900,11 @@
       <c r="W83" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -9861,7 +9986,7 @@
       </c>
       <c r="P84" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R84" s="6" t="inlineStr">
@@ -9887,6 +10012,11 @@
       <c r="W84" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -9968,7 +10098,7 @@
       </c>
       <c r="P85" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R85" s="6" t="inlineStr">
@@ -9994,6 +10124,11 @@
       <c r="W85" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -10075,7 +10210,7 @@
       </c>
       <c r="P86" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R86" s="6" t="inlineStr">
@@ -10101,6 +10236,11 @@
       <c r="W86" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -10182,7 +10322,7 @@
       </c>
       <c r="P87" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R87" s="6" t="inlineStr">
@@ -10208,6 +10348,11 @@
       <c r="W87" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -10289,7 +10434,7 @@
       </c>
       <c r="P88" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R88" s="6" t="inlineStr">
@@ -10319,7 +10464,7 @@
       </c>
       <c r="Y88" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Promoted as the canonical recommendation baseline — candidates from enrolled subject, SpecificationPoints, prerequisite state, weak evidence, unresolved problems, due reviews, exam goals, validated resources; candidate reasons inspectable; learning progress, not engagement.</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Promoted as the canonical recommendation baseline — candidates from enrolled subject, SpecificationPoints, prerequisite state, weak evidence, unresolved problems, due reviews, exam goals, validated resources; candidate reasons inspectable; learning progress, not engagement. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -10401,7 +10546,7 @@
       </c>
       <c r="P89" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R89" s="6" t="inlineStr">
@@ -10431,7 +10576,7 @@
       </c>
       <c r="Y89" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Kept as candidate expansion — metadata/pgvector similarity expands candidates around a diagnosed need within subject/curriculum constraints; similarity is not the final objective.</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Kept as candidate expansion — metadata/pgvector similarity expands candidates around a diagnosed need within subject/curriculum constraints; similarity is not the final objective. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -10513,7 +10658,7 @@
       </c>
       <c r="P90" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R90" s="6" t="inlineStr">
@@ -10543,7 +10688,7 @@
       </c>
       <c r="Y90" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Future experiment — collaborative signals only after sufficient interaction data and offline/downstream learning evaluation; can never override prerequisite/safety/subject/teacher hard constraints.</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Future experiment — collaborative signals only after sufficient interaction data and offline/downstream learning evaluation; can never override prerequisite/safety/subject/teacher hard constraints. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -10625,7 +10770,7 @@
       </c>
       <c r="P91" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R91" s="6" t="inlineStr">
@@ -10655,7 +10800,7 @@
       </c>
       <c r="Y91" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Canonical long-term architecture — hybrid cascade: hard constraints, rule candidates, content-based expansion, optional learned ranking, constrained exploration, next-best-action.</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Canonical long-term architecture — hybrid cascade: hard constraints, rule candidates, content-based expansion, optional learned ranking, constrained exploration, next-best-action. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -10737,7 +10882,7 @@
       </c>
       <c r="P92" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R92" s="6" t="inlineStr">
@@ -10767,7 +10912,7 @@
       </c>
       <c r="Y92" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 + ADR-017 (2026-09-07): Recommendation signals require real attempt evidence (low marks, unresolved problems, self-doubt, prerequisite weakness, review due-ness); ADR-017 rejects the hard-coded 10% random epsilon-greedy rule as a product rule — exploration targets uncovered SpecificationPoints within hard constraints.</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 + ADR-017 (2026-09-07): Recommendation signals require real attempt evidence (low marks, unresolved problems, self-doubt, prerequisite weakness, review due-ness); ADR-017 rejects the hard-coded 10% random epsilon-greedy rule as a product rule — exploration targets uncovered SpecificationPoints within hard constraints. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -10849,7 +10994,7 @@
       </c>
       <c r="P93" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q93" s="6" t="inlineStr">
@@ -10885,7 +11030,7 @@
       <c r="Y93" s="6" t="inlineStr">
         <is>
           <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-017 (2026-09-07): Promoted as the primary learner-facing orchestration — next best learning action (notes, video, questions, Target Test, Tutor, review, assignment) from learner state, diagnosis, prerequisite graph, evidence, goals; recommendations are actions, not just resources. Syllabus completion / goal pacing stays a contextual ranking signal (coverage, mastery, prerequisites, review needs, exam date, study time) — completion means appropriate evidence, not mere exposure. | T-033 (2026-09-08): minimal Cycle-1 slice implemented per the user's finish-the-product directive — deterministic nba-rules/v1 baseline (GET /api/v1/learners/me/recommendations, ADR-017 rule tiers with structured evidence-backed reason codes; NextBestActionsCard on the student dashboard) on core PR #8 + web PR #4, CI green, awaiting human merge. Full F-087..F-093 architecture (learned ranking, collaborative filtering, exploration machinery, exposure evaluation) stays Cycle 2+.
-T-033 MERGE (2026-09-08): core PR #8 (main c7d22b9 -&gt; 18e92ee, post-merge CI 34151756702 SUCCESS) then web PR #4 (main 2c404a4 -&gt; 9e2931d, post-merge CI 34151763333 SUCCESS) — the documented merge order respected, both fast-forward, user-authorized. Status stays In Progress: pilot-time browser verification of the full loop remains open; the full F-087..F-093 architecture stays Cycle 2+. | Session 20 (2026-09-08): browser-verified THE ADAPTIVE LOOP live: same learner, one real wrong misconception-tagged answer -&gt; NBA changed from UNCOVERED_TOPIC to MISCONCEPTION_SUSPECTED (prob 0.75, 1 evidence, parent topic cited); after a correct retry -&gt; weakened 0.50 + LOW_MASTERY (0.38 measured, 2 attempts) ranked action. The MISCONCEPTION rule family NEVER fired before core PR #11 (inverted read query); now pinned by MisconceptionSurfaceFlowIT (CI 30/30 ITs). Deployed verification pending.</t>
+T-033 MERGE (2026-09-08): core PR #8 (main c7d22b9 -&gt; 18e92ee, post-merge CI 34151756702 SUCCESS) then web PR #4 (main 2c404a4 -&gt; 9e2931d, post-merge CI 34151763333 SUCCESS) — the documented merge order respected, both fast-forward, user-authorized. Status stays In Progress: pilot-time browser verification of the full loop remains open; the full F-087..F-093 architecture stays Cycle 2+. | Session 20 (2026-09-08): browser-verified THE ADAPTIVE LOOP live: same learner, one real wrong misconception-tagged answer -&gt; NBA changed from UNCOVERED_TOPIC to MISCONCEPTION_SUSPECTED (prob 0.75, 1 evidence, parent topic cited); after a correct retry -&gt; weakened 0.50 + LOW_MASTERY (0.38 measured, 2 attempts) ranked action. The MISCONCEPTION rule family NEVER fired before core PR #11 (inverted read query); now pinned by MisconceptionSurfaceFlowIT (CI 30/30 ITs). Deployed verification pending. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -11079,7 +11224,7 @@
       </c>
       <c r="P95" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R95" s="6" t="inlineStr">
@@ -11109,7 +11254,7 @@
       </c>
       <c r="Y95" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -11191,7 +11336,7 @@
       </c>
       <c r="P96" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q96" s="6" t="inlineStr">
@@ -11231,7 +11376,7 @@
       </c>
       <c r="Y96" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -11313,7 +11458,7 @@
       </c>
       <c r="P97" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q97" s="6" t="inlineStr">
@@ -11348,7 +11493,7 @@
       </c>
       <c r="Y97" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -11430,7 +11575,7 @@
       </c>
       <c r="P98" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R98" s="6" t="inlineStr">
@@ -11460,7 +11605,7 @@
       </c>
       <c r="Y98" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -11542,7 +11687,7 @@
       </c>
       <c r="P99" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R99" s="6" t="inlineStr">
@@ -11572,7 +11717,7 @@
       </c>
       <c r="Y99" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -12923,7 +13068,7 @@
       </c>
       <c r="P112" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R112" s="6" t="inlineStr">
@@ -12949,6 +13094,11 @@
       <c r="W112" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -13132,7 +13282,7 @@
       </c>
       <c r="P114" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R114" s="6" t="inlineStr">
@@ -13162,7 +13312,7 @@
       </c>
       <c r="Y114" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -13244,7 +13394,7 @@
       </c>
       <c r="P115" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R115" s="6" t="inlineStr">
@@ -13270,6 +13420,11 @@
       <c r="W115" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y115" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -13351,7 +13506,7 @@
       </c>
       <c r="P116" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R116" s="6" t="inlineStr">
@@ -13381,7 +13536,7 @@
       </c>
       <c r="Y116" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -13463,7 +13618,7 @@
       </c>
       <c r="P117" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R117" s="6" t="inlineStr">
@@ -13493,7 +13648,7 @@
       </c>
       <c r="Y117" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -13575,7 +13730,7 @@
       </c>
       <c r="P118" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R118" s="6" t="inlineStr">
@@ -13605,7 +13760,7 @@
       </c>
       <c r="Y118" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -13687,7 +13842,7 @@
       </c>
       <c r="P119" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R119" s="6" t="inlineStr">
@@ -13717,7 +13872,7 @@
       </c>
       <c r="Y119" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -13799,7 +13954,7 @@
       </c>
       <c r="P120" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R120" s="6" t="inlineStr">
@@ -13829,7 +13984,7 @@
       </c>
       <c r="Y120" s="6" t="inlineStr">
         <is>
-          <t>PATCHED v2: was FastAPI/DRF - contradicted Java ADR-001. | Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>PATCHED v2: was FastAPI/DRF - contradicted Java ADR-001. | Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -13911,7 +14066,7 @@
       </c>
       <c r="P121" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R121" s="6" t="inlineStr">
@@ -13937,6 +14092,11 @@
       <c r="W121" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y121" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -14018,7 +14178,7 @@
       </c>
       <c r="P122" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R122" s="6" t="inlineStr">
@@ -14044,6 +14204,11 @@
       <c r="W122" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="Y122" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -14125,7 +14290,7 @@
       </c>
       <c r="P123" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R123" s="6" t="inlineStr">
@@ -14155,7 +14320,7 @@
       </c>
       <c r="Y123" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -14237,7 +14402,7 @@
       </c>
       <c r="P124" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R124" s="6" t="inlineStr">
@@ -14267,7 +14432,7 @@
       </c>
       <c r="Y124" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -14349,7 +14514,7 @@
       </c>
       <c r="P125" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R125" s="6" t="inlineStr">
@@ -14375,6 +14540,11 @@
       <c r="W125" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y125" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -14456,7 +14626,7 @@
       </c>
       <c r="P126" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R126" s="6" t="inlineStr">
@@ -14482,6 +14652,11 @@
       <c r="W126" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="Y126" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -14563,7 +14738,7 @@
       </c>
       <c r="P127" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R127" s="6" t="inlineStr">
@@ -14589,6 +14764,11 @@
       <c r="W127" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y127" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -14670,7 +14850,7 @@
       </c>
       <c r="P128" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R128" s="6" t="inlineStr">
@@ -14696,6 +14876,11 @@
       <c r="W128" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y128" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -14777,7 +14962,7 @@
       </c>
       <c r="P129" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R129" s="6" t="inlineStr">
@@ -14803,6 +14988,11 @@
       <c r="W129" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -14884,7 +15074,7 @@
       </c>
       <c r="P130" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R130" s="6" t="inlineStr">
@@ -14910,6 +15100,11 @@
       <c r="W130" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="Y130" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -14991,7 +15186,7 @@
       </c>
       <c r="P131" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R131" s="6" t="inlineStr">
@@ -15017,6 +15212,11 @@
       <c r="W131" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y131" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -15210,7 +15410,7 @@
       </c>
       <c r="P133" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q133" s="6" t="inlineStr">
@@ -15245,7 +15445,7 @@
       </c>
       <c r="Y133" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -15327,7 +15527,7 @@
       </c>
       <c r="P134" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q134" s="6" t="inlineStr">
@@ -15362,7 +15562,7 @@
       </c>
       <c r="Y134" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -15444,7 +15644,7 @@
       </c>
       <c r="P135" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q135" s="6" t="inlineStr">
@@ -15479,7 +15679,7 @@
       </c>
       <c r="Y135" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -15561,7 +15761,7 @@
       </c>
       <c r="P136" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q136" s="6" t="inlineStr">
@@ -15596,7 +15796,7 @@
       </c>
       <c r="Y136" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -15678,7 +15878,7 @@
       </c>
       <c r="P137" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q137" s="6" t="inlineStr">
@@ -15713,7 +15913,7 @@
       </c>
       <c r="Y137" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -15795,7 +15995,7 @@
       </c>
       <c r="P138" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q138" s="6" t="inlineStr">
@@ -15830,7 +16030,7 @@
       </c>
       <c r="Y138" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -15912,7 +16112,7 @@
       </c>
       <c r="P139" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q139" s="6" t="inlineStr">
@@ -15947,7 +16147,7 @@
       </c>
       <c r="Y139" s="6" t="inlineStr">
         <is>
-          <t>T-027 MERGED with T-026 (2026-09-08, core PR #1 rebased onto main, V13-&gt;V14 migration renumber, CI green incl. Docker ITs): prereq-gap / 3b fluency / 5a self-doubt signals live; supersede-keeps-history, 7-day expiry on reads, unsupported types never emitted.</t>
+          <t>T-027 MERGED with T-026 (2026-09-08, core PR #1 rebased onto main, V13-&gt;V14 migration renumber, CI green incl. Docker ITs): prereq-gap / 3b fluency / 5a self-doubt signals live; supersede-keeps-history, 7-day expiry on reads, unsupported types never emitted. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -16029,7 +16229,7 @@
       </c>
       <c r="P140" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q140" s="6" t="inlineStr">
@@ -16064,7 +16264,7 @@
       </c>
       <c r="Y140" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -16146,7 +16346,7 @@
       </c>
       <c r="P141" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q141" s="6" t="inlineStr">
@@ -16181,7 +16381,7 @@
       </c>
       <c r="Y141" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -16263,7 +16463,7 @@
       </c>
       <c r="P142" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q142" s="6" t="inlineStr">
@@ -16298,7 +16498,7 @@
       </c>
       <c r="Y142" s="6" t="inlineStr">
         <is>
-          <t>T-029 MERGED 2026-09-07 (session 16, audit passed): the human-mark override surface ships as the teacher UI's record-mark form (marks 0..partMarks bound client-side AND server-side via ConflictException, per-point decisions for kappa pairing seeded from the smart breakdown, rationale comments). Backend semantics unchanged from T-022 on main: first human mark is authoritative and fires evidence exactly once; later marks revise without re-firing BKT — surfaced in the UI copy. Merged evidence: core PR #7 fast-forward ab7a52b -&gt; c7d22b9 (post-merge CI 34094254832 green, 240/240); web PR #3 fast-forward 18543d2 -&gt; 2c404a4 (post-merge CI 34094459463 green). Authorization is backend-enforced (SecurityConfig route rule /api/v1/teacher/** = TEACHER/ADMIN) and regression-proven by TeacherRouteSecurityIT. Remaining: pilot-time browser verification of the override flow against the live backend.</t>
+          <t>T-029 MERGED 2026-09-07 (session 16, audit passed): the human-mark override surface ships as the teacher UI's record-mark form (marks 0..partMarks bound client-side AND server-side via ConflictException, per-point decisions for kappa pairing seeded from the smart breakdown, rationale comments). Backend semantics unchanged from T-022 on main: first human mark is authoritative and fires evidence exactly once; later marks revise without re-firing BKT — surfaced in the UI copy. Merged evidence: core PR #7 fast-forward ab7a52b -&gt; c7d22b9 (post-merge CI 34094254832 green, 240/240); web PR #3 fast-forward 18543d2 -&gt; 2c404a4 (post-merge CI 34094459463 green). Authorization is backend-enforced (SecurityConfig route rule /api/v1/teacher/** = TEACHER/ADMIN) and regression-proven by TeacherRouteSecurityIT. Remaining: pilot-time browser verification of the override flow against the live backend. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -16380,7 +16580,7 @@
       </c>
       <c r="P143" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q143" s="6" t="inlineStr">
@@ -16415,7 +16615,7 @@
       </c>
       <c r="Y143" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -16497,7 +16697,7 @@
       </c>
       <c r="P144" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q144" s="6" t="inlineStr">
@@ -16532,7 +16732,7 @@
       </c>
       <c r="Y144" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -16726,7 +16926,7 @@
       </c>
       <c r="P146" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q146" s="6" t="inlineStr">
@@ -16761,7 +16961,7 @@
       </c>
       <c r="Y146" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -16843,7 +17043,7 @@
       </c>
       <c r="P147" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q147" s="6" t="inlineStr">
@@ -16878,7 +17078,7 @@
       </c>
       <c r="Y147" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -16960,7 +17160,7 @@
       </c>
       <c r="P148" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q148" s="6" t="inlineStr">
@@ -16991,6 +17191,11 @@
       <c r="W148" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Y148" t="inlineStr">
+        <is>
+          <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -17072,7 +17277,7 @@
       </c>
       <c r="P149" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q149" s="6" t="inlineStr">
@@ -17107,7 +17312,7 @@
       </c>
       <c r="Y149" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -17189,7 +17394,7 @@
       </c>
       <c r="P150" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q150" s="6" t="inlineStr">
@@ -17224,7 +17429,7 @@
       </c>
       <c r="Y150" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -17306,7 +17511,7 @@
       </c>
       <c r="P151" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q151" s="6" t="inlineStr">
@@ -17341,7 +17546,7 @@
       </c>
       <c r="Y151" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -17423,7 +17628,7 @@
       </c>
       <c r="P152" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q152" s="6" t="inlineStr">
@@ -17458,7 +17663,7 @@
       </c>
       <c r="Y152" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 + ADR-017 (2026-09-07): Research layer — research-only telemetry (timing, self-assessment) versioned and governed separately from product-critical evidence; recommendation evaluation records policy/version, exposure, action and downstream learning outcome (CTR/watch time alone cannot establish educational benefit).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | ADR-016 + ADR-017 (2026-09-07): Research layer — research-only telemetry (timing, self-assessment) versioned and governed separately from product-critical evidence; recommendation evaluation records policy/version, exposure, action and downstream learning outcome (CTR/watch time alone cannot establish educational benefit). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -17764,7 +17969,7 @@
       </c>
       <c r="P155" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q155" s="6" t="inlineStr">
@@ -17799,7 +18004,7 @@
       </c>
       <c r="Y155" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -17881,7 +18086,7 @@
       </c>
       <c r="P156" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q156" s="6" t="inlineStr">
@@ -17916,7 +18121,7 @@
       </c>
       <c r="Y156" s="6" t="inlineStr">
         <is>
-          <t>Repo remapped v2 (4-repo plan, ADR-012).</t>
+          <t>Repo remapped v2 (4-repo plan, ADR-012). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -17998,7 +18203,7 @@
       </c>
       <c r="P157" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q157" s="6" t="inlineStr">
@@ -18033,7 +18238,7 @@
       </c>
       <c r="Y157" s="6" t="inlineStr">
         <is>
-          <t>ADDED v2: decay engine was missing from ChatGPT v1 backlog (Task 7 gap).</t>
+          <t>ADDED v2: decay engine was missing from ChatGPT v1 backlog (Task 7 gap). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -18115,7 +18320,7 @@
       </c>
       <c r="P158" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q158" s="6" t="inlineStr">
@@ -18150,7 +18355,7 @@
       </c>
       <c r="Y158" s="6" t="inlineStr">
         <is>
-          <t>ADDED v2: research telemetry was the single biggest paper-fidelity gap. | Status amended 2026-09-13 (tracker audit): TODO T-020 is [x] complete &amp; merged, but this row was left Not Started — a Master Spec §37 Definition-of-Done violation. Set to In Progress per the F-092 precedent (merged; pilot-time verification ongoing).</t>
+          <t>ADDED v2: research telemetry was the single biggest paper-fidelity gap. | Status amended 2026-09-13 (tracker audit): TODO T-020 is [x] complete &amp; merged, but this row was left Not Started — a Master Spec §37 Definition-of-Done violation. Set to In Progress per the F-092 precedent (merged; pilot-time verification ongoing). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -18232,7 +18437,7 @@
       </c>
       <c r="P159" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q159" s="6" t="inlineStr">
@@ -18267,7 +18472,7 @@
       </c>
       <c r="Y159" s="6" t="inlineStr">
         <is>
-          <t>T-029 MERGED 2026-09-07 (session 16, audit passed): the kappa agreement gate is now visible to teachers — latest evaluation card (kappa value, sample size, threshold, passed badge, scope, age) + recompute action with honest states (404 'no evaluation recorded yet'; 409 'no paired smart/human point decisions available yet'). Fail-closed semantics unchanged from T-022 on main: below threshold (or with no evaluation at all), smart marks stay provisional and never drive evidence; SmartMarkService checks the newest ALL/paper evaluation before firing. Merged evidence: core PR #7 fast-forward ab7a52b -&gt; c7d22b9 (post-merge CI 34094254832 green); web PR #3 fast-forward 18543d2 -&gt; 2c404a4 (post-merge CI 34094459463 green). Remaining: the actual agreement calibration (human double-marking to produce the paired decisions) is a pilot-time human activity, not a code task; per-paper scoping exists in the backend API but the UI currently calls the ALL scope (future work, audit class C).</t>
+          <t>T-029 MERGED 2026-09-07 (session 16, audit passed): the kappa agreement gate is now visible to teachers — latest evaluation card (kappa value, sample size, threshold, passed badge, scope, age) + recompute action with honest states (404 'no evaluation recorded yet'; 409 'no paired smart/human point decisions available yet'). Fail-closed semantics unchanged from T-022 on main: below threshold (or with no evaluation at all), smart marks stay provisional and never drive evidence; SmartMarkService checks the newest ALL/paper evaluation before firing. Merged evidence: core PR #7 fast-forward ab7a52b -&gt; c7d22b9 (post-merge CI 34094254832 green); web PR #3 fast-forward 18543d2 -&gt; 2c404a4 (post-merge CI 34094459463 green). Remaining: the actual agreement calibration (human double-marking to produce the paired decisions) is a pilot-time human activity, not a code task; per-paper scoping exists in the backend API but the UI currently calls the ALL scope (future work, audit class C). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -18349,7 +18554,7 @@
       </c>
       <c r="P160" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q160" s="6" t="inlineStr">
@@ -18384,7 +18589,7 @@
       </c>
       <c r="Y160" s="6" t="inlineStr">
         <is>
-          <t>ADDED v2: F-053 was only a product timer; the paired-condition construct was missing.</t>
+          <t>ADDED v2: F-053 was only a product timer; the paired-condition construct was missing. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -18466,7 +18671,7 @@
       </c>
       <c r="P161" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q161" s="6" t="inlineStr">
@@ -18501,7 +18706,7 @@
       </c>
       <c r="Y161" s="6" t="inlineStr">
         <is>
-          <t>ADDED v2: ChatGPT v1 listed OpenAI/Anthropic with no free-tier strategy.</t>
+          <t>ADDED v2: ChatGPT v1 listed OpenAI/Anthropic with no free-tier strategy. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -18583,7 +18788,7 @@
       </c>
       <c r="P162" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-web</t>
+          <t>syllabai-v2 + syllabai-web</t>
         </is>
       </c>
       <c r="R162" s="6" t="inlineStr">
@@ -18613,7 +18818,7 @@
       </c>
       <c r="Y162" s="6" t="inlineStr">
         <is>
-          <t>Long-term product boundary; does not expand Cycle 1. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md).</t>
+          <t>Long-term product boundary; does not expand Cycle 1. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -18695,7 +18900,7 @@
       </c>
       <c r="P163" s="6" t="inlineStr">
         <is>
-          <t>syllabai-web + syllabai-core</t>
+          <t>syllabai-web + syllabai-v2</t>
         </is>
       </c>
       <c r="R163" s="6" t="inlineStr">
@@ -18725,7 +18930,7 @@
       </c>
       <c r="Y163" s="6" t="inlineStr">
         <is>
-          <t>Save My Exams is UX reference only; SyllabAI owns the architecture/content. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md).</t>
+          <t>Save My Exams is UX reference only; SyllabAI owns the architecture/content. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -18807,7 +19012,7 @@
       </c>
       <c r="P164" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-parser</t>
+          <t>syllabai-v2 + syllabai-parser</t>
         </is>
       </c>
       <c r="R164" s="6" t="inlineStr">
@@ -18837,7 +19042,7 @@
       </c>
       <c r="Y164" s="6" t="inlineStr">
         <is>
-          <t>Canonical bridge for notes, questions, learner evidence and adaptive features. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md).</t>
+          <t>Canonical bridge for notes, questions, learner evidence and adaptive features. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -18919,7 +19124,7 @@
       </c>
       <c r="P165" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R165" s="6" t="inlineStr">
@@ -18949,7 +19154,7 @@
       </c>
       <c r="Y165" s="6" t="inlineStr">
         <is>
-          <t>Existing notes should be migrated/tagged to official points rather than flattened into broad topics. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md).</t>
+          <t>Existing notes should be migrated/tagged to official points rather than flattened into broad topics. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -19031,7 +19236,7 @@
       </c>
       <c r="P166" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-parser</t>
+          <t>syllabai-v2 + syllabai-parser</t>
         </is>
       </c>
       <c r="R166" s="6" t="inlineStr">
@@ -19061,7 +19266,7 @@
       </c>
       <c r="Y166" s="6" t="inlineStr">
         <is>
-          <t>Future extension of the existing multi-topic question direction; unvalidated mappings never become authoritative. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md).</t>
+          <t>Future extension of the existing multi-topic question direction; unvalidated mappings never become authoritative. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -19143,7 +19348,7 @@
       </c>
       <c r="P167" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-web</t>
+          <t>syllabai-v2 + syllabai-web</t>
         </is>
       </c>
       <c r="R167" s="6" t="inlineStr">
@@ -19173,7 +19378,7 @@
       </c>
       <c r="Y167" s="6" t="inlineStr">
         <is>
-          <t>Knowledge graph is structural backbone; learner state is time-aware overlay. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md).</t>
+          <t>Knowledge graph is structural backbone; learner state is time-aware overlay. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -19255,7 +19460,7 @@
       </c>
       <c r="P168" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-web</t>
+          <t>syllabai-v2 + syllabai-web</t>
         </is>
       </c>
       <c r="R168" s="6" t="inlineStr">
@@ -19285,7 +19490,7 @@
       </c>
       <c r="Y168" s="6" t="inlineStr">
         <is>
-          <t>Save My Exams-inspired product capability; SyllabAI adaptation must remain grounded in learner evidence. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md).</t>
+          <t>Save My Exams-inspired product capability; SyllabAI adaptation must remain grounded in learner evidence. Synced into the master workbook 2026-09-07 from subject-architecture-feature-addendum.tsv (ADR-014; canonical: SUBJECT_ARCHITECTURE.md). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -19362,7 +19567,7 @@
       </c>
       <c r="P169" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-web</t>
+          <t>syllabai-v2 + syllabai-web</t>
         </is>
       </c>
       <c r="R169" s="6" t="inlineStr">
@@ -19392,7 +19597,7 @@
       </c>
       <c r="Y169" s="6" t="inlineStr">
         <is>
-          <t>Canonical teacher product boundary; not a second curriculum. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum.</t>
+          <t>Canonical teacher product boundary; not a second curriculum. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -19469,7 +19674,7 @@
       </c>
       <c r="P170" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-web</t>
+          <t>syllabai-v2 + syllabai-web</t>
         </is>
       </c>
       <c r="R170" s="6" t="inlineStr">
@@ -19499,7 +19704,7 @@
       </c>
       <c r="Y170" s="6" t="inlineStr">
         <is>
-          <t>A student may simultaneously be independent and class-enrolled. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum.</t>
+          <t>A student may simultaneously be independent and class-enrolled. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -19576,7 +19781,7 @@
       </c>
       <c r="P171" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="R171" s="6" t="inlineStr">
@@ -19606,7 +19811,7 @@
       </c>
       <c r="Y171" s="6" t="inlineStr">
         <is>
-          <t>Grey graph nodes semantically mean absent teaching coverage, not low understanding. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum.</t>
+          <t>Grey graph nodes semantically mean absent teaching coverage, not low understanding. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -19683,7 +19888,7 @@
       </c>
       <c r="P172" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-web</t>
+          <t>syllabai-v2 + syllabai-web</t>
         </is>
       </c>
       <c r="R172" s="6" t="inlineStr">
@@ -19713,7 +19918,7 @@
       </c>
       <c r="Y172" s="6" t="inlineStr">
         <is>
-          <t>Separate from Data Assistant; academic/content copilot, not learner analytics. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum.</t>
+          <t>Separate from Data Assistant; academic/content copilot, not learner analytics. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -19790,7 +19995,7 @@
       </c>
       <c r="P173" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-web</t>
+          <t>syllabai-v2 + syllabai-web</t>
         </is>
       </c>
       <c r="R173" s="6" t="inlineStr">
@@ -19820,7 +20025,7 @@
       </c>
       <c r="Y173" s="6" t="inlineStr">
         <is>
-          <t>Example: Which topic is 10A weakest at? Why? What did Sara score in the latest mock?. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum.</t>
+          <t>Example: Which topic is 10A weakest at? Why? What did Sara score in the latest mock?. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -19897,7 +20102,7 @@
       </c>
       <c r="P174" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-web</t>
+          <t>syllabai-v2 + syllabai-web</t>
         </is>
       </c>
       <c r="R174" s="6" t="inlineStr">
@@ -19927,7 +20132,7 @@
       </c>
       <c r="Y174" s="6" t="inlineStr">
         <is>
-          <t>Save My Exams reference confirms topic/difficulty filtering, teacher-only questions, reuse/edit and print-ready PDFs. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum.</t>
+          <t>Save My Exams reference confirms topic/difficulty filtering, teacher-only questions, reuse/edit and print-ready PDFs. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -20004,7 +20209,7 @@
       </c>
       <c r="P175" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-web</t>
+          <t>syllabai-v2 + syllabai-web</t>
         </is>
       </c>
       <c r="R175" s="6" t="inlineStr">
@@ -20034,7 +20239,7 @@
       </c>
       <c r="Y175" s="6" t="inlineStr">
         <is>
-          <t>Class graph is an aggregation/lens over learner states. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum. | 2026-09-30 live-verified on prod Render core: full drill chain via API — class KG (329 nodes), §13.5 node→students panel, §14 member KG (374 nodes), non-member 404 (§17 gate), archived-readable; TEST fixture (archived class + 1 TEST learner + 6 attempts).</t>
+          <t>Class graph is an aggregation/lens over learner states. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum. | 2026-09-30 live-verified on prod Render core: full drill chain via API — class KG (329 nodes), §13.5 node→students panel, §14 member KG (374 nodes), non-member 404 (§17 gate), archived-readable; TEST fixture (archived class + 1 TEST learner + 6 attempts). | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -20111,7 +20316,7 @@
       </c>
       <c r="P176" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core + syllabai-web</t>
+          <t>syllabai-v2 + syllabai-web</t>
         </is>
       </c>
       <c r="R176" s="6" t="inlineStr">
@@ -20141,7 +20346,7 @@
       </c>
       <c r="Y176" s="6" t="inlineStr">
         <is>
-          <t>Never present an unexplained AI risk score. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum.</t>
+          <t>Never present an unexplained AI risk score. Synced into the master workbook 2026-09-07 from teacher-lms-feature-addendum.tsv (ADR-015; canonical: TEACHER_ARCHITECTURE.md). Complexity not scoped in the addendum. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -20223,7 +20428,7 @@
       </c>
       <c r="P177" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q177" s="6" t="inlineStr">
@@ -20263,7 +20468,7 @@
       </c>
       <c r="Y177" s="6" t="inlineStr">
         <is>
-          <t>New capability; do not duplicate F-051. IDs avoid collision with existing F-164…F-170 subject-architecture rows. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized.</t>
+          <t>New capability; do not duplicate F-051. IDs avoid collision with existing F-164…F-170 subject-architecture rows. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -20345,7 +20550,7 @@
       </c>
       <c r="P178" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q178" s="6" t="inlineStr">
@@ -20385,7 +20590,7 @@
       </c>
       <c r="Y178" s="6" t="inlineStr">
         <is>
-          <t>New supporting capability. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized.</t>
+          <t>New supporting capability. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -20467,7 +20672,7 @@
       </c>
       <c r="P179" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q179" s="6" t="inlineStr">
@@ -20507,7 +20712,7 @@
       </c>
       <c r="Y179" s="6" t="inlineStr">
         <is>
-          <t>New supporting capability. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized.</t>
+          <t>New supporting capability. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -20589,7 +20794,7 @@
       </c>
       <c r="P180" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q180" s="6" t="inlineStr">
@@ -20629,7 +20834,7 @@
       </c>
       <c r="Y180" s="6" t="inlineStr">
         <is>
-          <t>New capability; distinct from Problem Buster. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized.</t>
+          <t>New capability; distinct from Problem Buster. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -20711,7 +20916,7 @@
       </c>
       <c r="P181" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q181" s="6" t="inlineStr">
@@ -20751,7 +20956,7 @@
       </c>
       <c r="Y181" s="6" t="inlineStr">
         <is>
-          <t>Later capability; high-risk and not Cycle 1. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized.</t>
+          <t>Later capability; high-risk and not Cycle 1. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
       </c>
     </row>
@@ -20833,7 +21038,7 @@
       </c>
       <c r="P182" s="6" t="inlineStr">
         <is>
-          <t>syllabai-core</t>
+          <t>syllabai-v2</t>
         </is>
       </c>
       <c r="Q182" s="6" t="inlineStr">
@@ -20873,7 +21078,622 @@
       </c>
       <c r="Y182" s="6" t="inlineStr">
         <is>
-          <t>Future research feature; not a fake predicted-grade card. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized.</t>
+          <t>Future research feature; not a fake predicted-grade card. Synced into the master workbook 2026-09-08 from mock-exam-generator-feature-addendum.tsv (ADR-018; canonical: MOCK_EXAM_GENERATOR_ARCHITECTURE.md). Cycle 2+ — documentation only, no Cycle-1 implementation authorized. | Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>F-177</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Interactive Book Rail (T-BOOK band)</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Frontend + Content Pipeline</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>The hub serves notes and question sets but no interactive student-book spine; Unit 1 packs need a viewer with checks, glossary and tutor anchoring.</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Two-pane rail viewer over the book.block/1 contracts (11 block types) with a generic widget set, chemistry validation, glossary infrastructure, BOOK_CHECK attempt wiring and the tutor rail; pack pipeline S0-S4 with gates G1-G4.</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>ADR-BOOK-0001 band law (rollout levers, licensing gate); T-BOOK-001..010 merged (PRs #237 #238 #243 #246 #247 #248); Unit 1 rail packs (chem c01-c05) through the demo gate.</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>books/ workspaces; packages/contracts book.block/1.</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>Wave 1 - Knowledge &amp; Content</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>Cycle 1</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>syllabai-v2</t>
+        </is>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>ADR-BOOK-0001; docs/books/BOOKS-START-HERE.md</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>S0-S4 gates green; c01-c05 demo gate passed</t>
+        </is>
+      </c>
+      <c r="S183" t="inlineStr">
+        <is>
+          <t>F-148</t>
+        </is>
+      </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="V183" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X183" t="inlineStr"/>
+      <c r="Y183" t="inlineStr">
+        <is>
+          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. Original T-BOOK-xxx task ids live in the v2 .syllabai channel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>F-178</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Assessment &amp; Practice Tools</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Official past-paper question serving (ADR-037)</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Content Pipeline + Backend</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>The licensed SME corpus is topic-organized (524 questions) and cannot provide full-paper coverage; free-form LLM generation fabricates question text while answer keys stay plausible - the worst failure mode for an exam product.</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Verbatim-first converter over frozen syllabai-pastpapers artifacts with fail-closed gates (G1-G7); 16 series of 4CH1/1C wired into the hub bundle; markPoints persist per point (converter v0.7, 169/169 questions anchored).</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>ADR-037; converter + agent kit in syllabai-resources/Official-ExamQuestion/; wiring record syllabai-v2 docs/ADR-037-OFFICIAL_PAPERS_WIRING.md (restored 2026-10-21); 169 q / 930 parts / 1,405 markPoints / 135 crops.</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>syllabai-pastpapers (byte-frozen); spec-point registry; packages/contracts markPoints.</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>Wave 2 - Learner &amp; Assessment</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>Cycle 1</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>syllabai-v2</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>ADR-037; CLEAN_VERIFY_PROTOCOL_QP_MS_MARKDOWN.md</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>Gates G1-G7 green; 1754/1760 marks; negative controls 3/3 per series; independent cross-diff 161/161</t>
+        </is>
+      </c>
+      <c r="S184" t="inlineStr">
+        <is>
+          <t>F-047; F-055</t>
+        </is>
+      </c>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="V184" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="W184" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X184" t="inlineStr"/>
+      <c r="Y184" t="inlineStr">
+        <is>
+          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. (PRs #239 #249); the master-pack ADR-037 GO-gated items (tracker claim + 2C-4C scheduling) remain operator-adjudicated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>F-179</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Question/part anchor census + triage (CIE phase 4)</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Data + Tooling</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Corpus-wide question/part anchoring had gaps: anchor targets drifted across series and census run ceilings/floors were unproven, so anchor coverage could not be asserted by construction.</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Part-ROW census law (floors 5,618 by construction); fleetPaceOfRow ceiling fixes (cow-proof 180-&gt;240, prod-apply 120-&gt;300); anchor-gap census + triage of record re-pinned 12,479 questions / 17,693 parts (run-009 onGreen audit: 44/45 CIE rows mapped).</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>PRs #240 #241 #244 #250 (cie-phase4 lanes); receipts under .syllabai/receipts.</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>Wave 1 - Knowledge &amp; Content</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>syllabai-v2</t>
+        </is>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>Census re-pin receipt byte-exact (PR #250)</t>
+        </is>
+      </c>
+      <c r="S185" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U185" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="V185" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="W185" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X185" t="inlineStr"/>
+      <c r="Y185" t="inlineStr">
+        <is>
+          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record.; corpus-wide scope so left unassigned to a Cycle cut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>F-180</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>RAG AI Chatbot</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Hub assistant + question-rail management band (dc6)</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Frontend + Backend</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>The reserved assistant surface had no v2 writer and question-rail sets lacked management verbs (rename/delete).</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Assistant-surface sync wiring (v2-native, additive); question-rail rename + delete(+undo) wired to the shipped PUT/DELETE endpoints; CLA sync tier plans recorded.</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>dc6-p3b (PR #232), dc6-p3c (PR #245); plan docs DC6-* under syllabai-v2 docs/.</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>Wave 3 - Tutor &amp; Diagnostic Intelligence</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>Cycle 1</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>syllabai-v2</t>
+        </is>
+      </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>Master Spec Addendum 1.5 (Contextual Learning Assistant)</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>PR CI green; verbs wired to PUT/DELETE of record</t>
+        </is>
+      </c>
+      <c r="S186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="V186" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="W186" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X186" t="inlineStr"/>
+      <c r="Y186" t="inlineStr">
+        <is>
+          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>F-181</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Core Platform &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>v2 platform migration + cutover (T-MIG band)</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Backend + Migration</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>The Java core on the Render free tier plus a separate hub repo meant cold starts, two deployment planes and pre-cutover dual system-of-record risk.</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>TS monorepo re-platform (apps/api Hono+Drizzle+Neon serverless, apps/hub) behind golden-master parity gates; 100% migrated with the zero-core census LIVE=0 gate CI-enforced; cutover 2026-10-13 - syllabai-v2 sole system of record; syllabai-core/syllabai-hub archived read-only; Render retired.</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>MIGRATION_PLAN waves + W7-CUTOVER receipts; census gate scripts/preflight_zero_core_census.py --gate in ci.yml (commit 32272d2); CUTOVER_RETIREMENT_2026-10-13.md of record; ADR-MIG-0001/0002.</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Neon Postgres; Vercel.</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>Wave 0 - Foundations</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>Cycle 2+</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>syllabai-v2</t>
+        </is>
+      </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>docs/MIGRATION_REPORT.md 7/8</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>Zero-core census LIVE=0 (pins=7, rides-v2=2, rollback-fallback=1, dormant=5, unmapped/stale/unknown=0); bake battery 9/9 GREEN on the production alias</t>
+        </is>
+      </c>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U187" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="V187" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="W187" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X187" t="inlineStr"/>
+      <c r="Y187" t="inlineStr">
+        <is>
+          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record.; historical syllabai-core mappings on pre-existing rows corrected in this pass.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(adr-037): GO RULING — GO granted on three terms (operator adjudication, chat trace 1a15ebd93809a525): (1) the executed 1C wiring (v2 PRs #239 #249) ratified post-hoc, recorded as a process exception not a precedent; (2) tracker-claim gate CLEARED (F-178, row 184:F-178); (3) scheduling GRANTED for the remaining 4CH1 variants — registry-corrected from the prose label 2C–4C to the actual archive set {1C,1CR,2C,2CR}: 2C x16 + 1CR x11 + 2CR x11 = 38 papers through the unchanged pipeline (G0–G6 + negative controls + canaries), UNVERIFIED list = scheduled gates — and DEFERRED for new courses (ADR-019 Cycle-1 scope / §39a holds). DECISIONS.md ADR-037 entry -> ACCEPTED — GO granted; F-178 Agent Notes extended (TSV+XLSX logical parity re-verified cell-by-cell, only the 3 pre-existing quirks differ). ADR-037 body preserved verbatim — the ruling banner supersedes only the 'Still awaiting operator GO' clause.
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -1941,7 +1941,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="Y13" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -2053,7 +2053,7 @@
           <t>Partial (UI based on role)</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="Y14" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -2165,7 +2165,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="Y15" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -2277,7 +2277,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="Y16" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -2389,7 +2389,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
+      <c r="Y17" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -2501,7 +2501,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y18" t="inlineStr">
+      <c r="Y18" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -2613,7 +2613,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
+      <c r="Y19" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -3188,7 +3188,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y24" t="inlineStr">
+      <c r="Y24" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -3300,7 +3300,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y25" t="inlineStr">
+      <c r="Y25" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -3641,7 +3641,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y28" t="inlineStr">
+      <c r="Y28" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -6521,7 +6521,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y53" t="inlineStr">
+      <c r="Y53" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -7662,7 +7662,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y63" t="inlineStr">
+      <c r="Y63" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -7774,7 +7774,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y64" t="inlineStr">
+      <c r="Y64" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -7886,7 +7886,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y65" t="inlineStr">
+      <c r="Y65" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -7998,7 +7998,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y66" t="inlineStr">
+      <c r="Y66" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -8217,7 +8217,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y68" t="inlineStr">
+      <c r="Y68" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -8329,7 +8329,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y69" t="inlineStr">
+      <c r="Y69" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -8441,7 +8441,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y70" t="inlineStr">
+      <c r="Y70" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -8553,7 +8553,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y71" t="inlineStr">
+      <c r="Y71" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -8665,7 +8665,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y72" t="inlineStr">
+      <c r="Y72" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -9123,7 +9123,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y76" t="inlineStr">
+      <c r="Y76" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -9342,7 +9342,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y78" t="inlineStr">
+      <c r="Y78" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -9678,7 +9678,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y81" t="inlineStr">
+      <c r="Y81" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -9790,7 +9790,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y82" t="inlineStr">
+      <c r="Y82" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -9902,7 +9902,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y83" t="inlineStr">
+      <c r="Y83" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -10014,7 +10014,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y84" t="inlineStr">
+      <c r="Y84" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -10126,7 +10126,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y85" t="inlineStr">
+      <c r="Y85" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -10238,7 +10238,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y86" t="inlineStr">
+      <c r="Y86" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -10350,7 +10350,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y87" t="inlineStr">
+      <c r="Y87" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -13096,7 +13096,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y112" t="inlineStr">
+      <c r="Y112" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -13422,7 +13422,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y115" t="inlineStr">
+      <c r="Y115" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -14094,7 +14094,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y121" t="inlineStr">
+      <c r="Y121" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -14206,7 +14206,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Y122" t="inlineStr">
+      <c r="Y122" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -14542,7 +14542,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y125" t="inlineStr">
+      <c r="Y125" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -14654,7 +14654,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Y126" t="inlineStr">
+      <c r="Y126" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -14766,7 +14766,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y127" t="inlineStr">
+      <c r="Y127" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -14878,7 +14878,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y128" t="inlineStr">
+      <c r="Y128" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -14990,7 +14990,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y129" t="inlineStr">
+      <c r="Y129" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -15102,7 +15102,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Y130" t="inlineStr">
+      <c r="Y130" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -15214,7 +15214,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y131" t="inlineStr">
+      <c r="Y131" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -17193,7 +17193,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Y148" t="inlineStr">
+      <c r="Y148" s="6" t="inlineStr">
         <is>
           <t>Repo remapped syllabai-v2 (2026-10-13 cutover; syllabai-core archived read-only).</t>
         </is>
@@ -21083,615 +21083,615 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr">
+      <c r="A183" s="6" t="inlineStr">
         <is>
           <t>F-177</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr">
+      <c r="B183" s="6" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
+      <c r="C183" s="6" t="inlineStr">
         <is>
           <t>Interactive Book Rail (T-BOOK band)</t>
         </is>
       </c>
-      <c r="D183" t="inlineStr">
+      <c r="D183" s="6" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr">
+      <c r="E183" s="6" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr">
+      <c r="F183" s="6" t="inlineStr">
         <is>
           <t>Frontend + Content Pipeline</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr">
+      <c r="G183" s="6" t="inlineStr">
         <is>
           <t>The hub serves notes and question sets but no interactive student-book spine; Unit 1 packs need a viewer with checks, glossary and tutor anchoring.</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr">
+      <c r="H183" s="6" t="inlineStr">
         <is>
           <t>Two-pane rail viewer over the book.block/1 contracts (11 block types) with a generic widget set, chemistry validation, glossary infrastructure, BOOK_CHECK attempt wiring and the tutor rail; pack pipeline S0-S4 with gates G1-G4.</t>
         </is>
       </c>
-      <c r="I183" t="inlineStr">
+      <c r="I183" s="6" t="inlineStr">
         <is>
           <t>ADR-BOOK-0001 band law (rollout levers, licensing gate); T-BOOK-001..010 merged (PRs #237 #238 #243 #246 #247 #248); Unit 1 rail packs (chem c01-c05) through the demo gate.</t>
         </is>
       </c>
-      <c r="J183" t="inlineStr">
+      <c r="J183" s="6" t="inlineStr">
         <is>
           <t>books/ workspaces; packages/contracts book.block/1.</t>
         </is>
       </c>
-      <c r="K183" t="inlineStr">
+      <c r="K183" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="L183" t="inlineStr">
+      <c r="L183" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="M183" t="inlineStr">
+      <c r="M183" s="6" t="inlineStr">
         <is>
           <t>Wave 1 - Knowledge &amp; Content</t>
         </is>
       </c>
-      <c r="N183" t="inlineStr">
+      <c r="N183" s="6" t="inlineStr">
         <is>
           <t>Cycle 1</t>
         </is>
       </c>
-      <c r="O183" t="inlineStr">
+      <c r="O183" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="P183" t="inlineStr">
+      <c r="P183" s="6" t="inlineStr">
         <is>
           <t>syllabai-v2</t>
         </is>
       </c>
-      <c r="Q183" t="inlineStr">
+      <c r="Q183" s="6" t="inlineStr">
         <is>
           <t>ADR-BOOK-0001; docs/books/BOOKS-START-HERE.md</t>
         </is>
       </c>
-      <c r="R183" t="inlineStr">
+      <c r="R183" s="6" t="inlineStr">
         <is>
           <t>S0-S4 gates green; c01-c05 demo gate passed</t>
         </is>
       </c>
-      <c r="S183" t="inlineStr">
+      <c r="S183" s="6" t="inlineStr">
         <is>
           <t>F-148</t>
         </is>
       </c>
-      <c r="T183" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U183" t="inlineStr">
+      <c r="T183" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U183" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="V183" t="inlineStr">
+      <c r="V183" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W183" t="inlineStr">
+      <c r="W183" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="X183" t="inlineStr"/>
-      <c r="Y183" t="inlineStr">
+      <c r="X183" s="6" t="inlineStr"/>
+      <c r="Y183" s="6" t="inlineStr">
         <is>
           <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. Original T-BOOK-xxx task ids live in the v2 .syllabai channel.</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="inlineStr">
+      <c r="A184" s="6" t="inlineStr">
         <is>
           <t>F-178</t>
         </is>
       </c>
-      <c r="B184" t="inlineStr">
+      <c r="B184" s="6" t="inlineStr">
         <is>
           <t>Assessment &amp; Practice Tools</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr">
+      <c r="C184" s="6" t="inlineStr">
         <is>
           <t>Official past-paper question serving (ADR-037)</t>
         </is>
       </c>
-      <c r="D184" t="inlineStr">
+      <c r="D184" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr">
+      <c r="E184" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr">
+      <c r="F184" s="6" t="inlineStr">
         <is>
           <t>Content Pipeline + Backend</t>
         </is>
       </c>
-      <c r="G184" t="inlineStr">
+      <c r="G184" s="6" t="inlineStr">
         <is>
           <t>The licensed SME corpus is topic-organized (524 questions) and cannot provide full-paper coverage; free-form LLM generation fabricates question text while answer keys stay plausible - the worst failure mode for an exam product.</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr">
+      <c r="H184" s="6" t="inlineStr">
         <is>
           <t>Verbatim-first converter over frozen syllabai-pastpapers artifacts with fail-closed gates (G1-G7); 16 series of 4CH1/1C wired into the hub bundle; markPoints persist per point (converter v0.7, 169/169 questions anchored).</t>
         </is>
       </c>
-      <c r="I184" t="inlineStr">
+      <c r="I184" s="6" t="inlineStr">
         <is>
           <t>ADR-037; converter + agent kit in syllabai-resources/Official-ExamQuestion/; wiring record syllabai-v2 docs/ADR-037-OFFICIAL_PAPERS_WIRING.md (restored 2026-10-21); 169 q / 930 parts / 1,405 markPoints / 135 crops.</t>
         </is>
       </c>
-      <c r="J184" t="inlineStr">
+      <c r="J184" s="6" t="inlineStr">
         <is>
           <t>syllabai-pastpapers (byte-frozen); spec-point registry; packages/contracts markPoints.</t>
         </is>
       </c>
-      <c r="K184" t="inlineStr">
+      <c r="K184" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="L184" t="inlineStr">
+      <c r="L184" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="M184" t="inlineStr">
+      <c r="M184" s="6" t="inlineStr">
         <is>
           <t>Wave 2 - Learner &amp; Assessment</t>
         </is>
       </c>
-      <c r="N184" t="inlineStr">
+      <c r="N184" s="6" t="inlineStr">
         <is>
           <t>Cycle 1</t>
         </is>
       </c>
-      <c r="O184" t="inlineStr">
+      <c r="O184" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="P184" t="inlineStr">
+      <c r="P184" s="6" t="inlineStr">
         <is>
           <t>syllabai-v2</t>
         </is>
       </c>
-      <c r="Q184" t="inlineStr">
+      <c r="Q184" s="6" t="inlineStr">
         <is>
           <t>ADR-037; CLEAN_VERIFY_PROTOCOL_QP_MS_MARKDOWN.md</t>
         </is>
       </c>
-      <c r="R184" t="inlineStr">
+      <c r="R184" s="6" t="inlineStr">
         <is>
           <t>Gates G1-G7 green; 1754/1760 marks; negative controls 3/3 per series; independent cross-diff 161/161</t>
         </is>
       </c>
-      <c r="S184" t="inlineStr">
+      <c r="S184" s="6" t="inlineStr">
         <is>
           <t>F-047; F-055</t>
         </is>
       </c>
-      <c r="T184" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U184" t="inlineStr">
+      <c r="T184" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U184" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="V184" t="inlineStr">
+      <c r="V184" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W184" t="inlineStr">
+      <c r="W184" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="X184" t="inlineStr"/>
-      <c r="Y184" t="inlineStr">
-        <is>
-          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. (PRs #239 #249); the master-pack ADR-037 GO-gated items (tracker claim + 2C-4C scheduling) remain operator-adjudicated.</t>
+      <c r="X184" s="6" t="inlineStr"/>
+      <c r="Y184" s="6" t="inlineStr">
+        <is>
+          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. (PRs #239 #249); the master-pack ADR-037 GO-gated items (tracker claim + 2C-4C scheduling) remain operator-adjudicated.| GO RULING v2 (2026-10-21, operator trace 1a15ebd93809a525): GO granted - the executed 1C wiring (PRs #239 #249) is ratified post-hoc (process exception, not precedent); tracker-claim gate CLEARED; scheduling GRANTED for the remaining 4CH1 variants 2C x16 + 1CR x11 + 2CR x11 = 38 papers (registry-corrected from the ADR prose label "2C-4C"; same pipeline unchanged, UNVERIFIED list = scheduled gates); new courses DEFERRED (ADR-019 Cycle-1 scope / spec 39a).</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" t="inlineStr">
+      <c r="A185" s="6" t="inlineStr">
         <is>
           <t>F-179</t>
         </is>
       </c>
-      <c r="B185" t="inlineStr">
+      <c r="B185" s="6" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr">
+      <c r="C185" s="6" t="inlineStr">
         <is>
           <t>Question/part anchor census + triage (CIE phase 4)</t>
         </is>
       </c>
-      <c r="D185" t="inlineStr">
+      <c r="D185" s="6" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="E185" t="inlineStr">
+      <c r="E185" s="6" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr">
+      <c r="F185" s="6" t="inlineStr">
         <is>
           <t>Data + Tooling</t>
         </is>
       </c>
-      <c r="G185" t="inlineStr">
+      <c r="G185" s="6" t="inlineStr">
         <is>
           <t>Corpus-wide question/part anchoring had gaps: anchor targets drifted across series and census run ceilings/floors were unproven, so anchor coverage could not be asserted by construction.</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr">
+      <c r="H185" s="6" t="inlineStr">
         <is>
           <t>Part-ROW census law (floors 5,618 by construction); fleetPaceOfRow ceiling fixes (cow-proof 180-&gt;240, prod-apply 120-&gt;300); anchor-gap census + triage of record re-pinned 12,479 questions / 17,693 parts (run-009 onGreen audit: 44/45 CIE rows mapped).</t>
         </is>
       </c>
-      <c r="I185" t="inlineStr">
+      <c r="I185" s="6" t="inlineStr">
         <is>
           <t>PRs #240 #241 #244 #250 (cie-phase4 lanes); receipts under .syllabai/receipts.</t>
         </is>
       </c>
-      <c r="J185" t="inlineStr">
+      <c r="J185" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K185" t="inlineStr">
+      <c r="K185" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="L185" t="inlineStr">
+      <c r="L185" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="M185" t="inlineStr">
+      <c r="M185" s="6" t="inlineStr">
         <is>
           <t>Wave 1 - Knowledge &amp; Content</t>
         </is>
       </c>
-      <c r="N185" t="inlineStr">
+      <c r="N185" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O185" t="inlineStr">
+      <c r="O185" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="P185" t="inlineStr">
+      <c r="P185" s="6" t="inlineStr">
         <is>
           <t>syllabai-v2</t>
         </is>
       </c>
-      <c r="Q185" t="inlineStr">
+      <c r="Q185" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="R185" t="inlineStr">
+      <c r="R185" s="6" t="inlineStr">
         <is>
           <t>Census re-pin receipt byte-exact (PR #250)</t>
         </is>
       </c>
-      <c r="S185" t="inlineStr">
+      <c r="S185" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="T185" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U185" t="inlineStr">
+      <c r="T185" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U185" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="V185" t="inlineStr">
+      <c r="V185" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W185" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="X185" t="inlineStr"/>
-      <c r="Y185" t="inlineStr">
+      <c r="W185" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X185" s="6" t="inlineStr"/>
+      <c r="Y185" s="6" t="inlineStr">
         <is>
           <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record.; corpus-wide scope so left unassigned to a Cycle cut.</t>
         </is>
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="inlineStr">
+      <c r="A186" s="6" t="inlineStr">
         <is>
           <t>F-180</t>
         </is>
       </c>
-      <c r="B186" t="inlineStr">
+      <c r="B186" s="6" t="inlineStr">
         <is>
           <t>RAG AI Chatbot</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr">
+      <c r="C186" s="6" t="inlineStr">
         <is>
           <t>Hub assistant + question-rail management band (dc6)</t>
         </is>
       </c>
-      <c r="D186" t="inlineStr">
+      <c r="D186" s="6" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="E186" t="inlineStr">
+      <c r="E186" s="6" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr">
+      <c r="F186" s="6" t="inlineStr">
         <is>
           <t>Frontend + Backend</t>
         </is>
       </c>
-      <c r="G186" t="inlineStr">
+      <c r="G186" s="6" t="inlineStr">
         <is>
           <t>The reserved assistant surface had no v2 writer and question-rail sets lacked management verbs (rename/delete).</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr">
+      <c r="H186" s="6" t="inlineStr">
         <is>
           <t>Assistant-surface sync wiring (v2-native, additive); question-rail rename + delete(+undo) wired to the shipped PUT/DELETE endpoints; CLA sync tier plans recorded.</t>
         </is>
       </c>
-      <c r="I186" t="inlineStr">
+      <c r="I186" s="6" t="inlineStr">
         <is>
           <t>dc6-p3b (PR #232), dc6-p3c (PR #245); plan docs DC6-* under syllabai-v2 docs/.</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr">
+      <c r="J186" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K186" t="inlineStr">
+      <c r="K186" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="L186" t="inlineStr">
+      <c r="L186" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="M186" t="inlineStr">
+      <c r="M186" s="6" t="inlineStr">
         <is>
           <t>Wave 3 - Tutor &amp; Diagnostic Intelligence</t>
         </is>
       </c>
-      <c r="N186" t="inlineStr">
+      <c r="N186" s="6" t="inlineStr">
         <is>
           <t>Cycle 1</t>
         </is>
       </c>
-      <c r="O186" t="inlineStr">
+      <c r="O186" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P186" t="inlineStr">
+      <c r="P186" s="6" t="inlineStr">
         <is>
           <t>syllabai-v2</t>
         </is>
       </c>
-      <c r="Q186" t="inlineStr">
+      <c r="Q186" s="6" t="inlineStr">
         <is>
           <t>Master Spec Addendum 1.5 (Contextual Learning Assistant)</t>
         </is>
       </c>
-      <c r="R186" t="inlineStr">
+      <c r="R186" s="6" t="inlineStr">
         <is>
           <t>PR CI green; verbs wired to PUT/DELETE of record</t>
         </is>
       </c>
-      <c r="S186" t="inlineStr">
+      <c r="S186" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="T186" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U186" t="inlineStr">
+      <c r="T186" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U186" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="V186" t="inlineStr">
+      <c r="V186" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W186" t="inlineStr">
+      <c r="W186" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="X186" t="inlineStr"/>
-      <c r="Y186" t="inlineStr">
+      <c r="X186" s="6" t="inlineStr"/>
+      <c r="Y186" s="6" t="inlineStr">
         <is>
           <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record.</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="inlineStr">
+      <c r="A187" s="6" t="inlineStr">
         <is>
           <t>F-181</t>
         </is>
       </c>
-      <c r="B187" t="inlineStr">
+      <c r="B187" s="6" t="inlineStr">
         <is>
           <t>Core Platform &amp; Infrastructure</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr">
+      <c r="C187" s="6" t="inlineStr">
         <is>
           <t>v2 platform migration + cutover (T-MIG band)</t>
         </is>
       </c>
-      <c r="D187" t="inlineStr">
+      <c r="D187" s="6" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="E187" t="inlineStr">
+      <c r="E187" s="6" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr">
+      <c r="F187" s="6" t="inlineStr">
         <is>
           <t>Backend + Migration</t>
         </is>
       </c>
-      <c r="G187" t="inlineStr">
+      <c r="G187" s="6" t="inlineStr">
         <is>
           <t>The Java core on the Render free tier plus a separate hub repo meant cold starts, two deployment planes and pre-cutover dual system-of-record risk.</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr">
+      <c r="H187" s="6" t="inlineStr">
         <is>
           <t>TS monorepo re-platform (apps/api Hono+Drizzle+Neon serverless, apps/hub) behind golden-master parity gates; 100% migrated with the zero-core census LIVE=0 gate CI-enforced; cutover 2026-10-13 - syllabai-v2 sole system of record; syllabai-core/syllabai-hub archived read-only; Render retired.</t>
         </is>
       </c>
-      <c r="I187" t="inlineStr">
+      <c r="I187" s="6" t="inlineStr">
         <is>
           <t>MIGRATION_PLAN waves + W7-CUTOVER receipts; census gate scripts/preflight_zero_core_census.py --gate in ci.yml (commit 32272d2); CUTOVER_RETIREMENT_2026-10-13.md of record; ADR-MIG-0001/0002.</t>
         </is>
       </c>
-      <c r="J187" t="inlineStr">
+      <c r="J187" s="6" t="inlineStr">
         <is>
           <t>Neon Postgres; Vercel.</t>
         </is>
       </c>
-      <c r="K187" t="inlineStr">
+      <c r="K187" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="L187" t="inlineStr">
+      <c r="L187" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="M187" t="inlineStr">
+      <c r="M187" s="6" t="inlineStr">
         <is>
           <t>Wave 0 - Foundations</t>
         </is>
       </c>
-      <c r="N187" t="inlineStr">
+      <c r="N187" s="6" t="inlineStr">
         <is>
           <t>Cycle 2+</t>
         </is>
       </c>
-      <c r="O187" t="inlineStr">
+      <c r="O187" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="P187" t="inlineStr">
+      <c r="P187" s="6" t="inlineStr">
         <is>
           <t>syllabai-v2</t>
         </is>
       </c>
-      <c r="Q187" t="inlineStr">
+      <c r="Q187" s="6" t="inlineStr">
         <is>
           <t>docs/MIGRATION_REPORT.md 7/8</t>
         </is>
       </c>
-      <c r="R187" t="inlineStr">
+      <c r="R187" s="6" t="inlineStr">
         <is>
           <t>Zero-core census LIVE=0 (pins=7, rides-v2=2, rollback-fallback=1, dormant=5, unmapped/stale/unknown=0); bake battery 9/9 GREEN on the production alias</t>
         </is>
       </c>
-      <c r="S187" t="inlineStr">
+      <c r="S187" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="T187" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U187" t="inlineStr">
+      <c r="T187" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U187" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="V187" t="inlineStr">
+      <c r="V187" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W187" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="X187" t="inlineStr"/>
-      <c r="Y187" t="inlineStr">
+      <c r="W187" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X187" s="6" t="inlineStr"/>
+      <c r="Y187" s="6" t="inlineStr">
         <is>
           <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record.; historical syllabai-core mappings on pre-existing rows corrected in this pass.</t>
         </is>

</xml_diff>

<commit_message>
tracker(ADR-037): 2C spec-label wave ledger sync (F-178 leg note + F-182 gate cleared) + F-187 exporter hardening row (trace 1a16017ebd6ad2b5)
- F-178 Agent Notes: 2C spec-label leg LANDED — resources v0.9.0 (commit 89260832) -> syllabai-v2 PR #268 (merged 2026-10-21T19:02Z); 2C 607/607 resolved: 584 spec-tagged + 23 terminal no-spec-point; independent post-merge review census attached (0 structure/marks/exam-wording changes, SME 28/28 byte-preserved)
- F-182 Agent Notes: drill gate CLEARED — drill-eligible population now 927 (1C) + 584 (2C) spec-anchored parts; 26 terminal no-spec parts stay unmapped per anchor law
- New row F-187: exporter of record hardening G-E1..E4 (residue of closed resources PR #27, superseded by provenance exporter #31) — W2/C2+, P2, repo syllabai-resources
- TSV +5 lines net (+1 row, 2 note appends); XLSX openpyxl re-save, autofilter A1:Y192 -> A1:Y193
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Backlog" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Backlog'!$A$1:$Y$192</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Backlog'!$A$1:$Y$193</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y192"/>
+  <dimension ref="A1:Y193"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="6" min="1" max="1"/>
@@ -21324,7 +21324,7 @@
       <c r="X184" s="6" t="inlineStr"/>
       <c r="Y184" s="6" t="inlineStr">
         <is>
-          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. (PRs #239 #249); the master-pack ADR-037 GO-gated items (tracker claim + 2C-4C scheduling) remain operator-adjudicated.| GO RULING v2 (2026-10-21, operator trace 1a15ebd93809a525): GO granted - the executed 1C wiring (PRs #239 #249) is ratified post-hoc (process exception, not precedent); tracker-claim gate CLEARED; scheduling GRANTED for the remaining 4CH1 variants 2C x16 + 1CR x11 + 2CR x11 = 38 papers (registry-corrected from the ADR prose label "2C-4C"; same pipeline unchanged, UNVERIFIED list = scheduled gates); new courses DEFERRED (ADR-019 Cycle-1 scope / spec 39a).| 2C TRANCHE DONE (2026-10-21, trace 1a15ee5761b7a4a5): 16/16 4CH1/2C slices converted end-to-end, all gates PASS, 1120/1120 marks, 27/27 MCQs keyed (converter v0.8.0 = F34 paper parametrization + F35 MS question-marker discipline + F36 sentence-form positives; syllabai-resources PR #25, merge 1a5a8e6). Remaining GO-approved schedule: 1CR x11 + 2CR x11. 2C follow-ups (spec-label waves, crop-review eyeballs, parsed-layer cross-diff) recorded in Official-ExamQuestion/AGENTS.md known-open-work.</t>
+          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. (PRs #239 #249); the master-pack ADR-037 GO-gated items (tracker claim + 2C-4C scheduling) remain operator-adjudicated.| GO RULING v2 (2026-10-21, operator trace 1a15ebd93809a525): GO granted - the executed 1C wiring (PRs #239 #249) is ratified post-hoc (process exception, not precedent); tracker-claim gate CLEARED; scheduling GRANTED for the remaining 4CH1 variants 2C x16 + 1CR x11 + 2CR x11 = 38 papers (registry-corrected from the ADR prose label "2C-4C"; same pipeline unchanged, UNVERIFIED list = scheduled gates); new courses DEFERRED (ADR-019 Cycle-1 scope / spec 39a).| 2C TRANCHE DONE (2026-10-21, trace 1a15ee5761b7a4a5): 16/16 4CH1/2C slices converted end-to-end, all gates PASS, 1120/1120 marks, 27/27 MCQs keyed (converter v0.8.0 = F34 paper parametrization + F35 MS question-marker discipline + F36 sentence-form positives; syllabai-resources PR #25, merge 1a5a8e6). Remaining GO-approved schedule: 1CR x11 + 2CR x11. 2C follow-ups (spec-label waves, crop-review eyeballs, parsed-layer cross-diff) recorded in Official-ExamQuestion/AGENTS.md known-open-work. | UPDATE 2026-10-22 (trace 1a16017ebd6ad2b5): 2C spec-label leg LANDED — resources v0.9.0 (commit 89260832) re-exported all 32 official sets; syllabai-v2 PR #268 merged 2026-10-21T19:02Z. 2C 607/607 parts resolved: 584 spec-tagged (registry-validated, 0 invalid codes) + 23 terminal no-spec-point honestly unmapped. Independent post-merge review: change census 584 labels + 8 solutionMd + 8 markPoints + 7 answerStatus (1C unmatched→linked) + F40 crop re-binds + 16 stub-banner rewordings; 0 structure/marks/exam-wording changes; SME 28/28 byte-preserved; official-set topicId re-key contained (0 external refs in bundle).</t>
         </is>
       </c>
     </row>
@@ -21698,622 +21698,745 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr">
+      <c r="A188" s="6" t="inlineStr">
         <is>
           <t>F-182</t>
         </is>
       </c>
-      <c r="B188" t="inlineStr">
+      <c r="B188" s="6" t="inlineStr">
         <is>
           <t>Assessment &amp; Practice Tools</t>
         </is>
       </c>
-      <c r="C188" t="inlineStr">
+      <c r="C188" s="6" t="inlineStr">
         <is>
           <t>Per-spec-point drill surface (strength-test analog)</t>
         </is>
       </c>
-      <c r="D188" t="inlineStr">
+      <c r="D188" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr">
+      <c r="E188" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr">
+      <c r="F188" s="6" t="inlineStr">
         <is>
           <t>Full Stack</t>
         </is>
       </c>
-      <c r="G188" t="inlineStr">
+      <c r="G188" s="6" t="inlineStr">
         <is>
           <t>Kognity's most-praised feature (verified review corpus) is a 5-question random per-section drill with instant solutions and a persistent strength bar; SyllabAI has no equivalent self-directed, zero-stakes diagnostic keyed to the syllabus address space.</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr">
+      <c r="H188" s="6" t="inlineStr">
         <is>
           <t>5-part randomized drill keyed to spec points, drawn from the canonical corpus (1C+2C) and SME bank; zero stakes, always available, retakable with a fresh draw; ships only where spec-tagging exists (anchor law: unmapped content stays out).</t>
         </is>
       </c>
-      <c r="I188" t="inlineStr">
+      <c r="I188" s="6" t="inlineStr">
         <is>
           <t>Draw excludes recently seen items (naive dedupe); instant solution reveal; emits attempt evidence in the F-055 contract; MCQ and structured parts both allowed (structured parts route through Smart Mark).</t>
         </is>
       </c>
-      <c r="J188" t="inlineStr">
+      <c r="J188" s="6" t="inlineStr">
         <is>
           <t>Spec-point coverage census; fresh-draw guarantee; instant reveal; evidence emission; zero-stakes (no gradebook event).</t>
         </is>
       </c>
-      <c r="K188" t="inlineStr">
+      <c r="K188" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="L188" t="inlineStr">
+      <c r="L188" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="M188" t="inlineStr">
+      <c r="M188" s="6" t="inlineStr">
         <is>
           <t>Wave 2 - Learner &amp; Assessment</t>
         </is>
       </c>
-      <c r="N188" t="inlineStr">
+      <c r="N188" s="6" t="inlineStr">
         <is>
           <t>Cycle 1</t>
         </is>
       </c>
-      <c r="O188" t="inlineStr">
+      <c r="O188" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P188" t="inlineStr">
+      <c r="P188" s="6" t="inlineStr">
         <is>
           <t>syllabai-v2</t>
         </is>
       </c>
-      <c r="Q188" t="inlineStr">
+      <c r="Q188" s="6" t="inlineStr">
         <is>
           <t>Kognity competitive dossier v1.1, Deep Dive D (docs/research/KOGNITY_COMPETITIVE_RESEARCH_DOSSIER_2026-10-20.md)</t>
         </is>
       </c>
-      <c r="R188" t="inlineStr">
+      <c r="R188" s="6" t="inlineStr">
         <is>
           <t>Drill starts/completions per active learner; % spec points drill-covered</t>
         </is>
       </c>
-      <c r="S188" t="inlineStr">
+      <c r="S188" s="6" t="inlineStr">
         <is>
           <t>F-028; F-049; F-178</t>
         </is>
       </c>
-      <c r="T188" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U188" t="inlineStr">
+      <c r="T188" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U188" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V188" t="inlineStr">
+      <c r="V188" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W188" t="inlineStr">
+      <c r="W188" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="X188" t="inlineStr"/>
-      <c r="Y188" t="inlineStr">
-        <is>
-          <t>Added 2026-10-22 from the Kognity Strength Test deep dive (dossier v1.1, trace 1a15fe54423bf93d). Gated by the 2C spec-tagging wave inside F-178 scope (607 pending-llm parts).</t>
+      <c r="X188" s="6" t="inlineStr"/>
+      <c r="Y188" s="6" t="inlineStr">
+        <is>
+          <t>Added 2026-10-22 from the Kognity Strength Test deep dive (dossier v1.1, trace 1a15fe54423bf93d). Gated by the 2C spec-tagging wave inside F-178 scope (607 pending-llm parts). | UPDATE 2026-10-22 (trace 1a16017ebd6ad2b5): gate CLEARED — 2C spec-tagging wave completed via resources v0.9.0 + syllabai-v2 #268 (584/607 parts spec-tagged; 23 terminal no-spec-point excluded per anchor law). Drill-eligible population now 927 (1C) + 584 (2C) spec-anchored parts; 26 terminal no-spec parts stay unmapped.</t>
         </is>
       </c>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr">
+      <c r="A189" s="6" t="inlineStr">
         <is>
           <t>F-183</t>
         </is>
       </c>
-      <c r="B189" t="inlineStr">
+      <c r="B189" s="6" t="inlineStr">
         <is>
           <t>Assessment &amp; Practice Tools</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr">
+      <c r="C189" s="6" t="inlineStr">
         <is>
           <t>Instant MS-reveal law in drill mode (real mark schemes, method credit)</t>
         </is>
       </c>
-      <c r="D189" t="inlineStr">
+      <c r="D189" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="E189" t="inlineStr">
+      <c r="E189" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr">
+      <c r="F189" s="6" t="inlineStr">
         <is>
           <t>Backend + Integration</t>
         </is>
       </c>
-      <c r="G189" t="inlineStr">
+      <c r="G189" s="6" t="inlineStr">
         <is>
           <t>Kognity's documented weakness: shallow explanations on wrong answers and exact-answer marking without method credit (the two loudest verified complaints). A drill whose reveal paraphrases instead of showing the real mark scheme repeats the weakness.</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr">
+      <c r="H189" s="6" t="inlineStr">
         <is>
           <t>In drill mode only, the solution reveal renders the actual MS from the corpus of record (M1..Mn points) with Smart Mark method-credit verdicts on structured parts; instant and never teacher-gated; everywhere else reveal gating stays as-is (practice/assessment boundary preserved).</t>
         </is>
       </c>
-      <c r="I189" t="inlineStr">
+      <c r="I189" s="6" t="inlineStr">
         <is>
           <t>MS rendering from the corpus of record; Smart Mark wiring for structured drill parts; gating law: instant in drill, gated elsewhere; no leakage of gated MS into other surfaces.</t>
         </is>
       </c>
-      <c r="J189" t="inlineStr">
+      <c r="J189" s="6" t="inlineStr">
         <is>
           <t>MS-from-corpus rendering; Smart Mark wiring; gating law; method-credit verdicts on structured parts.</t>
         </is>
       </c>
-      <c r="K189" t="inlineStr">
+      <c r="K189" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="L189" t="inlineStr">
+      <c r="L189" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="M189" t="inlineStr">
+      <c r="M189" s="6" t="inlineStr">
         <is>
           <t>Wave 2 - Learner &amp; Assessment</t>
         </is>
       </c>
-      <c r="N189" t="inlineStr">
+      <c r="N189" s="6" t="inlineStr">
         <is>
           <t>Cycle 1</t>
         </is>
       </c>
-      <c r="O189" t="inlineStr">
+      <c r="O189" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P189" t="inlineStr">
+      <c r="P189" s="6" t="inlineStr">
         <is>
           <t>syllabai-v2</t>
         </is>
       </c>
-      <c r="Q189" t="inlineStr">
+      <c r="Q189" s="6" t="inlineStr">
         <is>
           <t>Kognity dossier v1.1 Deep Dive D 8.4-8.5; ADR-025 Smart Mark product contract</t>
         </is>
       </c>
-      <c r="R189" t="inlineStr">
+      <c r="R189" s="6" t="inlineStr">
         <is>
           <t>% drill reveals showing full M-point MS; method-credit agreement on structured drill parts</t>
         </is>
       </c>
-      <c r="S189" t="inlineStr">
+      <c r="S189" s="6" t="inlineStr">
         <is>
           <t>F-182; F-047; F-144</t>
         </is>
       </c>
-      <c r="T189" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U189" t="inlineStr">
+      <c r="T189" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U189" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V189" t="inlineStr">
+      <c r="V189" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W189" t="inlineStr">
+      <c r="W189" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="X189" t="inlineStr"/>
-      <c r="Y189" t="inlineStr">
+      <c r="X189" s="6" t="inlineStr"/>
+      <c r="Y189" s="6" t="inlineStr">
         <is>
           <t>Added 2026-10-22 from the Kognity Strength Test deep dive (dossier v1.1, trace 1a15fe54423bf93d). Positioning line: the solutions are the examiner's.</t>
         </is>
       </c>
     </row>
     <row r="190">
-      <c r="A190" t="inlineStr">
+      <c r="A190" s="6" t="inlineStr">
         <is>
           <t>F-184</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr">
+      <c r="B190" s="6" t="inlineStr">
         <is>
           <t>Assessment &amp; Practice Tools</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr">
+      <c r="C190" s="6" t="inlineStr">
         <is>
           <t>Decay-driven strength surface (mastery bar with computed decay)</t>
         </is>
       </c>
-      <c r="D190" t="inlineStr">
+      <c r="D190" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="E190" t="inlineStr">
+      <c r="E190" s="6" t="inlineStr">
         <is>
           <t>Learner/Research</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr">
+      <c r="F190" s="6" t="inlineStr">
         <is>
           <t>Full Stack</t>
         </is>
       </c>
-      <c r="G190" t="inlineStr">
+      <c r="G190" s="6" t="inlineStr">
         <is>
           <t>Kognity's strength bar is engagement-coupled (rises with usage) - effort visibility, not mastery. A monotonic bar cannot signal retention loss, which is the actual enemy between lessons and before exams.</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr">
+      <c r="H190" s="6" t="inlineStr">
         <is>
           <t>Per-spec-point strength display driven by learner state + computed decay (ADR-031: decay computed, never persisted); the bar honestly falls as skills decay and doubles as the practice-now queue at decaying addresses.</t>
         </is>
       </c>
-      <c r="I190" t="inlineStr">
+      <c r="I190" s="6" t="inlineStr">
         <is>
           <t>Bar semantics = mastery x decay, documented explicitly; not-a-grade framing; feeds the practice-now queue; surfaced on the learner overview (the strength-bar position Kognity validated).</t>
         </is>
       </c>
-      <c r="J190" t="inlineStr">
+      <c r="J190" s="6" t="inlineStr">
         <is>
           <t>ADR-031 decay engine; spec-point learner overlay; explicit bar-semantics documentation; no engagement-only component.</t>
         </is>
       </c>
-      <c r="K190" t="inlineStr">
+      <c r="K190" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="L190" t="inlineStr">
+      <c r="L190" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="M190" t="inlineStr">
+      <c r="M190" s="6" t="inlineStr">
         <is>
           <t>Wave 3 - Tutor &amp; Diagnostic Intelligence</t>
         </is>
       </c>
-      <c r="N190" t="inlineStr">
+      <c r="N190" s="6" t="inlineStr">
         <is>
           <t>Cycle 2+</t>
         </is>
       </c>
-      <c r="O190" t="inlineStr">
+      <c r="O190" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="P190" t="inlineStr">
+      <c r="P190" s="6" t="inlineStr">
         <is>
           <t>syllabai-v2</t>
         </is>
       </c>
-      <c r="Q190" t="inlineStr">
+      <c r="Q190" s="6" t="inlineStr">
         <is>
           <t>Kognity dossier v1.1 Deep Dive D 8.3 (law 3) + 8.5; ADR-031</t>
         </is>
       </c>
-      <c r="R190" t="inlineStr">
+      <c r="R190" s="6" t="inlineStr">
         <is>
           <t>Decay-driven bar vs later performance correlation; return-rate after decay nudges</t>
         </is>
       </c>
-      <c r="S190" t="inlineStr">
+      <c r="S190" s="6" t="inlineStr">
         <is>
           <t>F-137; F-159; F-169; F-033</t>
         </is>
       </c>
-      <c r="T190" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U190" t="inlineStr">
+      <c r="T190" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U190" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V190" t="inlineStr">
+      <c r="V190" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W190" t="inlineStr">
+      <c r="W190" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="X190" t="inlineStr"/>
-      <c r="Y190" t="inlineStr">
+      <c r="X190" s="6" t="inlineStr"/>
+      <c r="Y190" s="6" t="inlineStr">
         <is>
           <t>Added 2026-10-22 from the Kognity Strength Test deep dive (dossier v1.1, trace 1a15fe54423bf93d). Replaces engagement-coupled bar semantics with calibrated mastery x decay.</t>
         </is>
       </c>
     </row>
     <row r="191">
-      <c r="A191" t="inlineStr">
+      <c r="A191" s="6" t="inlineStr">
         <is>
           <t>F-185</t>
         </is>
       </c>
-      <c r="B191" t="inlineStr">
+      <c r="B191" s="6" t="inlineStr">
         <is>
           <t>Assessment &amp; Practice Tools</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr">
+      <c r="C191" s="6" t="inlineStr">
         <is>
           <t>Model-driven drill draw (BKT/decay-informed question selection)</t>
         </is>
       </c>
-      <c r="D191" t="inlineStr">
+      <c r="D191" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr">
+      <c r="E191" s="6" t="inlineStr">
         <is>
           <t>Learner/Research</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr">
+      <c r="F191" s="6" t="inlineStr">
         <is>
           <t>Backend + Research</t>
         </is>
       </c>
-      <c r="G191" t="inlineStr">
+      <c r="G191" s="6" t="inlineStr">
         <is>
           <t>Kognity's random draw samples the bank by chance; retakes re-roll dice instead of targeting gaps. There is no model selecting the next 5 questions - the adaptivity vacuum at the smallest possible surface.</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr">
+      <c r="H191" s="6" t="inlineStr">
         <is>
           <t>Replace the naive random draw with information-maximizing selection over learner state: pick the 5 parts that maximize evidence on the weakest, most-decayed skills at the address (BKT engine + decay); fallback to random when the state is sparse.</t>
         </is>
       </c>
-      <c r="I191" t="inlineStr">
+      <c r="I191" s="6" t="inlineStr">
         <is>
           <t>BKT posterior read; selection policy with an exploration floor; sparse-state fallback to random; latency budget on the draw; no gaming feedback loop (selection must not be predictable).</t>
         </is>
       </c>
-      <c r="J191" t="inlineStr">
+      <c r="J191" s="6" t="inlineStr">
         <is>
           <t>BKT posterior read; selection policy; sparse fallback; latency budget; anti-gaming.</t>
         </is>
       </c>
-      <c r="K191" t="inlineStr">
+      <c r="K191" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="L191" t="inlineStr">
+      <c r="L191" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="M191" t="inlineStr">
+      <c r="M191" s="6" t="inlineStr">
         <is>
           <t>Wave 3 - Tutor &amp; Diagnostic Intelligence</t>
         </is>
       </c>
-      <c r="N191" t="inlineStr">
+      <c r="N191" s="6" t="inlineStr">
         <is>
           <t>Cycle 2+</t>
         </is>
       </c>
-      <c r="O191" t="inlineStr">
+      <c r="O191" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="P191" t="inlineStr">
+      <c r="P191" s="6" t="inlineStr">
         <is>
           <t>syllabai-v2</t>
         </is>
       </c>
-      <c r="Q191" t="inlineStr">
+      <c r="Q191" s="6" t="inlineStr">
         <is>
           <t>Kognity dossier v1.1 Deep Dive D 8.5; ADR-033 (BKT emission is format-aware); ADR-031</t>
         </is>
       </c>
-      <c r="R191" t="inlineStr">
+      <c r="R191" s="6" t="inlineStr">
         <is>
           <t>Post-draw mastery gain vs random draw (A/B); draw latency; evidence value per attempt</t>
         </is>
       </c>
-      <c r="S191" t="inlineStr">
+      <c r="S191" s="6" t="inlineStr">
         <is>
           <t>F-182; F-184; F-138; F-139; F-055</t>
         </is>
       </c>
-      <c r="T191" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U191" t="inlineStr">
+      <c r="T191" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U191" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V191" t="inlineStr">
+      <c r="V191" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W191" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="X191" t="inlineStr"/>
-      <c r="Y191" t="inlineStr">
+      <c r="W191" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X191" s="6" t="inlineStr"/>
+      <c r="Y191" s="6" t="inlineStr">
         <is>
           <t>Added 2026-10-22 from the Kognity Strength Test deep dive (dossier v1.1, trace 1a15fe54423bf93d). The category-making substitution per Deep Dive D; research-gated.</t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="A192" t="inlineStr">
+      <c r="A192" s="6" t="inlineStr">
         <is>
           <t>F-186</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr">
+      <c r="B192" s="6" t="inlineStr">
         <is>
           <t>Assessment &amp; Practice Tools</t>
         </is>
       </c>
-      <c r="C192" t="inlineStr">
+      <c r="C192" s="6" t="inlineStr">
         <is>
           <t>Strength Battle mode (3-question / 60-second head-to-head)</t>
         </is>
       </c>
-      <c r="D192" t="inlineStr">
+      <c r="D192" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr">
+      <c r="E192" s="6" t="inlineStr">
         <is>
           <t>Experience</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr">
+      <c r="F192" s="6" t="inlineStr">
         <is>
           <t>Full Stack</t>
         </is>
       </c>
-      <c r="G192" t="inlineStr">
+      <c r="G192" s="6" t="inlineStr">
         <is>
           <t>Kognity's 3-question/60-second head-to-head battle (vs classmate or bot) logged 5M+ battles (vendor claim) - competitive energy reuses the same question bank at near-zero content cost, and class brackets are a proven teacher-community mechanic.</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr">
+      <c r="H192" s="6" t="inlineStr">
         <is>
           <t>Same drill bank, 3-question / 60-second synchronous head-to-head vs classmate or a bot opponent; class-bracket mode for teachers; strictly sequenced after the drill surface and model-driven draw so battles inherit model-drawn sets.</t>
         </is>
       </c>
-      <c r="I192" t="inlineStr">
+      <c r="I192" s="6" t="inlineStr">
         <is>
           <t>Matchmaking or async ghost opponent; bot opponent; fairness policy (same address, same format); opt-in; leaderboard posture must respect the k-anonymity research rule (ADR-036).</t>
         </is>
       </c>
-      <c r="J192" t="inlineStr">
+      <c r="J192" s="6" t="inlineStr">
         <is>
           <t>Matchmaking/ghost; bot opponent; fairness policy; opt-in + ADR-036-adjacent leaderboard privacy.</t>
         </is>
       </c>
-      <c r="K192" t="inlineStr">
+      <c r="K192" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="L192" t="inlineStr">
+      <c r="L192" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="M192" t="inlineStr">
+      <c r="M192" s="6" t="inlineStr">
         <is>
           <t>Wave 2 - Learner &amp; Assessment</t>
         </is>
       </c>
-      <c r="N192" t="inlineStr">
+      <c r="N192" s="6" t="inlineStr">
         <is>
           <t>Cycle 2+</t>
         </is>
       </c>
-      <c r="O192" t="inlineStr">
+      <c r="O192" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P192" t="inlineStr">
+      <c r="P192" s="6" t="inlineStr">
         <is>
           <t>syllabai-v2</t>
         </is>
       </c>
-      <c r="Q192" t="inlineStr">
+      <c r="Q192" s="6" t="inlineStr">
         <is>
           <t>Kognity dossier v1.1 Deep Dive D 8.1 (Battle row) + 8.5</t>
         </is>
       </c>
-      <c r="R192" t="inlineStr">
+      <c r="R192" s="6" t="inlineStr">
         <is>
           <t>Battles per active learner; opt-in rate; bracket adoption by teachers</t>
         </is>
       </c>
-      <c r="S192" t="inlineStr">
+      <c r="S192" s="6" t="inlineStr">
         <is>
           <t>F-182; F-185</t>
         </is>
       </c>
-      <c r="T192" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U192" t="inlineStr">
+      <c r="T192" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U192" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V192" t="inlineStr">
+      <c r="V192" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W192" t="inlineStr">
+      <c r="W192" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="X192" t="inlineStr"/>
-      <c r="Y192" t="inlineStr">
+      <c r="X192" s="6" t="inlineStr"/>
+      <c r="Y192" s="6" t="inlineStr">
         <is>
           <t>Added 2026-10-22 from the Kognity Strength Test deep dive (dossier v1.1, trace 1a15fe54423bf93d). Explicitly a later wave; the 5M-battle engagement figure is vendor-claimed (single-source).</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>F-187</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Assessment &amp; Practice Tools</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Exporter of record hardening — G-E1..G-E4 fail-closed gates (residue of closed resources PR #27)</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Data + Tooling</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>The ADR-037 exporter of record (resources PR #31) runs gate-free: a silent regression in a re-export could corrupt a hub-bundle sync before any human notices. Closed PR #27 carried the hardened variant with fail-closed gates (G-E1 bundle-of-record diff classes; G-E2 per-question Σparts.marks = totalMarks + markPoints closure; G-E3 per-series census constants; G-E4 SME-prefix byte-identity) but was closed as superseded to keep the provenance exporter; its gates were recorded for a future hardening wave.</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Port G-E1..G-E4 onto the #31 exporter as a verification harness (wrapper or CI job): an export may only ship if it matches the bundle of record or differs solely in disclosed diff classes; mark law holds per question; per-series census equals frozen constants; the SME prefix re-serializes byte-identical. Seed-fault negative tests prove the gates refuse.</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>ADR-037; provenance exporter syllabai-resources/scripts/official_examq_export_hub.py@main; hardened reference implementation existed session-locally (19,229 B; output hash-proven == served bundle during the #263 review).</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>syllabai-resources exporter; bundle of record in syllabai-v2 hub content; frozen per-series census constants.</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>Wave 2 - Learner &amp; Assessment</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>Cycle 2+</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>syllabai-resources</t>
+        </is>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>ADR-037</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>4/4 gates pass on the of-record corpus and refuse on seeded faults; exporter CI green on resources main.</t>
+        </is>
+      </c>
+      <c r="S193" t="inlineStr">
+        <is>
+          <t>F-178</t>
+        </is>
+      </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="V193" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="W193" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X193" t="inlineStr"/>
+      <c r="Y193" t="inlineStr">
+        <is>
+          <t>Added 2026-10-22 (trace 1a16017ebd6ad2b5) from the operator-ordered "proceed" on resources PR #27 — the supersession (provenance exporter via #31, #27 closed 2026-10-21T19:20Z) is already executed; the actionable residue is this hardening wave. Provenance law: the #31 exporter is the of record; G-E1..G-E4 are additive verification only.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y192"/>
+  <autoFilter ref="A1:Y193"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
tracker(ADR-037): R-variant schedule footer-verified (1CR x11 + 2CR x11) + F-187 build-open note (trace 1a1604c4c6b5c9a5)
- F-178 Agent Notes: R-VARIANT SCHEDULE appended — the GO'd remaining variants (1CR x11 + 2CR x11 = 22 papers)
  are footer-verified from the archive of record, 22/22 OK (1CR @ 110 marks, Q counts 10-12; 2CR @ 70 marks,
  Q counts 7-8; contiguous numbering + manifest paper_number_variant matches --paper 22/22). Run protocol,
  registry-entry plan, and gate routing recorded in the note; legacy 4CH0 R papers explicitly out of scope.
- F-187 Agent Notes: build OPEN as resources PR #34 (G-E1..G-E4 harness, 4/4 seeds refused, CI green;
  the F39 topicSlug drift it caught on first run fixed one-liner).
- TSV +2 note appends only (192 data rows x 25 cols); XLSX openpyxl cell edits, autofilter A1:Y193 unchanged.
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -21324,7 +21324,7 @@
       <c r="X184" s="6" t="inlineStr"/>
       <c r="Y184" s="6" t="inlineStr">
         <is>
-          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. (PRs #239 #249); the master-pack ADR-037 GO-gated items (tracker claim + 2C-4C scheduling) remain operator-adjudicated.| GO RULING v2 (2026-10-21, operator trace 1a15ebd93809a525): GO granted - the executed 1C wiring (PRs #239 #249) is ratified post-hoc (process exception, not precedent); tracker-claim gate CLEARED; scheduling GRANTED for the remaining 4CH1 variants 2C x16 + 1CR x11 + 2CR x11 = 38 papers (registry-corrected from the ADR prose label "2C-4C"; same pipeline unchanged, UNVERIFIED list = scheduled gates); new courses DEFERRED (ADR-019 Cycle-1 scope / spec 39a).| 2C TRANCHE DONE (2026-10-21, trace 1a15ee5761b7a4a5): 16/16 4CH1/2C slices converted end-to-end, all gates PASS, 1120/1120 marks, 27/27 MCQs keyed (converter v0.8.0 = F34 paper parametrization + F35 MS question-marker discipline + F36 sentence-form positives; syllabai-resources PR #25, merge 1a5a8e6). Remaining GO-approved schedule: 1CR x11 + 2CR x11. 2C follow-ups (spec-label waves, crop-review eyeballs, parsed-layer cross-diff) recorded in Official-ExamQuestion/AGENTS.md known-open-work. | UPDATE 2026-10-22 (trace 1a16017ebd6ad2b5): 2C spec-label leg LANDED — resources v0.9.0 (commit 89260832) re-exported all 32 official sets; syllabai-v2 PR #268 merged 2026-10-21T19:02Z. 2C 607/607 parts resolved: 584 spec-tagged (registry-validated, 0 invalid codes) + 23 terminal no-spec-point honestly unmapped. Independent post-merge review: change census 584 labels + 8 solutionMd + 8 markPoints + 7 answerStatus (1C unmatched→linked) + F40 crop re-binds + 16 stub-banner rewordings; 0 structure/marks/exam-wording changes; SME 28/28 byte-preserved; official-set topicId re-key contained (0 external refs in bundle).</t>
+          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. (PRs #239 #249); the master-pack ADR-037 GO-gated items (tracker claim + 2C-4C scheduling) remain operator-adjudicated.| GO RULING v2 (2026-10-21, operator trace 1a15ebd93809a525): GO granted - the executed 1C wiring (PRs #239 #249) is ratified post-hoc (process exception, not precedent); tracker-claim gate CLEARED; scheduling GRANTED for the remaining 4CH1 variants 2C x16 + 1CR x11 + 2CR x11 = 38 papers (registry-corrected from the ADR prose label "2C-4C"; same pipeline unchanged, UNVERIFIED list = scheduled gates); new courses DEFERRED (ADR-019 Cycle-1 scope / spec 39a).| 2C TRANCHE DONE (2026-10-21, trace 1a15ee5761b7a4a5): 16/16 4CH1/2C slices converted end-to-end, all gates PASS, 1120/1120 marks, 27/27 MCQs keyed (converter v0.8.0 = F34 paper parametrization + F35 MS question-marker discipline + F36 sentence-form positives; syllabai-resources PR #25, merge 1a5a8e6). Remaining GO-approved schedule: 1CR x11 + 2CR x11. 2C follow-ups (spec-label waves, crop-review eyeballs, parsed-layer cross-diff) recorded in Official-ExamQuestion/AGENTS.md known-open-work. | UPDATE 2026-10-22 (trace 1a16017ebd6ad2b5): 2C spec-label leg LANDED — resources v0.9.0 (commit 89260832) re-exported all 32 official sets; syllabai-v2 PR #268 merged 2026-10-21T19:02Z. 2C 607/607 parts resolved: 584 spec-tagged (registry-validated, 0 invalid codes) + 23 terminal no-spec-point honestly unmapped. Independent post-merge review: change census 584 labels + 8 solutionMd + 8 markPoints + 7 answerStatus (1C unmatched→linked) + F40 crop re-binds + 16 stub-banner rewordings; 0 structure/marks/exam-wording changes; SME 28/28 byte-preserved; official-set topicId re-key contained (0 external refs in bundle). | R-VARIANT SCHEDULE (2026-10-22, trace 1a1604c4c6b5c9a5): GO'd 1CR x11 + 2CR x11 footer-verified from the archive of record — 22/22 OK (contiguous numbering 22/22; manifest paper_number_variant matches --paper 22/22; legacy 4CH0 R papers 2013-2017 in the archive are a DIFFERENT spec, out of scope). 1CR @ 110 marks, printed question counts: 2019-06:10, 2020-01:11, 2020-11:10, 2021-01:10, 2022-01:11, 2022-06:11, 2023-01:10, 2023-06:11, 2024-06:12, 2025-06:11, 2026-06:11. 2CR @ 70 marks: 2019-06:7, 2020-01:7, 2020-11:7, 2021-01:8, 2022-01:7, 2022-06:7, 2023-01:8, 2023-06:7, 2024-06:7, 2025-06:7, 2026-06:7. Run protocol (same kit, --paper 1CR/2CR): registry entries land in the run PR (PAPER_TOTALS 1CR=110/2CR=70 + EXPECT_QUESTIONS with these counts) per the outputs-and-pipeline commit law; per-paper G0-G7 + negative controls 3/3 per series; layout findings through the improvement loop (F-ledger + canaries); MCQ ambiguities -&gt; MCQ-KEYS.json human adjudication with rendered-page evidence; crop flags -&gt; CROP-REVIEW.json eyeball verdicts; per-paper spec-label waves after conversion (labels only, G6 judges) — anchor law: untagged parts stay unmapped/out of the learner model. Export via the #31 exporter + the F-187 harness (resources PR #34: --allow-new-official + EXPECTED_CENSUS extension in the same PR); then hub PR + live verification. Order: 1CR tranche first (110-mark format closest to the proven 1C pipeline), series ascending.</t>
         </is>
       </c>
     </row>
@@ -22313,125 +22313,125 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" t="inlineStr">
+      <c r="A193" s="6" t="inlineStr">
         <is>
           <t>F-187</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr">
+      <c r="B193" s="6" t="inlineStr">
         <is>
           <t>Assessment &amp; Practice Tools</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr">
+      <c r="C193" s="6" t="inlineStr">
         <is>
           <t>Exporter of record hardening — G-E1..G-E4 fail-closed gates (residue of closed resources PR #27)</t>
         </is>
       </c>
-      <c r="D193" t="inlineStr">
+      <c r="D193" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="E193" t="inlineStr">
+      <c r="E193" s="6" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr">
+      <c r="F193" s="6" t="inlineStr">
         <is>
           <t>Data + Tooling</t>
         </is>
       </c>
-      <c r="G193" t="inlineStr">
+      <c r="G193" s="6" t="inlineStr">
         <is>
           <t>The ADR-037 exporter of record (resources PR #31) runs gate-free: a silent regression in a re-export could corrupt a hub-bundle sync before any human notices. Closed PR #27 carried the hardened variant with fail-closed gates (G-E1 bundle-of-record diff classes; G-E2 per-question Σparts.marks = totalMarks + markPoints closure; G-E3 per-series census constants; G-E4 SME-prefix byte-identity) but was closed as superseded to keep the provenance exporter; its gates were recorded for a future hardening wave.</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr">
+      <c r="H193" s="6" t="inlineStr">
         <is>
           <t>Port G-E1..G-E4 onto the #31 exporter as a verification harness (wrapper or CI job): an export may only ship if it matches the bundle of record or differs solely in disclosed diff classes; mark law holds per question; per-series census equals frozen constants; the SME prefix re-serializes byte-identical. Seed-fault negative tests prove the gates refuse.</t>
         </is>
       </c>
-      <c r="I193" t="inlineStr">
+      <c r="I193" s="6" t="inlineStr">
         <is>
           <t>ADR-037; provenance exporter syllabai-resources/scripts/official_examq_export_hub.py@main; hardened reference implementation existed session-locally (19,229 B; output hash-proven == served bundle during the #263 review).</t>
         </is>
       </c>
-      <c r="J193" t="inlineStr">
+      <c r="J193" s="6" t="inlineStr">
         <is>
           <t>syllabai-resources exporter; bundle of record in syllabai-v2 hub content; frozen per-series census constants.</t>
         </is>
       </c>
-      <c r="K193" t="inlineStr">
+      <c r="K193" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="L193" t="inlineStr">
+      <c r="L193" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="M193" t="inlineStr">
+      <c r="M193" s="6" t="inlineStr">
         <is>
           <t>Wave 2 - Learner &amp; Assessment</t>
         </is>
       </c>
-      <c r="N193" t="inlineStr">
+      <c r="N193" s="6" t="inlineStr">
         <is>
           <t>Cycle 2+</t>
         </is>
       </c>
-      <c r="O193" t="inlineStr">
+      <c r="O193" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P193" t="inlineStr">
+      <c r="P193" s="6" t="inlineStr">
         <is>
           <t>syllabai-resources</t>
         </is>
       </c>
-      <c r="Q193" t="inlineStr">
+      <c r="Q193" s="6" t="inlineStr">
         <is>
           <t>ADR-037</t>
         </is>
       </c>
-      <c r="R193" t="inlineStr">
+      <c r="R193" s="6" t="inlineStr">
         <is>
           <t>4/4 gates pass on the of-record corpus and refuse on seeded faults; exporter CI green on resources main.</t>
         </is>
       </c>
-      <c r="S193" t="inlineStr">
+      <c r="S193" s="6" t="inlineStr">
         <is>
           <t>F-178</t>
         </is>
       </c>
-      <c r="T193" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U193" t="inlineStr">
+      <c r="T193" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U193" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="V193" t="inlineStr">
+      <c r="V193" s="6" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="W193" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="X193" t="inlineStr"/>
-      <c r="Y193" t="inlineStr">
-        <is>
-          <t>Added 2026-10-22 (trace 1a16017ebd6ad2b5) from the operator-ordered "proceed" on resources PR #27 — the supersession (provenance exporter via #31, #27 closed 2026-10-21T19:20Z) is already executed; the actionable residue is this hardening wave. Provenance law: the #31 exporter is the of record; G-E1..G-E4 are additive verification only.</t>
+      <c r="W193" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X193" s="6" t="inlineStr"/>
+      <c r="Y193" s="6" t="inlineStr">
+        <is>
+          <t>Added 2026-10-22 (trace 1a16017ebd6ad2b5) from the operator-ordered "proceed" on resources PR #27 — the supersession (provenance exporter via #31, #27 closed 2026-10-21T19:20Z) is already executed; the actionable residue is this hardening wave. Provenance law: the #31 exporter is the of record; G-E1..G-E4 are additive verification only. | UPDATE 2026-10-22 (trace 1a1604c4c6b5c9a5): build OPEN as resources PR #34 (branch f187/export-gates-r0) — G-E1..G-E4 artifact-level harness over the #31 exporter (additive only) + seed-fault self-test 4/4 refused on the of-record corpus + CI job official-export-gates green. G-E1's first run caught a real drift: the exporter regenerated topicSlug=official-past-papers (pre-F39) where the served bundle carries the per-set topic law; PR #34 fixes the exporter one-liner, after which it reproduces the bundle of record exactly (0 part deltas, SME prefix byte-identical 2,605,414 B).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker(ADR-037): F-187 merge receipt + 2C crop-review closure re-verified (trace 1a1608c3ae515a7d)
- F-187 Agent Notes: build MERGED as resources PR #34 (merge b5701769b9ca) — reconciled onto wave-14
  main (0ad59ca5935): the exporter of record untouched (F44/#41 supersede the branch one-liner); the
  G-E1..G-E4 harness + official-export-gates CI job now enforce the G-E law on every scripts/PR, with
  the new --disclosure census cross-check; 2019-06 damage repaired of record (EXPECTED_MARK_GAPS empty);
  census rebased to v0.10.0; self-test 4/4.
- F-178 Agent Notes: CROP-REVIEW CLOSURE RE-VERIFIED post wave-13/14 — 86 2C figure assets, 0
  review-flagged, CROP-REVIEW re-eyeballed 2026-10-22 (37 accepted + 4 stub-accepted, 24 homes);
  the 22x 2C crop-review queue item closed at ground truth.
- TSV +2 note appends only (192 data rows x 25 cols); XLSX openpyxl cell edits; legacy r2/r60/r93
  quote-wrappers asserted byte-unchanged; parity 0 mismatches.
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -21324,7 +21324,7 @@
       <c r="X184" s="6" t="inlineStr"/>
       <c r="Y184" s="6" t="inlineStr">
         <is>
-          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. (PRs #239 #249); the master-pack ADR-037 GO-gated items (tracker claim + 2C-4C scheduling) remain operator-adjudicated.| GO RULING v2 (2026-10-21, operator trace 1a15ebd93809a525): GO granted - the executed 1C wiring (PRs #239 #249) is ratified post-hoc (process exception, not precedent); tracker-claim gate CLEARED; scheduling GRANTED for the remaining 4CH1 variants 2C x16 + 1CR x11 + 2CR x11 = 38 papers (registry-corrected from the ADR prose label "2C-4C"; same pipeline unchanged, UNVERIFIED list = scheduled gates); new courses DEFERRED (ADR-019 Cycle-1 scope / spec 39a).| 2C TRANCHE DONE (2026-10-21, trace 1a15ee5761b7a4a5): 16/16 4CH1/2C slices converted end-to-end, all gates PASS, 1120/1120 marks, 27/27 MCQs keyed (converter v0.8.0 = F34 paper parametrization + F35 MS question-marker discipline + F36 sentence-form positives; syllabai-resources PR #25, merge 1a5a8e6). Remaining GO-approved schedule: 1CR x11 + 2CR x11. 2C follow-ups (spec-label waves, crop-review eyeballs, parsed-layer cross-diff) recorded in Official-ExamQuestion/AGENTS.md known-open-work. | UPDATE 2026-10-22 (trace 1a16017ebd6ad2b5): 2C spec-label leg LANDED — resources v0.9.0 (commit 89260832) re-exported all 32 official sets; syllabai-v2 PR #268 merged 2026-10-21T19:02Z. 2C 607/607 parts resolved: 584 spec-tagged (registry-validated, 0 invalid codes) + 23 terminal no-spec-point honestly unmapped. Independent post-merge review: change census 584 labels + 8 solutionMd + 8 markPoints + 7 answerStatus (1C unmatched→linked) + F40 crop re-binds + 16 stub-banner rewordings; 0 structure/marks/exam-wording changes; SME 28/28 byte-preserved; official-set topicId re-key contained (0 external refs in bundle). | R-VARIANT SCHEDULE (2026-10-22, trace 1a1604c4c6b5c9a5): GO'd 1CR x11 + 2CR x11 footer-verified from the archive of record — 22/22 OK (contiguous numbering 22/22; manifest paper_number_variant matches --paper 22/22; legacy 4CH0 R papers 2013-2017 in the archive are a DIFFERENT spec, out of scope). 1CR @ 110 marks, printed question counts: 2019-06:10, 2020-01:11, 2020-11:10, 2021-01:10, 2022-01:11, 2022-06:11, 2023-01:10, 2023-06:11, 2024-06:12, 2025-06:11, 2026-06:11. 2CR @ 70 marks: 2019-06:7, 2020-01:7, 2020-11:7, 2021-01:8, 2022-01:7, 2022-06:7, 2023-01:8, 2023-06:7, 2024-06:7, 2025-06:7, 2026-06:7. Run protocol (same kit, --paper 1CR/2CR): registry entries land in the run PR (PAPER_TOTALS 1CR=110/2CR=70 + EXPECT_QUESTIONS with these counts) per the outputs-and-pipeline commit law; per-paper G0-G7 + negative controls 3/3 per series; layout findings through the improvement loop (F-ledger + canaries); MCQ ambiguities -&gt; MCQ-KEYS.json human adjudication with rendered-page evidence; crop flags -&gt; CROP-REVIEW.json eyeball verdicts; per-paper spec-label waves after conversion (labels only, G6 judges) — anchor law: untagged parts stay unmapped/out of the learner model. Export via the #31 exporter + the F-187 harness (resources PR #34: --allow-new-official + EXPECTED_CENSUS extension in the same PR); then hub PR + live verification. Order: 1CR tranche first (110-mark format closest to the proven 1C pipeline), series ascending.</t>
+          <t>ADDED v2 (2026-10-21 docs reconciliation, operator trace 1a15e714070287a9): v2-era epic registered from the merged PR record. (PRs #239 #249); the master-pack ADR-037 GO-gated items (tracker claim + 2C-4C scheduling) remain operator-adjudicated.| GO RULING v2 (2026-10-21, operator trace 1a15ebd93809a525): GO granted - the executed 1C wiring (PRs #239 #249) is ratified post-hoc (process exception, not precedent); tracker-claim gate CLEARED; scheduling GRANTED for the remaining 4CH1 variants 2C x16 + 1CR x11 + 2CR x11 = 38 papers (registry-corrected from the ADR prose label "2C-4C"; same pipeline unchanged, UNVERIFIED list = scheduled gates); new courses DEFERRED (ADR-019 Cycle-1 scope / spec 39a).| 2C TRANCHE DONE (2026-10-21, trace 1a15ee5761b7a4a5): 16/16 4CH1/2C slices converted end-to-end, all gates PASS, 1120/1120 marks, 27/27 MCQs keyed (converter v0.8.0 = F34 paper parametrization + F35 MS question-marker discipline + F36 sentence-form positives; syllabai-resources PR #25, merge 1a5a8e6). Remaining GO-approved schedule: 1CR x11 + 2CR x11. 2C follow-ups (spec-label waves, crop-review eyeballs, parsed-layer cross-diff) recorded in Official-ExamQuestion/AGENTS.md known-open-work. | UPDATE 2026-10-22 (trace 1a16017ebd6ad2b5): 2C spec-label leg LANDED — resources v0.9.0 (commit 89260832) re-exported all 32 official sets; syllabai-v2 PR #268 merged 2026-10-21T19:02Z. 2C 607/607 parts resolved: 584 spec-tagged (registry-validated, 0 invalid codes) + 23 terminal no-spec-point honestly unmapped. Independent post-merge review: change census 584 labels + 8 solutionMd + 8 markPoints + 7 answerStatus (1C unmatched→linked) + F40 crop re-binds + 16 stub-banner rewordings; 0 structure/marks/exam-wording changes; SME 28/28 byte-preserved; official-set topicId re-key contained (0 external refs in bundle). | R-VARIANT SCHEDULE (2026-10-22, trace 1a1604c4c6b5c9a5): GO'd 1CR x11 + 2CR x11 footer-verified from the archive of record — 22/22 OK (contiguous numbering 22/22; manifest paper_number_variant matches --paper 22/22; legacy 4CH0 R papers 2013-2017 in the archive are a DIFFERENT spec, out of scope). 1CR @ 110 marks, printed question counts: 2019-06:10, 2020-01:11, 2020-11:10, 2021-01:10, 2022-01:11, 2022-06:11, 2023-01:10, 2023-06:11, 2024-06:12, 2025-06:11, 2026-06:11. 2CR @ 70 marks: 2019-06:7, 2020-01:7, 2020-11:7, 2021-01:8, 2022-01:7, 2022-06:7, 2023-01:8, 2023-06:7, 2024-06:7, 2025-06:7, 2026-06:7. Run protocol (same kit, --paper 1CR/2CR): registry entries land in the run PR (PAPER_TOTALS 1CR=110/2CR=70 + EXPECT_QUESTIONS with these counts) per the outputs-and-pipeline commit law; per-paper G0-G7 + negative controls 3/3 per series; layout findings through the improvement loop (F-ledger + canaries); MCQ ambiguities -&gt; MCQ-KEYS.json human adjudication with rendered-page evidence; crop flags -&gt; CROP-REVIEW.json eyeball verdicts; per-paper spec-label waves after conversion (labels only, G6 judges) — anchor law: untagged parts stay unmapped/out of the learner model. Export via the #31 exporter + the F-187 harness (resources PR #34: --allow-new-official + EXPECTED_CENSUS extension in the same PR); then hub PR + live verification. Order: 1CR tranche first (110-mark format closest to the proven 1C pipeline), series ascending. | CROP-REVIEW CLOSURE RE-VERIFIED (2026-10-22, trace 1a1608c3ae515a7d): post wave-13-crop-pass + wave-14, the 16 2C topic.json files carry 86 figure assets (85 crop + 1 crop-required) with 0 review-flagged parts — nothing awaits an eyeball verdict; CROP-REVIEW.json of record re-eyeballed 2026-10-22 (37 accepted + 4 stub-accepted across 24 homes incl. 10 2C homes; stem-table crops via canaries C33-C35). The wave-13 crop pass applied the last 4 part fixes through the exporter's disclosed census (matched exactly). The 22x 2C crop-review queue item is closed at ground truth.</t>
         </is>
       </c>
     </row>
@@ -22431,7 +22431,7 @@
       <c r="X193" s="6" t="inlineStr"/>
       <c r="Y193" s="6" t="inlineStr">
         <is>
-          <t>Added 2026-10-22 (trace 1a16017ebd6ad2b5) from the operator-ordered "proceed" on resources PR #27 — the supersession (provenance exporter via #31, #27 closed 2026-10-21T19:20Z) is already executed; the actionable residue is this hardening wave. Provenance law: the #31 exporter is the of record; G-E1..G-E4 are additive verification only. | UPDATE 2026-10-22 (trace 1a1604c4c6b5c9a5): build OPEN as resources PR #34 (branch f187/export-gates-r0) — G-E1..G-E4 artifact-level harness over the #31 exporter (additive only) + seed-fault self-test 4/4 refused on the of-record corpus + CI job official-export-gates green. G-E1's first run caught a real drift: the exporter regenerated topicSlug=official-past-papers (pre-F39) where the served bundle carries the per-set topic law; PR #34 fixes the exporter one-liner, after which it reproduces the bundle of record exactly (0 part deltas, SME prefix byte-identical 2,605,414 B).</t>
+          <t>Added 2026-10-22 (trace 1a16017ebd6ad2b5) from the operator-ordered "proceed" on resources PR #27 — the supersession (provenance exporter via #31, #27 closed 2026-10-21T19:20Z) is already executed; the actionable residue is this hardening wave. Provenance law: the #31 exporter is the of record; G-E1..G-E4 are additive verification only. | UPDATE 2026-10-22 (trace 1a1604c4c6b5c9a5): build OPEN as resources PR #34 (branch f187/export-gates-r0) — G-E1..G-E4 artifact-level harness over the #31 exporter (additive only) + seed-fault self-test 4/4 refused on the of-record corpus + CI job official-export-gates green. G-E1's first run caught a real drift: the exporter regenerated topicSlug=official-past-papers (pre-F39) where the served bundle carries the per-set topic law; PR #34 fixes the exporter one-liner, after which it reproduces the bundle of record exactly (0 part deltas, SME prefix byte-identical 2,605,414 B). | UPDATE 2026-10-22 (trace 1a1608c3ae515a7d): build MERGED as resources PR #34 (merge b5701769b9ca) — reconciled onto wave-14 main as commit 0ad59ca5935 (2 files: the G-E1..G-E4 harness + the official-export-gates CI job; the exporter of record NOT modified — the branch's original topicSlug one-liner was superseded by F44 bf8d56c30f + #41 and dropped in the reconciliation). CI-enforced on every scripts/PR: G-E1 lattice + disclosed-class parity with the harness's own census == the exporter-disclosures of record (new --disclosure gate, artifact-level mirror of the exporter's --expected-deltas law); G-E2 strict mark law on all 32 sets — the 2019-06 1C damage (104/110, gaps 3+6+2+3=14) was REPAIRED by v0.10.0's F41 OCR re-capture (EXPECTED_MARK_GAPS now empty, repair of record documented in-file); G-E3 census rebased to converter v0.10.0 (2019-06 1C (15,64,110,110); other 31 tuples unchanged) + --report cross-check; G-E4 SME prefix byte-identity (2,605,414 B). Self-test 4/4 seeds refused — acceptance met. One CI iteration: the fresh-checkout ls -t tie-break picked wave13-crop-pass (4 parts) over wave14 (298); replaced with deterministic sort -V on the wave-numbered filename. Run-protocol wiring for 1CR/2CR unchanged: EXPECTED_CENSUS extension + --allow-new-official land in the run PR per the outputs-and-pipeline law.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: F-185 build-open flip — In Progress + the BUILD OPEN receipt (model-driven draw + method-credit agreement landed, syllabai-v2 PR #332, trace 1a168845df85bf7d)
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -22169,7 +22169,7 @@
       </c>
       <c r="U191" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V191" s="6" t="inlineStr">
@@ -22185,7 +22185,7 @@
       <c r="X191" s="6" t="inlineStr"/>
       <c r="Y191" s="6" t="inlineStr">
         <is>
-          <t>Added 2026-10-22 from the Kognity Strength Test deep dive (dossier v1.1, trace 1a15fe54423bf93d). The category-making substitution per Deep Dive D; research-gated.</t>
+          <t>Added 2026-10-22 from the Kognity Strength Test deep dive (dossier v1.1, trace 1a15fe54423bf93d). The category-making substitution per Deep Dive D; research-gated. | BUILD OPEN — MODEL-DRIVEN DRAW + METHOD-CREDIT AGREEMENT LANDED (2026-10-23, trace 1a168845df85bf7d): the model-driven drill draw is LIVE and the agreement measurement of record is filed. syllabai-v2 PR #332 (merge 07c7315145fb1ff8987fbf04ee1733a3d0f3cd7a) — the selection law M1..M8 (M1 read-only learner reading — ADR-031 computed-never-persisted verbatim: every learner number computed at the injected now from the drill's own immutable evidence rows, no learner-state table exists, none added; M2 the F-184 strength law composed not re-adjudicated — S1 marks-weighted anchor + S2 decayed strength per code, unexplored = honest null; M3 the secondary-code information PROXY of record: I(part) = sum of u(c) over codes(part) \ {address}, u = 1 - strength, UNEXPLORED_WEIGHT 0.5 — a disclosed proxy, not BKT information gain; M4 sparse-state fallback below 5 course-graded rows to the F-182 random law P1..P6 verbatim, disclosed policy 'random' + sparseFallback true; M5 exploration floor 1 of 5 slots uniform-random seeded; M6 anti-gaming — determinism P5 extended by the reading, fresh per-draw seed, the wire carries the POLICY never a learner-state number; M7 synchronous pure selection — no LLM in the draw path, the only new read is the exact SELECT the F-184 strengths projection already performs; M8 zero stakes P6 verbatim) + the method-credit agreement law A1..A5 (two-rater Cohen's kappa over the F-183 acks — the F-183 plan s7 handoff 'agreement measurement is F-185's title, consuming these acks' consumed; point-paired denominator with disclosed exclusions; Pe from the joint marginals; the degenerate honest null; T-SM-KAPPA-SUBJECT precedent at drill scale). Wire: ONE additive required field — drillDrawResponseSchema.selection {policy model|random, sparseFallback, explorationSlots}; no answer facts (the F-183 L5 boundary pin green through the extended schema); no hub file (Frontend Impl = No); NO DB migration (Q8: the A/B policy-label column waits for a quiet db journal — the Seneca lane owns it; disclosed residual). Prereg docs/F185-MODEL-DRIVEN-DRAW-PLAN.md committed WITH the implementation (Q1..Q10); receipt .syllabai/receipts/F185-MODEL-DRAW/f185-model-draw-build-run-001-r0.json. Battery: root typecheck 0 + hub tsc 0; full v2 suite 2788 pass / 13 skip / 0 fail (150 files; +36 pins over the F-184 build receipt's 2752: model-draw 22, agreement 10, contracts 1, routes 3); retrieval-eval 22 pass + 19/19 selftest vectors; golden selftest OK; zero-core census gate GREEN; census anti-drift pin green (no census surface touched). Dependency posture (the F-184 disclosed precedent): F-138/F-139/F-055 Not Started — substance composed not re-adjudicated; the BKT posterior read swaps in behind the same seam when F-138 lands, the policy untouched by construction. Residuals: no live agreement number (the two-rater collection runs — second generator pass or teacher reference — are operator-gated research runs; the F-183 precedent 'the metric infrastructure is what lands'); the draw picks WITHIN an address (address-level guidance remains the picker + the F-184 practice-now queue). Next per the filed dossier line: F-186 battle wave, strictly sequenced after F-185 per its filed row — battles inherit model-drawn sets through drawForLearner. Status -&gt; In Progress.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: F-186 build-open flip — In Progress + the BUILD OPEN receipt (the Strength Battle mode landed, syllabai-v2 PR #335, trace 1a168cedec59d1ad)
</commit_message>
<xml_diff>
--- a/backlog/syllabai-master-project.xlsx
+++ b/backlog/syllabai-master-project.xlsx
@@ -22292,7 +22292,7 @@
       </c>
       <c r="U192" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="V192" s="6" t="inlineStr">
@@ -22308,7 +22308,7 @@
       <c r="X192" s="6" t="inlineStr"/>
       <c r="Y192" s="6" t="inlineStr">
         <is>
-          <t>Added 2026-10-22 from the Kognity Strength Test deep dive (dossier v1.1, trace 1a15fe54423bf93d). Explicitly a later wave; the 5M-battle engagement figure is vendor-claimed (single-source).</t>
+          <t>Added 2026-10-22 from the Kognity Strength Test deep dive (dossier v1.1, trace 1a15fe54423bf93d). Explicitly a later wave; the 5M-battle engagement figure is vendor-claimed (single-source). | BUILD OPEN — STRENGTH BATTLE MODE LANDED (2026-10-23, trace 1a168cedec59d1ad): the same drill bank wears competitive energy — the 3-question / 60-second head-to-head vs the bot opponent of record is LIVE. syllabai-v2 PR #335 (merge 6e9bb8554c3347a61f9a4b9c29e7517908ca5c41) — the battle law B1..B8 (B1 SAME BANK SECOND MODE: the EXACT F-185 drawForLearner composition — the model law M1..M8 + the sparse fallback to P1..P6 — over the BATTLE-ELIGIBLE pool with floor 3; battles inherit model-drawn sets verbatim per the filed Solution line; B2 the format of record: BATTLE_SIZE 3 / BATTLE_CLOCK_MS 60_000 / P3 fail-closed — never a short battle; B3 FAIRNESS: one draw both sides + THE one server-side grader (bank.isCorrectChoice) + choice-gradable parts only — a head-to-head cannot server-grade a structured part without inventing marks and the seam refuses; B4 the opponent of record: seeded-coin-v1, a fair coin HONESTLY disclosed as a coin not a model — per part one credit draw + one latency draw (band [5s,15s], inside the clock by construction) from mulberry32(draw.seed), pure and audit-reconstructible; B5 THE CLOCK LAW: the draw row's created_at is the start of record, an evidence row counts iff its immutable write time &lt;= start+60s, over-clock rows stay real drill evidence but score zero and are disclosed inClock:false — the server clock is the law, the client countdown the affordance; B6 MARKS ARE THE CURRENCY: credited iff server-graded correct within the clock, both-correct = wonBy 'split' with BOTH sides scoring — deliberately NO race, DB write jitter is not a speed skill; B7 the settlement computed AT READ, never persisted (ADR-031 posture) — no battle table exists none added, no answer key in the shape, the battle wire schemas STRICT end to end; B8 zero stakes + opt-in: only a learner POST starts a battle, only the drill's own drill_draws + drill_part_evidence rows are written, no gradebook surface, no leaderboard). Wire: POST /drill/battles + GET /battles/:drawId/settlement (additive drill-family routes; battle ANSWERS ride the UNCHANGED /evidence seam — the F-183 instant MS-reveal law covers battle parts verbatim, dossier law 2: 'Strength Tests and Strength Battles always show your score and solutions once you answer'); hub (Frontend Impl = Yes): /practice/battle the opt-in player (the ?code= deep link preselects, never auto-starts) + 2 additive strengths-panel links. REAL-bundle numbers of record: 443 battle-eligible parts, 68 battle-ready addresses of 157 drillable; the drill flagship 4CH1-1.25 carries exactly 2 eligible and the battle REFUSES there (the fail-closed floor demonstrated on the real bank); the strongest battle-ready address 4CH1-1.16 settles a real card in the battery. Prereg docs/F186-BATTLE-MODE-PLAN.md committed WITH the implementation (Q1..Q10); receipt .syllabai/receipts/F186-BATTLE/f186-battle-build-run-001-r0.json. Battery: root typecheck 0 + hub tsc 0; full v2 suite 2822 pass / 13 skip / 0 fail (151 files; +34 pins over the afbfcfb450 baseline 2788/13/0: battle law 20, battle routes 10 + 2 authz paths, battle contracts 2); retrieval-eval 22 pass + 19/19 selftest vectors; golden selftest OK; zero-core census gate GREEN; census anti-drift pin green. Residuals (disclosed in the prereg s9): live matchmaking / async ghost opponents (the 'vs classmate' arm — needs realtime infra); class brackets + any leaderboard (ADR-036 k-anonymity territory, operator-gated — nothing leaderboard-shaped ships, not even a per-address high score); the model-driven bot (the seeded coin is the honest v1; swaps in behind botCard); the battle-kind column (the 3-part discriminator is pinned; a column needs the db journal). THE FILED DOSSIER LINE IS NOW FULLY OPEN: F-182/F-183/F-184/F-185/F-186 all In Progress. Status -&gt; In Progress.</t>
         </is>
       </c>
     </row>

</xml_diff>